<commit_message>
Add GANK combat event rule
</commit_message>
<xml_diff>
--- a/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
+++ b/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="R965e8122d04041e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R5d639a315f974e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="Rc2870fb8c7bc4993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="R3769a2ae2e9046da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="R4a6b1f9eecaf42a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="R0a7da6e0a6ab4203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="R1f500c505d9246e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="R4975916be45e4b95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="R1a5176bb81ea4ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R93b76d182b554a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="R6112f865ee8d45a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="R0c42d555412c4133"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="R5002ef89733c4eae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="Rdfd145d613414f72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="R89e6bfc0659e407b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="R8e1b3b069d774904"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,10 +320,10 @@
         <x:v>输出标签数</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>对线分路、勾兵、断线、拉野、囤野/堆野、控符、蹲人、开雾、小规模冲突、团战、肉山团、肉山击杀、高地团、守塔团、肉山尝试、魔晶团、资源获得、带盾阵亡</x:v>
+        <x:v>对线分路、勾兵、断线、拉野、囤野/堆野、控符、蹲人、开雾、GANK、小规模冲突、团战、肉山团、肉山击杀、高地团、守塔团、肉山尝试、魔晶团、资源获得、带盾阵亡</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str"/>
     </x:row>
@@ -335,7 +335,7 @@
         <x:v>抓人</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>不作为最终输出标签；历史候选会重映射/合并为小规模冲突或团战</x:v>
+        <x:v>不作为最终输出标签；历史候选会重映射/合并为GANK、小规模冲突或团战</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str"/>
     </x:row>
@@ -794,7 +794,7 @@
     </x:row>
     <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>小规模冲突</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -803,40 +803,40 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+        <x:v>combat_logs; player_intervals2</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>双方局部伤害/控制/死亡聚类；通常双方各2人以上且总人数&lt;=7，或总人数&gt;=4且有死亡但未达团战规模</x:v>
+        <x:v>战斗聚类中一方N抓1：一方直接参与英雄&gt;=2，另一方参与英雄&lt;=1</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>聚类开始-结束；候选先手可提前到控制/大伤害/先手技能时刻</x:v>
+        <x:v>聚类开始-结束</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
-        <x:v>10秒桶；raw聚类38；跨桶间隔12秒；聚类距离48 raw；细化事件前后6秒、中心62 raw；英雄参与默认1600码</x:v>
+        <x:v>继承战斗聚类时间/空间阈值；直接参与=造成伤害或施加控制</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str">
-        <x:v>只保留战斗核心附近或对参与英雄造成伤害/控制的英雄；排除远处未命中核心的独立消耗</x:v>
+        <x:v>gank方英雄 + 被抓英雄</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
         <x:v>结果=击杀比分；死亡列表；无死亡写未记录英雄击杀/死亡无</x:v>
       </x:c>
       <x:c r="J10" s="5" t="str">
-        <x:v>v1.7+吸收旧单点候选；v1.8/v1.9继续合并重复短窗口</x:v>
+        <x:v>优先于小规模冲突判定；后续可被守塔团/高地团/肉山团等特殊上下文修饰</x:v>
       </x:c>
       <x:c r="K10" s="5" t="str">
-        <x:v>低于团战，高于纯资源/控符事实</x:v>
+        <x:v>低于团战特殊上下文，高于小规模冲突</x:v>
       </x:c>
       <x:c r="L10" s="5" t="str">
-        <x:v>边界和语义建议录像复核</x:v>
+        <x:v>需要人工校准N抓1但未实质开战、远程消耗等边界</x:v>
       </x:c>
       <x:c r="M10" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N10" s="5" t="str"/>
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -848,28 +848,28 @@
         <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>双方多人持续交战；双方总参与通常各4人以上，且直接参与各&gt;=3人，并满足总伤害&gt;=2500、死亡&gt;=2或持续&gt;=15秒之一</x:v>
+        <x:v>双方局部伤害/控制/死亡聚类；通常双方各2人以上且总人数&lt;=7，或总人数&gt;=4且有死亡但未达团战规模</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>聚类开始-结束；先手技能可提前开始</x:v>
+        <x:v>聚类开始-结束；候选先手可提前到控制/大伤害/先手技能时刻</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
-        <x:v>团战人数阈值4v4；直接参与3v3；伤害2500；死亡2；持续15秒</x:v>
+        <x:v>10秒桶；raw聚类38；跨桶间隔12秒；聚类距离48 raw；细化事件前后6秒、中心62 raw；英雄参与默认1600码</x:v>
       </x:c>
       <x:c r="H11" s="5" t="str">
-        <x:v>同小规模冲突，按空间/交互排除远端独立交互</x:v>
+        <x:v>只保留战斗核心附近或对参与英雄造成伤害/控制的英雄；排除远处未命中核心的独立消耗</x:v>
       </x:c>
       <x:c r="I11" s="5" t="str">
-        <x:v>结果=击杀比分；死亡列表；带盾阵亡需标注</x:v>
+        <x:v>结果=击杀比分；死亡列表；无死亡写未记录英雄击杀/死亡无</x:v>
       </x:c>
       <x:c r="J11" s="5" t="str">
-        <x:v>与特殊战斗标签可并存：肉山团/高地团/守塔团/魔晶团</x:v>
+        <x:v>v1.7+吸收旧单点候选；v1.8/v1.9继续合并重复短窗口</x:v>
       </x:c>
       <x:c r="K11" s="5" t="str">
-        <x:v>优先级高于小规模冲突；被特殊战斗标签修饰</x:v>
+        <x:v>低于团战，高于纯资源/控符事实</x:v>
       </x:c>
       <x:c r="L11" s="5" t="str">
-        <x:v>远距离同时开战要拆分，不可只按时间合并</x:v>
+        <x:v>边界和语义建议录像复核</x:v>
       </x:c>
       <x:c r="M11" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -878,7 +878,7 @@
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -890,28 +890,28 @@
         <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>肉山仍存活，且战斗围绕肉山坑/肉山伤害/肉山击杀上下文展开</x:v>
+        <x:v>双方多人持续交战；双方总参与通常各4人以上，且直接参与各&gt;=3人，并满足总伤害&gt;=2500、死亡&gt;=2或持续&gt;=15秒之一</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
-        <x:v>战斗窗口；肉山伤害前后30秒；肉山击杀前45秒到后75秒</x:v>
+        <x:v>聚类开始-结束；先手技能可提前开始</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
-        <x:v>肉山坑2000码；肉山死亡后480秒内视为未刷新</x:v>
+        <x:v>团战人数阈值4v4；直接参与3v3；伤害2500；死亡2；持续15秒</x:v>
       </x:c>
       <x:c r="H12" s="5" t="str">
-        <x:v>参与战斗双方英雄</x:v>
+        <x:v>同小规模冲突，按空间/交互排除远端独立交互</x:v>
       </x:c>
       <x:c r="I12" s="5" t="str">
-        <x:v>结果追加目标：肉山相关；肉山击杀结果由肉山击杀标签独立记录</x:v>
+        <x:v>结果=击杀比分；死亡列表；带盾阵亡需标注</x:v>
       </x:c>
       <x:c r="J12" s="5" t="str">
-        <x:v>肉山死亡后的追击不再因靠近肉山坑误标肉山团</x:v>
+        <x:v>与特殊战斗标签可并存：肉山团/高地团/守塔团/魔晶团</x:v>
       </x:c>
       <x:c r="K12" s="5" t="str">
-        <x:v>可与团战/小规模冲突并存</x:v>
+        <x:v>优先级高于小规模冲突；被特殊战斗标签修饰</x:v>
       </x:c>
       <x:c r="L12" s="5" t="str">
-        <x:v>需区分肉山尝试、肉山击杀、肉山后追击</x:v>
+        <x:v>远距离同时开战要拆分，不可只按时间合并</x:v>
       </x:c>
       <x:c r="M12" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -920,91 +920,91 @@
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>auto</x:v>
+        <x:v>candidate_review</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>combat_logs; match_chat_events</x:v>
+        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>Roshan死亡事件；统一记录为肉山击杀，不再作为普通资源获得输出；合并同一波肉山掉落</x:v>
+        <x:v>肉山仍存活，且战斗围绕肉山坑/肉山伤害/肉山击杀上下文展开</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
-        <x:v>击杀时刻到最后一个20秒内相关掉落</x:v>
+        <x:v>战斗窗口；肉山伤害前后30秒；肉山击杀前45秒到后75秒</x:v>
       </x:c>
       <x:c r="G13" s="5" t="str">
-        <x:v>掉落合并窗口20秒；击杀归属优先combat_logs roshan_death；缺失时用5秒内掉落阵营兜底</x:v>
+        <x:v>肉山坑2000码；肉山死亡后480秒内视为未刷新</x:v>
       </x:c>
       <x:c r="H13" s="5" t="str">
-        <x:v>获得掉落的英雄/阵营；heroes合并击杀和掉落相关英雄</x:v>
+        <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I13" s="5" t="str">
-        <x:v>结果=哪方击杀肉山；哪个英雄获得盾/奶酪/刷新碎片/战旗等</x:v>
+        <x:v>结果追加目标：肉山相关；肉山击杀结果由肉山击杀标签独立记录</x:v>
       </x:c>
       <x:c r="J13" s="5" t="str">
-        <x:v>CHAT_MESSAGE_ROSHAN_KILL的player/value不作为击杀英雄依据</x:v>
+        <x:v>肉山死亡后的追击不再因靠近肉山坑误标肉山团</x:v>
       </x:c>
       <x:c r="K13" s="5" t="str">
-        <x:v>优先级高于资源获得；同一肉山只一行</x:v>
+        <x:v>可与团战/小规模冲突并存</x:v>
       </x:c>
       <x:c r="L13" s="5" t="str">
-        <x:v>需人工检查掉落事件是否完整合并</x:v>
+        <x:v>需区分肉山尝试、肉山击杀、肉山后追击</x:v>
       </x:c>
       <x:c r="M13" s="5" t="str">
-        <x:v>v1.8-v1.9</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N13" s="5" t="str"/>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>高地团</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>candidate_review</x:v>
+        <x:v>auto</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
-        <x:v>combat_logs; tower/barracks events; player_intervals2</x:v>
+        <x:v>combat_logs; match_chat_events</x:v>
       </x:c>
       <x:c r="E14" s="5" t="str">
-        <x:v>一方或双方在高地、基地入口、破路区域发生团战/小规模冲突</x:v>
+        <x:v>Roshan死亡事件；统一记录为肉山击杀，不再作为普通资源获得输出；合并同一波肉山掉落</x:v>
       </x:c>
       <x:c r="F14" s="5" t="str">
-        <x:v>战斗窗口；兵营击杀前20秒到后60秒</x:v>
+        <x:v>击杀时刻到最后一个20秒内相关掉落</x:v>
       </x:c>
       <x:c r="G14" s="5" t="str">
-        <x:v>中心raw坐标x&lt;95且y&lt;95或x&gt;158且y&gt;158；或兵营事件附近</x:v>
+        <x:v>掉落合并窗口20秒；击杀归属优先combat_logs roshan_death；缺失时用5秒内掉落阵营兜底</x:v>
       </x:c>
       <x:c r="H14" s="5" t="str">
-        <x:v>参与战斗双方英雄</x:v>
+        <x:v>获得掉落的英雄/阵营；heroes合并击杀和掉落相关英雄</x:v>
       </x:c>
       <x:c r="I14" s="5" t="str">
-        <x:v>结果继承战斗结果</x:v>
+        <x:v>结果=哪方击杀肉山；哪个英雄获得盾/奶酪/刷新碎片/战旗等</x:v>
       </x:c>
       <x:c r="J14" s="5" t="str">
-        <x:v>作为附加标签插入战斗标签前</x:v>
+        <x:v>CHAT_MESSAGE_ROSHAN_KILL的player/value不作为击杀英雄依据</x:v>
       </x:c>
       <x:c r="K14" s="5" t="str">
-        <x:v>特殊战斗标签优先级高</x:v>
+        <x:v>优先级高于资源获得；同一肉山只一行</x:v>
       </x:c>
       <x:c r="L14" s="5" t="str">
-        <x:v>高地前poke与正式开团需复核</x:v>
+        <x:v>需人工检查掉落事件是否完整合并</x:v>
       </x:c>
       <x:c r="M14" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.8-v1.9</x:v>
       </x:c>
       <x:c r="N14" s="5" t="str"/>
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>守塔团</x:v>
+        <x:v>高地团</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1013,31 +1013,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D15" s="5" t="str">
-        <x:v>tower_status_update; combat_logs</x:v>
+        <x:v>combat_logs; tower/barracks events; player_intervals2</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
-        <x:v>一方在防御塔附近约1000码内防守时发生的战斗</x:v>
+        <x:v>一方或双方在高地、基地入口、破路区域发生团战/小规模冲突</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
-        <x:v>战斗开始前5秒到结束后5秒内塔上下文</x:v>
+        <x:v>战斗窗口；兵营击杀前20秒到后60秒</x:v>
       </x:c>
       <x:c r="G15" s="5" t="str">
-        <x:v>防御塔1000码；塔hp&gt;0</x:v>
+        <x:v>中心raw坐标x&lt;95且y&lt;95或x&gt;158且y&gt;158；或兵营事件附近</x:v>
       </x:c>
       <x:c r="H15" s="5" t="str">
         <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I15" s="5" t="str">
-        <x:v>结果继承战斗结果并附塔上下文</x:v>
+        <x:v>结果继承战斗结果</x:v>
       </x:c>
       <x:c r="J15" s="5" t="str">
-        <x:v>作为附加标签追加，可与小规模冲突/团战并存</x:v>
+        <x:v>作为附加标签插入战斗标签前</x:v>
       </x:c>
       <x:c r="K15" s="5" t="str">
-        <x:v>特殊上下文标签</x:v>
+        <x:v>特殊战斗标签优先级高</x:v>
       </x:c>
       <x:c r="L15" s="5" t="str">
-        <x:v>塔已掉或追击阶段不应误标</x:v>
+        <x:v>高地前poke与正式开团需复核</x:v>
       </x:c>
       <x:c r="M15" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -1046,7 +1046,7 @@
     </x:row>
     <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>守塔团</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1055,31 +1055,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>combat_logs</x:v>
+        <x:v>tower_status_update; combat_logs</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>对Roshan造成伤害但未完成击杀，也未转化为肉山团</x:v>
+        <x:v>一方在防御塔附近约1000码内防守时发生的战斗</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
-        <x:v>连续Roshan伤害组；组内间隔&lt;=45秒；结束后+10秒</x:v>
+        <x:v>战斗开始前5秒到结束后5秒内塔上下文</x:v>
       </x:c>
       <x:c r="G16" s="5" t="str">
-        <x:v>总伤害&gt;=1500；攻击英雄&gt;=1；组内无击杀且结束后8秒无击杀</x:v>
+        <x:v>防御塔1000码；塔hp&gt;0</x:v>
       </x:c>
       <x:c r="H16" s="5" t="str">
-        <x:v>对肉山造成伤害的英雄</x:v>
+        <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I16" s="5" t="str">
-        <x:v>结果=Roshan总伤害和未击杀说明</x:v>
+        <x:v>结果继承战斗结果并附塔上下文</x:v>
       </x:c>
       <x:c r="J16" s="5" t="str">
-        <x:v>若双方围绕肉山开战，优先肉山团</x:v>
+        <x:v>作为附加标签追加，可与小规模冲突/团战并存</x:v>
       </x:c>
       <x:c r="K16" s="5" t="str">
-        <x:v>低于肉山团/肉山击杀</x:v>
+        <x:v>特殊上下文标签</x:v>
       </x:c>
       <x:c r="L16" s="5" t="str">
-        <x:v>偷Roshan试探与真尝试需复核</x:v>
+        <x:v>塔已掉或追击阶段不应误标</x:v>
       </x:c>
       <x:c r="M16" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -1088,7 +1088,7 @@
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1097,31 +1097,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D17" s="5" t="str">
-        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+        <x:v>combat_logs</x:v>
       </x:c>
       <x:c r="E17" s="5" t="str">
-        <x:v>折磨者/魔晶仍存活时，围绕魔晶区域发生团战或资源争夺</x:v>
+        <x:v>对Roshan造成伤害但未完成击杀，也未转化为肉山团</x:v>
       </x:c>
       <x:c r="F17" s="5" t="str">
-        <x:v>战斗窗口；魔晶伤害前后30秒；击杀前45秒到后60秒</x:v>
+        <x:v>连续Roshan伤害组；组内间隔&lt;=45秒；结束后+10秒</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
-        <x:v>魔晶区域1500-2000码；20分钟后可存活；击杀后600秒内视为未刷新</x:v>
+        <x:v>总伤害&gt;=1500；攻击英雄&gt;=1；组内无击杀且结束后8秒无击杀</x:v>
       </x:c>
       <x:c r="H17" s="5" t="str">
-        <x:v>参与战斗双方英雄</x:v>
+        <x:v>对肉山造成伤害的英雄</x:v>
       </x:c>
       <x:c r="I17" s="5" t="str">
-        <x:v>结果继承战斗结果或写魔晶归属</x:v>
+        <x:v>结果=Roshan总伤害和未击杀说明</x:v>
       </x:c>
       <x:c r="J17" s="5" t="str">
-        <x:v>魔晶击杀后追击不再误标魔晶团</x:v>
+        <x:v>若双方围绕肉山开战，优先肉山团</x:v>
       </x:c>
       <x:c r="K17" s="5" t="str">
-        <x:v>特殊战斗标签优先级高</x:v>
+        <x:v>低于肉山团/肉山击杀</x:v>
       </x:c>
       <x:c r="L17" s="5" t="str">
-        <x:v>需区分单方打魔晶与双方争夺</x:v>
+        <x:v>偷Roshan试探与真尝试需复核</x:v>
       </x:c>
       <x:c r="M17" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -1130,87 +1130,129 @@
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>资源获得</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>auto</x:v>
+        <x:v>candidate_review</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>match_chat_events; combat_logs</x:v>
+        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
-        <x:v>独立记录关键资源事实：魔晶/折磨者、战旗等；v1.8后肉山击杀与肉山掉落并入肉山击杀，不再单独输出普通资源获得</x:v>
+        <x:v>折磨者/魔晶仍存活时，围绕魔晶区域发生团战或资源争夺</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>资源事件时刻</x:v>
+        <x:v>战斗窗口；魔晶伤害前后30秒；击杀前45秒到后60秒</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
-        <x:v>Roshan kill归属兜底5秒；普通资源按chat事件</x:v>
+        <x:v>魔晶区域1500-2000码；20分钟后可存活；击杀后600秒内视为未刷新</x:v>
       </x:c>
       <x:c r="H18" s="5" t="str">
-        <x:v>获得资源的英雄或阵营</x:v>
+        <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I18" s="5" t="str">
-        <x:v>结果=英雄/阵营+资源动作</x:v>
+        <x:v>结果继承战斗结果或写魔晶归属</x:v>
       </x:c>
       <x:c r="J18" s="5" t="str">
-        <x:v>旧抢盾/抢奶/抢刷新并入资源获得或肉山击杀口径</x:v>
+        <x:v>魔晶击杀后追击不再误标魔晶团</x:v>
       </x:c>
       <x:c r="K18" s="5" t="str">
-        <x:v>低于肉山击杀</x:v>
+        <x:v>特殊战斗标签优先级高</x:v>
       </x:c>
       <x:c r="L18" s="5" t="str">
-        <x:v>需要确认非肉山资源未被误合并</x:v>
+        <x:v>需区分单方打魔晶与双方争夺</x:v>
       </x:c>
       <x:c r="M18" s="5" t="str">
-        <x:v>v1.5-v1.9</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N18" s="5" t="str"/>
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>带盾阵亡</x:v>
+        <x:v>资源获得</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
         <x:v>auto</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
-        <x:v>A/B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D19" s="5" t="str">
         <x:v>match_chat_events; combat_logs</x:v>
       </x:c>
       <x:c r="E19" s="5" t="str">
-        <x:v>持有不朽盾的英雄死亡/消耗盾时独立记录；战斗死亡列表也标注[带盾阵亡]</x:v>
+        <x:v>独立记录关键资源事实：魔晶/折磨者、战旗等；v1.8后肉山击杀与肉山掉落并入肉山击杀，不再单独输出普通资源获得</x:v>
       </x:c>
       <x:c r="F19" s="5" t="str">
-        <x:v>死亡时刻</x:v>
+        <x:v>资源事件时刻</x:v>
       </x:c>
       <x:c r="G19" s="5" t="str">
-        <x:v>Aegis领取后300秒内的同英雄死亡；每个盾只消费一次</x:v>
+        <x:v>Roshan kill归属兜底5秒；普通资源按chat事件</x:v>
       </x:c>
       <x:c r="H19" s="5" t="str">
-        <x:v>带盾阵亡英雄及阵营</x:v>
+        <x:v>获得资源的英雄或阵营</x:v>
       </x:c>
       <x:c r="I19" s="5" t="str">
-        <x:v>结果=死亡时间、英雄、Aegis获取时间</x:v>
+        <x:v>结果=英雄/阵营+资源动作</x:v>
       </x:c>
       <x:c r="J19" s="5" t="str">
-        <x:v>可与团战/小规模冲突并存</x:v>
+        <x:v>旧抢盾/抢奶/抢刷新并入资源获得或肉山击杀口径</x:v>
       </x:c>
       <x:c r="K19" s="5" t="str">
-        <x:v>资源消耗事实类</x:v>
+        <x:v>低于肉山击杀</x:v>
       </x:c>
       <x:c r="L19" s="5" t="str">
-        <x:v>复活/盾消耗边界建议复核</x:v>
+        <x:v>需要确认非肉山资源未被误合并</x:v>
       </x:c>
       <x:c r="M19" s="5" t="str">
         <x:v>v1.5-v1.9</x:v>
       </x:c>
       <x:c r="N19" s="5" t="str"/>
+    </x:row>
+    <x:row r="20" ht="58.5" customHeight="1">
+      <x:c r="A20" s="5" t="str">
+        <x:v>带盾阵亡</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="str">
+        <x:v>auto</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="str">
+        <x:v>A/B</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="str">
+        <x:v>match_chat_events; combat_logs</x:v>
+      </x:c>
+      <x:c r="E20" s="5" t="str">
+        <x:v>持有不朽盾的英雄死亡/消耗盾时独立记录；战斗死亡列表也标注[带盾阵亡]</x:v>
+      </x:c>
+      <x:c r="F20" s="5" t="str">
+        <x:v>死亡时刻</x:v>
+      </x:c>
+      <x:c r="G20" s="5" t="str">
+        <x:v>Aegis领取后300秒内的同英雄死亡；每个盾只消费一次</x:v>
+      </x:c>
+      <x:c r="H20" s="5" t="str">
+        <x:v>带盾阵亡英雄及阵营</x:v>
+      </x:c>
+      <x:c r="I20" s="5" t="str">
+        <x:v>结果=死亡时间、英雄、Aegis获取时间</x:v>
+      </x:c>
+      <x:c r="J20" s="5" t="str">
+        <x:v>可与团战/小规模冲突并存</x:v>
+      </x:c>
+      <x:c r="K20" s="5" t="str">
+        <x:v>资源消耗事实类</x:v>
+      </x:c>
+      <x:c r="L20" s="5" t="str">
+        <x:v>复活/盾消耗边界建议复核</x:v>
+      </x:c>
+      <x:c r="M20" s="5" t="str">
+        <x:v>v1.5-v1.9</x:v>
+      </x:c>
+      <x:c r="N20" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2365,22 +2407,22 @@
     </x:row>
     <x:row r="48" ht="33" customHeight="1">
       <x:c r="A48" s="5" t="str">
-        <x:v>skirmish_max_total_heroes</x:v>
+        <x:v>gank_min_direct_attackers</x:v>
       </x:c>
       <x:c r="B48" s="5" t="str">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str">
         <x:v>人</x:v>
       </x:c>
       <x:c r="D48" s="5" t="str">
-        <x:v>小规模冲突</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E48" s="5" t="str">
-        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
+        <x:v>GANK方至少有2名直接参与英雄，直接参与指造成伤害或施加控制</x:v>
       </x:c>
       <x:c r="F48" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G48" s="5" t="str">
         <x:v>是</x:v>
@@ -2389,22 +2431,22 @@
     </x:row>
     <x:row r="49" ht="33" customHeight="1">
       <x:c r="A49" s="5" t="str">
-        <x:v>fight_dedup_gap_initial</x:v>
+        <x:v>gank_max_victim_side_heroes</x:v>
       </x:c>
       <x:c r="B49" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D49" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E49" s="5" t="str">
-        <x:v>初始fight record近邻合并时间</x:v>
+        <x:v>被抓一方参与英雄最多1人，即N抓1</x:v>
       </x:c>
       <x:c r="F49" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G49" s="5" t="str">
         <x:v>是</x:v>
@@ -2413,19 +2455,19 @@
     </x:row>
     <x:row r="50" ht="33" customHeight="1">
       <x:c r="A50" s="5" t="str">
-        <x:v>fight_dedup_distance_raw</x:v>
+        <x:v>skirmish_max_total_heroes</x:v>
       </x:c>
       <x:c r="B50" s="5" t="str">
-        <x:v>58</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D50" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E50" s="5" t="str">
-        <x:v>初始fight record近邻合并距离</x:v>
+        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
       </x:c>
       <x:c r="F50" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2437,19 +2479,19 @@
     </x:row>
     <x:row r="51" ht="33" customHeight="1">
       <x:c r="A51" s="5" t="str">
-        <x:v>fight_overlap_shared_heroes</x:v>
+        <x:v>fight_dedup_gap_initial</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D51" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E51" s="5" t="str">
-        <x:v>重叠fight record合并的共享英雄数</x:v>
+        <x:v>初始fight record近邻合并时间</x:v>
       </x:c>
       <x:c r="F51" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2461,22 +2503,22 @@
     </x:row>
     <x:row r="52" ht="33" customHeight="1">
       <x:c r="A52" s="5" t="str">
-        <x:v>pickoff_enemy_damage_ratio</x:v>
+        <x:v>fight_dedup_distance_raw</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>0.80</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D52" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E52" s="5" t="str">
-        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
+        <x:v>初始fight record近邻合并距离</x:v>
       </x:c>
       <x:c r="F52" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G52" s="5" t="str">
         <x:v>是</x:v>
@@ -2485,22 +2527,22 @@
     </x:row>
     <x:row r="53" ht="33" customHeight="1">
       <x:c r="A53" s="5" t="str">
-        <x:v>pickoff_ally_near_limit</x:v>
+        <x:v>fight_overlap_shared_heroes</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str">
         <x:v>人</x:v>
       </x:c>
       <x:c r="D53" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E53" s="5" t="str">
-        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
+        <x:v>重叠fight record合并的共享英雄数</x:v>
       </x:c>
       <x:c r="F53" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G53" s="5" t="str">
         <x:v>是</x:v>
@@ -2509,19 +2551,19 @@
     </x:row>
     <x:row r="54" ht="33" customHeight="1">
       <x:c r="A54" s="5" t="str">
-        <x:v>escape_pickoff_window</x:v>
+        <x:v>pickoff_enemy_damage_ratio</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>18</x:v>
+        <x:v>0.80</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D54" s="5" t="str">
         <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E54" s="5" t="str">
-        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
+        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
       </x:c>
       <x:c r="F54" s="5" t="str">
         <x:v>v1.6</x:v>
@@ -2533,19 +2575,19 @@
     </x:row>
     <x:row r="55" ht="33" customHeight="1">
       <x:c r="A55" s="5" t="str">
-        <x:v>escape_pickoff_damage_min</x:v>
+        <x:v>pickoff_ally_near_limit</x:v>
       </x:c>
       <x:c r="B55" s="5" t="str">
-        <x:v>180</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D55" s="5" t="str">
         <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E55" s="5" t="str">
-        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
+        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
       </x:c>
       <x:c r="F55" s="5" t="str">
         <x:v>v1.6</x:v>
@@ -2557,22 +2599,22 @@
     </x:row>
     <x:row r="56" ht="33" customHeight="1">
       <x:c r="A56" s="5" t="str">
-        <x:v>roshan_context_radius</x:v>
+        <x:v>escape_pickoff_window</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>2000</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D56" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E56" s="5" t="str">
-        <x:v>肉山团上下文范围</x:v>
+        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
       </x:c>
       <x:c r="F56" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G56" s="5" t="str">
         <x:v>是</x:v>
@@ -2581,22 +2623,22 @@
     </x:row>
     <x:row r="57" ht="33" customHeight="1">
       <x:c r="A57" s="5" t="str">
-        <x:v>roshan_context_min_time</x:v>
+        <x:v>escape_pickoff_damage_min</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D57" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E57" s="5" t="str">
-        <x:v>10分钟后靠近肉山坑可触发肉山上下文</x:v>
+        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
         <x:v>是</x:v>
@@ -2605,19 +2647,19 @@
     </x:row>
     <x:row r="58" ht="33" customHeight="1">
       <x:c r="A58" s="5" t="str">
-        <x:v>roshan_damage_context_pad</x:v>
+        <x:v>roshan_context_radius</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>30</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D58" s="5" t="str">
         <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E58" s="5" t="str">
-        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
+        <x:v>肉山团上下文范围</x:v>
       </x:c>
       <x:c r="F58" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2629,10 +2671,10 @@
     </x:row>
     <x:row r="59" ht="33" customHeight="1">
       <x:c r="A59" s="5" t="str">
-        <x:v>roshan_kill_context_before</x:v>
+        <x:v>roshan_context_min_time</x:v>
       </x:c>
       <x:c r="B59" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str">
         <x:v>秒</x:v>
@@ -2641,7 +2683,7 @@
         <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E59" s="5" t="str">
-        <x:v>肉山击杀与战斗关联前置时间</x:v>
+        <x:v>10分钟后靠近肉山坑可触发肉山上下文</x:v>
       </x:c>
       <x:c r="F59" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2653,10 +2695,10 @@
     </x:row>
     <x:row r="60" ht="33" customHeight="1">
       <x:c r="A60" s="5" t="str">
-        <x:v>roshan_kill_context_after</x:v>
+        <x:v>roshan_damage_context_pad</x:v>
       </x:c>
       <x:c r="B60" s="5" t="str">
-        <x:v>75</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C60" s="5" t="str">
         <x:v>秒</x:v>
@@ -2665,7 +2707,7 @@
         <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E60" s="5" t="str">
-        <x:v>肉山击杀与战斗关联后置时间</x:v>
+        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
       </x:c>
       <x:c r="F60" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2677,10 +2719,10 @@
     </x:row>
     <x:row r="61" ht="33" customHeight="1">
       <x:c r="A61" s="5" t="str">
-        <x:v>roshan_respawn_suppression</x:v>
+        <x:v>roshan_kill_context_before</x:v>
       </x:c>
       <x:c r="B61" s="5" t="str">
-        <x:v>480</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str">
         <x:v>秒</x:v>
@@ -2689,7 +2731,7 @@
         <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E61" s="5" t="str">
-        <x:v>肉山死亡后该时间内不视为存活</x:v>
+        <x:v>肉山击杀与战斗关联前置时间</x:v>
       </x:c>
       <x:c r="F61" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2701,19 +2743,19 @@
     </x:row>
     <x:row r="62" ht="33" customHeight="1">
       <x:c r="A62" s="5" t="str">
-        <x:v>roshan_attempt_group_gap</x:v>
+        <x:v>roshan_kill_context_after</x:v>
       </x:c>
       <x:c r="B62" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C62" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D62" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E62" s="5" t="str">
-        <x:v>Roshan伤害组分组间隔</x:v>
+        <x:v>肉山击杀与战斗关联后置时间</x:v>
       </x:c>
       <x:c r="F62" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2725,19 +2767,19 @@
     </x:row>
     <x:row r="63" ht="33" customHeight="1">
       <x:c r="A63" s="5" t="str">
-        <x:v>roshan_attempt_damage_min</x:v>
+        <x:v>roshan_respawn_suppression</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="C63" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D63" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E63" s="5" t="str">
-        <x:v>未击杀Roshan尝试最低伤害</x:v>
+        <x:v>肉山死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2749,10 +2791,10 @@
     </x:row>
     <x:row r="64" ht="33" customHeight="1">
       <x:c r="A64" s="5" t="str">
-        <x:v>roshan_attempt_kill_grace</x:v>
+        <x:v>roshan_attempt_group_gap</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C64" s="5" t="str">
         <x:v>秒</x:v>
@@ -2761,7 +2803,7 @@
         <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E64" s="5" t="str">
-        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
+        <x:v>Roshan伤害组分组间隔</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2773,22 +2815,22 @@
     </x:row>
     <x:row r="65" ht="33" customHeight="1">
       <x:c r="A65" s="5" t="str">
-        <x:v>roshan_drop_merge_window</x:v>
+        <x:v>roshan_attempt_damage_min</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
-        <x:v>20</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C65" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D65" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E65" s="5" t="str">
-        <x:v>肉山击杀后掉落合并窗口</x:v>
+        <x:v>未击杀Roshan尝试最低伤害</x:v>
       </x:c>
       <x:c r="F65" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G65" s="5" t="str">
         <x:v>是</x:v>
@@ -2797,22 +2839,22 @@
     </x:row>
     <x:row r="66" ht="33" customHeight="1">
       <x:c r="A66" s="5" t="str">
-        <x:v>roshan_owner_drop_fallback</x:v>
+        <x:v>roshan_attempt_kill_grace</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C66" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D66" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E66" s="5" t="str">
-        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
+        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G66" s="5" t="str">
         <x:v>是</x:v>
@@ -2821,22 +2863,22 @@
     </x:row>
     <x:row r="67" ht="33" customHeight="1">
       <x:c r="A67" s="5" t="str">
-        <x:v>tormentor_alive_start</x:v>
+        <x:v>roshan_drop_merge_window</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
-        <x:v>1200</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C67" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D67" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E67" s="5" t="str">
-        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
+        <x:v>肉山击杀后掉落合并窗口</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G67" s="5" t="str">
         <x:v>是</x:v>
@@ -2845,22 +2887,22 @@
     </x:row>
     <x:row r="68" ht="33" customHeight="1">
       <x:c r="A68" s="5" t="str">
-        <x:v>tormentor_respawn_suppression</x:v>
+        <x:v>roshan_owner_drop_fallback</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C68" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D68" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E68" s="5" t="str">
-        <x:v>魔晶死亡后该时间内不视为存活</x:v>
+        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
       </x:c>
       <x:c r="F68" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G68" s="5" t="str">
         <x:v>是</x:v>
@@ -2869,19 +2911,19 @@
     </x:row>
     <x:row r="69" ht="33" customHeight="1">
       <x:c r="A69" s="5" t="str">
-        <x:v>tormentor_near_radius</x:v>
+        <x:v>tormentor_alive_start</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="C69" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D69" s="5" t="str">
         <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E69" s="5" t="str">
-        <x:v>独立魔晶击杀附近英雄判断</x:v>
+        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2893,19 +2935,19 @@
     </x:row>
     <x:row r="70" ht="33" customHeight="1">
       <x:c r="A70" s="5" t="str">
-        <x:v>highground_raw_corner</x:v>
+        <x:v>tormentor_respawn_suppression</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
-        <x:v>95/158</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C70" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D70" s="5" t="str">
-        <x:v>高地团</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E70" s="5" t="str">
-        <x:v>高地团中心区域阈值</x:v>
+        <x:v>魔晶死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F70" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2917,19 +2959,19 @@
     </x:row>
     <x:row r="71" ht="33" customHeight="1">
       <x:c r="A71" s="5" t="str">
-        <x:v>tower_context_radius</x:v>
+        <x:v>tormentor_near_radius</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C71" s="5" t="str">
         <x:v>码</x:v>
       </x:c>
       <x:c r="D71" s="5" t="str">
-        <x:v>守塔团</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E71" s="5" t="str">
-        <x:v>防御塔上下文范围</x:v>
+        <x:v>独立魔晶击杀附近英雄判断</x:v>
       </x:c>
       <x:c r="F71" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2941,19 +2983,19 @@
     </x:row>
     <x:row r="72" ht="33" customHeight="1">
       <x:c r="A72" s="5" t="str">
-        <x:v>tower_context_time_pad</x:v>
+        <x:v>highground_raw_corner</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>95/158</x:v>
       </x:c>
       <x:c r="C72" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D72" s="5" t="str">
-        <x:v>守塔团</x:v>
+        <x:v>高地团</x:v>
       </x:c>
       <x:c r="E72" s="5" t="str">
-        <x:v>战斗窗口前后塔状态检测</x:v>
+        <x:v>高地团中心区域阈值</x:v>
       </x:c>
       <x:c r="F72" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2965,22 +3007,22 @@
     </x:row>
     <x:row r="73" ht="33" customHeight="1">
       <x:c r="A73" s="5" t="str">
-        <x:v>aegis_valid_duration</x:v>
+        <x:v>tower_context_radius</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
-        <x:v>300</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C73" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D73" s="5" t="str">
-        <x:v>带盾阵亡</x:v>
+        <x:v>守塔团</x:v>
       </x:c>
       <x:c r="E73" s="5" t="str">
-        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
+        <x:v>防御塔上下文范围</x:v>
       </x:c>
       <x:c r="F73" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G73" s="5" t="str">
         <x:v>是</x:v>
@@ -2989,22 +3031,22 @@
     </x:row>
     <x:row r="74" ht="33" customHeight="1">
       <x:c r="A74" s="5" t="str">
-        <x:v>v1_7_subordinate_overlap_ratio</x:v>
+        <x:v>tower_context_time_pad</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
-        <x:v>0.60</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C74" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D74" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>守塔团</x:v>
       </x:c>
       <x:c r="E74" s="5" t="str">
-        <x:v>旧单点候选与父窗口重叠比例</x:v>
+        <x:v>战斗窗口前后塔状态检测</x:v>
       </x:c>
       <x:c r="F74" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G74" s="5" t="str">
         <x:v>是</x:v>
@@ -3013,22 +3055,22 @@
     </x:row>
     <x:row r="75" ht="33" customHeight="1">
       <x:c r="A75" s="5" t="str">
-        <x:v>v1_7_parent_start_grace</x:v>
+        <x:v>aegis_valid_duration</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C75" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D75" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>带盾阵亡</x:v>
       </x:c>
       <x:c r="E75" s="5" t="str">
-        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
+        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G75" s="5" t="str">
         <x:v>是</x:v>
@@ -3037,19 +3079,19 @@
     </x:row>
     <x:row r="76" ht="33" customHeight="1">
       <x:c r="A76" s="5" t="str">
-        <x:v>v1_7_parent_end_grace</x:v>
+        <x:v>v1_7_subordinate_overlap_ratio</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>0.60</x:v>
       </x:c>
       <x:c r="C76" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D76" s="5" t="str">
         <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E76" s="5" t="str">
-        <x:v>父窗口允许比候选结束最多早5秒</x:v>
+        <x:v>旧单点候选与父窗口重叠比例</x:v>
       </x:c>
       <x:c r="F76" s="5" t="str">
         <x:v>v1.7</x:v>
@@ -3061,22 +3103,22 @@
     </x:row>
     <x:row r="77" ht="33" customHeight="1">
       <x:c r="A77" s="5" t="str">
-        <x:v>v1_8_duplicate_no_kill_gap</x:v>
+        <x:v>v1_7_parent_start_grace</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C77" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D77" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E77" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
+        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
       </x:c>
       <x:c r="F77" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="G77" s="5" t="str">
         <x:v>是</x:v>
@@ -3085,22 +3127,22 @@
     </x:row>
     <x:row r="78" ht="33" customHeight="1">
       <x:c r="A78" s="5" t="str">
-        <x:v>v1_8_duplicate_distance</x:v>
+        <x:v>v1_7_parent_end_grace</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
-        <x:v>1800</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C78" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D78" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E78" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
+        <x:v>父窗口允许比候选结束最多早5秒</x:v>
       </x:c>
       <x:c r="F78" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="G78" s="5" t="str">
         <x:v>是</x:v>
@@ -3109,19 +3151,19 @@
     </x:row>
     <x:row r="79" ht="33" customHeight="1">
       <x:c r="A79" s="5" t="str">
-        <x:v>v1_8_duplicate_jaccard</x:v>
+        <x:v>v1_8_duplicate_no_kill_gap</x:v>
       </x:c>
       <x:c r="B79" s="5" t="str">
-        <x:v>0.50</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C79" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D79" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E79" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
+        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
       </x:c>
       <x:c r="F79" s="5" t="str">
         <x:v>v1.8</x:v>
@@ -3133,19 +3175,19 @@
     </x:row>
     <x:row r="80" ht="33" customHeight="1">
       <x:c r="A80" s="5" t="str">
-        <x:v>v1_8_duplicate_shared_heroes</x:v>
+        <x:v>v1_8_duplicate_distance</x:v>
       </x:c>
       <x:c r="B80" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="C80" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D80" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E80" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
+        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
       </x:c>
       <x:c r="F80" s="5" t="str">
         <x:v>v1.8</x:v>
@@ -3157,22 +3199,22 @@
     </x:row>
     <x:row r="81" ht="33" customHeight="1">
       <x:c r="A81" s="5" t="str">
-        <x:v>v1_9_kill_parent_gap</x:v>
+        <x:v>v1_8_duplicate_jaccard</x:v>
       </x:c>
       <x:c r="B81" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>0.50</x:v>
       </x:c>
       <x:c r="C81" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D81" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E81" s="5" t="str">
-        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
+        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
       </x:c>
       <x:c r="F81" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G81" s="5" t="str">
         <x:v>是</x:v>
@@ -3181,22 +3223,22 @@
     </x:row>
     <x:row r="82" ht="33" customHeight="1">
       <x:c r="A82" s="5" t="str">
-        <x:v>v1_9_kill_parent_distance</x:v>
+        <x:v>v1_8_duplicate_shared_heroes</x:v>
       </x:c>
       <x:c r="B82" s="5" t="str">
-        <x:v>2500</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C82" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D82" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E82" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
+        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
       </x:c>
       <x:c r="F82" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G82" s="5" t="str">
         <x:v>是</x:v>
@@ -3205,19 +3247,19 @@
     </x:row>
     <x:row r="83" ht="33" customHeight="1">
       <x:c r="A83" s="5" t="str">
-        <x:v>v1_9_kill_parent_jaccard</x:v>
+        <x:v>v1_9_kill_parent_gap</x:v>
       </x:c>
       <x:c r="B83" s="5" t="str">
-        <x:v>0.33</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C83" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D83" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E83" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
+        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
       </x:c>
       <x:c r="F83" s="5" t="str">
         <x:v>v1.9</x:v>
@@ -3229,19 +3271,19 @@
     </x:row>
     <x:row r="84" ht="33" customHeight="1">
       <x:c r="A84" s="5" t="str">
-        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+        <x:v>v1_9_kill_parent_distance</x:v>
       </x:c>
       <x:c r="B84" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="C84" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D84" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E84" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
       </x:c>
       <x:c r="F84" s="5" t="str">
         <x:v>v1.9</x:v>
@@ -3253,19 +3295,19 @@
     </x:row>
     <x:row r="85" ht="33" customHeight="1">
       <x:c r="A85" s="5" t="str">
-        <x:v>adjacent_combat_qc_scan_window</x:v>
+        <x:v>v1_9_kill_parent_jaccard</x:v>
       </x:c>
       <x:c r="B85" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>0.33</x:v>
       </x:c>
       <x:c r="C85" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D85" s="5" t="str">
-        <x:v>质量控制</x:v>
+        <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E85" s="5" t="str">
-        <x:v>生成后复查相邻战斗事件的建议扫描窗口</x:v>
+        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
       </x:c>
       <x:c r="F85" s="5" t="str">
         <x:v>v1.9</x:v>
@@ -3274,6 +3316,54 @@
         <x:v>是</x:v>
       </x:c>
       <x:c r="H85" s="5" t="str"/>
+    </x:row>
+    <x:row r="86" ht="33" customHeight="1">
+      <x:c r="A86" s="5" t="str">
+        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+      </x:c>
+      <x:c r="B86" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C86" s="5" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="D86" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E86" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+      </x:c>
+      <x:c r="F86" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G86" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H86" s="5" t="str"/>
+    </x:row>
+    <x:row r="87" ht="33" customHeight="1">
+      <x:c r="A87" s="5" t="str">
+        <x:v>adjacent_combat_qc_scan_window</x:v>
+      </x:c>
+      <x:c r="B87" s="5" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C87" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D87" s="5" t="str">
+        <x:v>质量控制</x:v>
+      </x:c>
+      <x:c r="E87" s="5" t="str">
+        <x:v>生成后复查相邻战斗事件的建议扫描窗口</x:v>
+      </x:c>
+      <x:c r="F87" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G87" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H87" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3523,7 +3613,7 @@
         <x:v>战斗聚类结果</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>小规模冲突; 团战; 特殊战斗</x:v>
+        <x:v>GANK; 小规模冲突; 团战; 特殊战斗</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
         <x:v>供后处理、标签判定、结果字段生成</x:v>
@@ -3790,7 +3880,7 @@
         <x:v>fight_records</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>按参与人数、直接参与人数、伤害、死亡、持续时间输出小规模冲突或团战</x:v>
+        <x:v>先判断GANK：一方直接参与&gt;=2且另一方参与&lt;=1；否则按参与人数、直接参与人数、伤害、死亡、持续时间输出小规模冲突或团战</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
         <x:v>战斗类事件</x:v>
@@ -3799,7 +3889,7 @@
         <x:v>边界事件仍需人工复核</x:v>
       </x:c>
       <x:c r="G9" s="5" t="str">
-        <x:v>旧抓人候选不再作为最终标签</x:v>
+        <x:v>旧抓人候选不再作为最终标签，新增GANK承接N抓1语义</x:v>
       </x:c>
       <x:c r="H9" s="5" t="str"/>
     </x:row>
@@ -4139,13 +4229,13 @@
         <x:v>labels含抓人</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>删除抓人标签；按规则改为小规模冲突/团战或合并入父事件</x:v>
+        <x:v>删除抓人标签；按规则改为GANK/小规模冲突/团战或合并入父事件</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>v1.5后最终定义不再有抓人字段</x:v>
+        <x:v>v1.5后最终定义不再有抓人字段，v1.10新增GANK</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.6-v1.10</x:v>
       </x:c>
       <x:c r="H5" s="5" t="str">
         <x:v>是</x:v>
@@ -4190,7 +4280,7 @@
         <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>与已有团战窗口重叠则团战；与已有小规模冲突重叠则小规模冲突；否则总人数&gt;=8且双方&gt;=3为团战，其余为小规模冲突</x:v>
+        <x:v>符合N抓1则GANK；与已有团战窗口重叠则团战；与已有小规模冲突重叠则小规模冲突；否则总人数&gt;=8且双方&gt;=3为团战，其余为小规模冲突</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
         <x:v>输出新标签，不输出抓人</x:v>
@@ -4199,7 +4289,7 @@
         <x:v>删除抓人后仍保留战斗语义</x:v>
       </x:c>
       <x:c r="G7" s="5" t="str">
-        <x:v>v1.6/v1.7</x:v>
+        <x:v>v1.6/v1.7/v1.10</x:v>
       </x:c>
       <x:c r="H7" s="5" t="str">
         <x:v>是</x:v>
@@ -4495,7 +4585,7 @@
         <x:v>文本</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
-        <x:v>来自定义清单18标签</x:v>
+        <x:v>来自定义清单19标签</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Update tactical event detection rules
</commit_message>
<xml_diff>
--- a/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
+++ b/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="R52430d6d03b54468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R1a1dafd9342c4bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="Re7334227fca948aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="R5086d585c1cf4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="R032ee5b4c3684f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="Rc6e77f80072f440c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="Rf8c04ab986344579"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="R0a3280bdb40145c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="R0a21b3cc89e249be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R63c73b3cf1fa401a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="R5fa85baa19184443"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="R5536d8e563884136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="Rf506a7f3cfe348ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="R0c81e77238274d07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="R57aa5b0a3b014371"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="R4db5c72510df4e5f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -168,12 +168,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -512,28 +558,28 @@
         <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>某阵营某一路线上小兵死亡；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外；死亡小兵500范围内存在敌方线上小兵；若敌方英雄获得该小兵死亡经验，则输出勾兵</x:v>
+        <x:v>某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内存在敌方线上小兵；若敌方英雄获得该小兵死亡经验，则输出勾兵</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
         <x:v>通常00:00-10:00</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
-        <x:v>lane_zone外；附近敌方小兵半径500码；连续小兵死亡默认10秒窗口合并</x:v>
+        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；连续小兵死亡默认10秒窗口合并</x:v>
       </x:c>
       <x:c r="H3" s="5" t="str">
-        <x:v>获得经验的敌方英雄；多人获得经验则全部列入</x:v>
+        <x:v>获得经验的敌方英雄；多人获得经验则全部列入；结果中附获得经验英雄0-5分钟主对线路</x:v>
       </x:c>
       <x:c r="I3" s="5" t="str">
-        <x:v>结果=获得经验英雄获得被勾兵阵营某路线小兵死亡经验；可附死亡小兵数量和附近敌方小兵证据</x:v>
+        <x:v>结果=获得经验英雄获得被勾兵阵营某来源路线小兵死亡经验；可附死亡小兵数量、附近敌方小兵证据和source_lane_method</x:v>
       </x:c>
       <x:c r="J3" s="5" t="str">
-        <x:v>单个小兵死亡作为证据；按获得经验阵营+被勾兵阵营+路线聚合，连续窗口合并输出</x:v>
+        <x:v>单个小兵死亡作为证据；按获得经验阵营+被勾兵阵营+source_lane聚合，连续窗口合并输出；塔下吃兵不输出</x:v>
       </x:c>
       <x:c r="K3" s="5" t="str">
         <x:v>与断线互斥：附近无敌方小兵为断线证据，附近有敌方小兵且敌方英雄获经验则输出勾兵</x:v>
       </x:c>
       <x:c r="L3" s="5" t="str">
-        <x:v>需要lane_zone、活体线上小兵位置和经验获得明细；缺失时只能弱候选，不能填写确定结果</x:v>
+        <x:v>需要lane_zone、活体线上小兵位置、经验获得明细和source_lane；缺失个体轨迹时必须在evidence标记xy_fallback</x:v>
       </x:c>
       <x:c r="M3" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -554,28 +600,28 @@
         <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>10分钟前某阵营某一路线上小兵死亡；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外；死亡小兵500范围内无敌方线上小兵；击杀来源可映射为敌方英雄</x:v>
+        <x:v>10分钟前某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内无敌方线上小兵；击杀来源可映射为敌方英雄</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
         <x:v>通常00:00-10:00</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str">
-        <x:v>lane_zone外；附近敌方小兵半径500码；同一英雄同一路线10秒内连续触发&gt;=2或&gt;=3个小兵死亡后输出</x:v>
+        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；同一英雄同一source_lane 10秒内连续触发&gt;=2或&gt;=3个小兵死亡后输出</x:v>
       </x:c>
       <x:c r="H4" s="5" t="str">
-        <x:v>执行断兵的敌方英雄</x:v>
+        <x:v>执行断兵的敌方英雄；结果中附执行英雄0-5分钟主对线路</x:v>
       </x:c>
       <x:c r="I4" s="5" t="str">
-        <x:v>结果=断兵英雄、被断兵阵营、路线、小兵数量、一塔存活证据</x:v>
+        <x:v>结果=断兵英雄主对线路、被断兵阵营、小兵来源路线、小兵数量、一塔存活证据；例：中路英雄在下路断下路兵</x:v>
       </x:c>
       <x:c r="J4" s="5" t="str">
-        <x:v>单个小兵死亡只作为证据；按击杀英雄+被断兵阵营+路线聚合，连续10秒窗口达到阈值才输出事件</x:v>
+        <x:v>单个小兵死亡只作为证据；按击杀英雄+被断兵阵营+source_lane聚合，连续10秒窗口达到阈值才输出事件；塔下吃兵不输出</x:v>
       </x:c>
       <x:c r="K4" s="5" t="str">
         <x:v>与拉野、正常兵线交汇清线互斥；一塔已掉后不判断线</x:v>
       </x:c>
       <x:c r="L4" s="5" t="str">
-        <x:v>需要lane_zone和活体线上小兵位置；若缺少该数据，只能输出弱候选或暂不自动输出</x:v>
+        <x:v>需要lane_zone、活体线上小兵位置和source_lane；若缺少个体轨迹，必须在evidence标记xy_fallback</x:v>
       </x:c>
       <x:c r="M4" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -593,25 +639,25 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>combat_logs</x:v>
+        <x:v>combat_logs; dota_model_neutral_siege_creep; player_intervals2</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>15分钟前线上小兵与中立单位发生连续伤害/死亡交互；中路排除；同组位置相近且时间间隔&lt;=35秒</x:v>
+        <x:v>15分钟前线上小兵与中立单位发生直接伤害/死亡交互；combat直接交互作为锚点，若连续伤害缺失，则用锚点前8秒到后2秒内线兵-同名野怪距离&lt;=9 raw的状态贴近补证据；中路排除</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
         <x:v>00:00-15:00</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
-        <x:v>拉野组间隔35秒；位置距离28 raw；附近英雄1500码</x:v>
+        <x:v>拉野组间隔35秒；位置距离28 raw；状态贴近距离9 raw；附近英雄1500码</x:v>
       </x:c>
       <x:c r="H5" s="5" t="str">
         <x:v>附近双方/己方英雄，去重输出</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
-        <x:v>结果=线上小兵与中立单位交互样例</x:v>
+        <x:v>结果=某方某路小兵与中立单位连续交战；无ehandle时evidence写synthetic状态点</x:v>
       </x:c>
       <x:c r="J5" s="5" t="str">
-        <x:v>死亡&lt;2且交互&lt;3则过滤</x:v>
+        <x:v>死亡&lt;2且交互&lt;3则过滤；只有状态贴近、无combat锚点不输出</x:v>
       </x:c>
       <x:c r="K5" s="5" t="str">
         <x:v>与断线、普通野区交互需复核</x:v>
@@ -620,7 +666,7 @@
         <x:v>英雄拉仇恨起点仍需人工核查</x:v>
       </x:c>
       <x:c r="M5" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N5" s="5" t="str"/>
     </x:row>
@@ -806,28 +852,28 @@
         <x:v>combat_logs; player_intervals2</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>战斗聚类中一方N抓1：一方参与英雄&gt;=2，另一方参与英雄&lt;=1</x:v>
+        <x:v>发起阶段 N 抓 1：短窗口内同一目标被同一方至少2名英雄命中，且发起时刻目标附近被抓方只有该目标1人</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>聚类开始-结束</x:v>
+        <x:v>发起时刻t0所在战斗窗口</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
-        <x:v>继承战斗聚类时间/空间阈值；参与英雄=进入同一战斗簇的攻击者、受击者、被控制者或死亡者</x:v>
+        <x:v>GANK_OPEN_WINDOW=8秒；t0取第二名不同进攻方英雄第一次命中目标；读取t0±1秒英雄位置；以被抓目标为中心1600码统计附近英雄</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str">
-        <x:v>gank方英雄 + 被抓英雄</x:v>
+        <x:v>gank方发起英雄 + 被抓英雄 + 后续支援/反打英雄</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
-        <x:v>结果=击杀比分；死亡列表；无死亡写未记录英雄击杀/死亡无</x:v>
+        <x:v>结果=GANK方、被抓目标、后续支援/反打、击杀比分和死亡列表；1换1仍保留GANK语义</x:v>
       </x:c>
       <x:c r="J10" s="5" t="str">
-        <x:v>优先于小规模冲突判定；后续可被守塔团/高地团/肉山团等特殊上下文修饰</x:v>
+        <x:v>优先于小规模冲突；后续TP/走入/支援不取消GANK；塔附近信息写入结果/evidence，不自动改成守塔团</x:v>
       </x:c>
       <x:c r="K10" s="5" t="str">
-        <x:v>低于团战特殊上下文，高于小规模冲突</x:v>
+        <x:v>高于小规模冲突；默认不被守塔团/肉山团等上下文改写</x:v>
       </x:c>
       <x:c r="L10" s="5" t="str">
-        <x:v>需要人工校准N抓1但未实质开战、远程消耗等边界</x:v>
+        <x:v>需要人工校准远程消耗、多人已在场、支援是否已在t0±1秒战场半径内等边界</x:v>
       </x:c>
       <x:c r="M10" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1493,22 +1539,22 @@
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>stack_event_window</x:v>
+        <x:v>lane_zone_tower_protect_radius</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>±5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>囤野/堆野</x:v>
+        <x:v>对线区</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>堆野计数增加事件输出窗口</x:v>
+        <x:v>该路线任一存活一塔附近视为正常塔下吃兵区，不进入断线/勾兵候选</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
         <x:v>是</x:v>
@@ -1517,22 +1563,22 @@
     </x:row>
     <x:row r="11" ht="33" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>pull_lane_max_time</x:v>
+        <x:v>lane_creep_source_early_seconds</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>900</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>对线区</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>拉野候选只看前15分钟</x:v>
+        <x:v>有ehandle时用小兵最早出现后8秒内轨迹判断source_lane</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
         <x:v>是</x:v>
@@ -1541,19 +1587,19 @@
     </x:row>
     <x:row r="12" ht="33" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>pull_group_gap</x:v>
+        <x:v>stack_event_window</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>35</x:v>
+        <x:v>±5</x:v>
       </x:c>
       <x:c r="C12" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>囤野/堆野</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>线上兵与中立交互合并为同一拉野组的最大间隔</x:v>
+        <x:v>堆野计数增加事件输出窗口</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -1565,19 +1611,19 @@
     </x:row>
     <x:row r="13" ht="33" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>pull_group_distance_raw</x:v>
+        <x:v>pull_lane_max_time</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>28</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>拉野组位置合并距离</x:v>
+        <x:v>拉野候选只看前15分钟</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -1589,19 +1635,19 @@
     </x:row>
     <x:row r="14" ht="33" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>pull_nearby_hero_radius</x:v>
+        <x:v>pull_group_gap</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E14" s="5" t="str">
-        <x:v>拉野附近英雄归属半径</x:v>
+        <x:v>线上兵与中立交互合并为同一拉野组的最大间隔</x:v>
       </x:c>
       <x:c r="F14" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -1613,22 +1659,22 @@
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>aggro_lane_max_time</x:v>
+        <x:v>pull_group_distance_raw</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C15" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D15" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
-        <x:v>勾兵候选默认只看前10分钟，可由人工样本校准</x:v>
+        <x:v>拉野组位置合并距离</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G15" s="5" t="str">
         <x:v>是</x:v>
@@ -1637,19 +1683,19 @@
     </x:row>
     <x:row r="16" ht="33" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>aggro_lane_enemy_creep_radius</x:v>
+        <x:v>pull_status_proximity_raw</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>500</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>死亡小兵附近存在敌方线上小兵的判定半径</x:v>
+        <x:v>combat锚点附近线兵与同名中立野怪状态贴近的最大距离</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1661,22 +1707,22 @@
     </x:row>
     <x:row r="17" ht="33" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>aggro_lane_group_gap</x:v>
+        <x:v>pull_nearby_hero_radius</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C17" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D17" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E17" s="5" t="str">
-        <x:v>同一路线连续勾兵证据合并窗口</x:v>
+        <x:v>拉野附近英雄归属半径</x:v>
       </x:c>
       <x:c r="F17" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
         <x:v>是</x:v>
@@ -1685,7 +1731,7 @@
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>cut_lane_max_time</x:v>
+        <x:v>aggro_lane_max_time</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
         <x:v>600</x:v>
@@ -1694,10 +1740,10 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
-        <x:v>断线候选只看前10分钟</x:v>
+        <x:v>勾兵候选默认只看前10分钟，可由人工样本校准</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1709,7 +1755,7 @@
     </x:row>
     <x:row r="19" ht="33" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>cut_lane_enemy_creep_radius</x:v>
+        <x:v>aggro_lane_enemy_creep_radius</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
         <x:v>500</x:v>
@@ -1718,10 +1764,10 @@
         <x:v>码</x:v>
       </x:c>
       <x:c r="D19" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E19" s="5" t="str">
-        <x:v>死亡小兵附近无敌方线上小兵的判定半径</x:v>
+        <x:v>死亡小兵附近存在敌方线上小兵的判定半径</x:v>
       </x:c>
       <x:c r="F19" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1733,7 +1779,7 @@
     </x:row>
     <x:row r="20" ht="33" customHeight="1">
       <x:c r="A20" s="5" t="str">
-        <x:v>cut_lane_group_gap</x:v>
+        <x:v>aggro_lane_group_gap</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
         <x:v>10</x:v>
@@ -1742,10 +1788,10 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E20" s="5" t="str">
-        <x:v>同一英雄同一路线连续断兵证据合并窗口</x:v>
+        <x:v>同一路线连续勾兵证据合并窗口</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1757,19 +1803,19 @@
     </x:row>
     <x:row r="21" ht="33" customHeight="1">
       <x:c r="A21" s="5" t="str">
-        <x:v>cut_lane_min_creep_deaths</x:v>
+        <x:v>cut_lane_max_time</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>2或3</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C21" s="5" t="str">
-        <x:v>个</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
         <x:v>断线</x:v>
       </x:c>
       <x:c r="E21" s="5" t="str">
-        <x:v>10秒窗口内符合断线单条证据的小兵死亡数量阈值；2偏召回，3偏精确，需假设检验确定</x:v>
+        <x:v>断线候选只看前10分钟</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1781,22 +1827,22 @@
     </x:row>
     <x:row r="22" ht="33" customHeight="1">
       <x:c r="A22" s="5" t="str">
-        <x:v>rune_near_radius</x:v>
+        <x:v>cut_lane_enemy_creep_radius</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="C22" s="5" t="str">
         <x:v>码</x:v>
       </x:c>
       <x:c r="D22" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E22" s="5" t="str">
-        <x:v>符点附近两方英雄识别半径</x:v>
+        <x:v>死亡小兵附近无敌方线上小兵的判定半径</x:v>
       </x:c>
       <x:c r="F22" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G22" s="5" t="str">
         <x:v>是</x:v>
@@ -1805,22 +1851,22 @@
     </x:row>
     <x:row r="23" ht="33" customHeight="1">
       <x:c r="A23" s="5" t="str">
-        <x:v>power_rune_spawn_interval</x:v>
+        <x:v>cut_lane_group_gap</x:v>
       </x:c>
       <x:c r="B23" s="5" t="str">
-        <x:v>120</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C23" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D23" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E23" s="5" t="str">
-        <x:v>河道能量符刷新间隔，用于未刷新侧控符</x:v>
+        <x:v>同一英雄同一路线连续断兵证据合并窗口</x:v>
       </x:c>
       <x:c r="F23" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G23" s="5" t="str">
         <x:v>是</x:v>
@@ -1829,22 +1875,22 @@
     </x:row>
     <x:row r="24" ht="33" customHeight="1">
       <x:c r="A24" s="5" t="str">
-        <x:v>power_rune_min_spawn_time</x:v>
+        <x:v>cut_lane_min_creep_deaths</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
-        <x:v>360</x:v>
+        <x:v>2或3</x:v>
       </x:c>
       <x:c r="C24" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="D24" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E24" s="5" t="str">
-        <x:v>能量符最早按6分钟刷新计算</x:v>
+        <x:v>10秒窗口内符合断线单条证据的小兵死亡数量阈值；2偏召回，3偏精确，需假设检验确定</x:v>
       </x:c>
       <x:c r="F24" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G24" s="5" t="str">
         <x:v>是</x:v>
@@ -1853,19 +1899,19 @@
     </x:row>
     <x:row r="25" ht="33" customHeight="1">
       <x:c r="A25" s="5" t="str">
-        <x:v>power_rune_spawn_match_tolerance</x:v>
+        <x:v>rune_near_radius</x:v>
       </x:c>
       <x:c r="B25" s="5" t="str">
-        <x:v>90</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C25" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D25" s="5" t="str">
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E25" s="5" t="str">
-        <x:v>将结果事件反推到最近能量符刷新点的容差</x:v>
+        <x:v>符点附近两方英雄识别半径</x:v>
       </x:c>
       <x:c r="F25" s="5" t="str">
         <x:v>v1.5</x:v>
@@ -1877,10 +1923,10 @@
     </x:row>
     <x:row r="26" ht="33" customHeight="1">
       <x:c r="A26" s="5" t="str">
-        <x:v>rune_bottle_pickup_suppression</x:v>
+        <x:v>power_rune_spawn_interval</x:v>
       </x:c>
       <x:c r="B26" s="5" t="str">
-        <x:v>90</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C26" s="5" t="str">
         <x:v>秒</x:v>
@@ -1889,7 +1935,7 @@
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E26" s="5" t="str">
-        <x:v>同英雄同神符罐装后拾取日志去重窗口</x:v>
+        <x:v>河道能量符刷新间隔，用于未刷新侧控符</x:v>
       </x:c>
       <x:c r="F26" s="5" t="str">
         <x:v>v1.5</x:v>
@@ -1901,10 +1947,10 @@
     </x:row>
     <x:row r="27" ht="33" customHeight="1">
       <x:c r="A27" s="5" t="str">
-        <x:v>wisdom_rune_window</x:v>
+        <x:v>power_rune_min_spawn_time</x:v>
       </x:c>
       <x:c r="B27" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str">
         <x:v>秒</x:v>
@@ -1913,7 +1959,7 @@
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E27" s="5" t="str">
-        <x:v>智慧符事件起点=t-10</x:v>
+        <x:v>能量符最早按6分钟刷新计算</x:v>
       </x:c>
       <x:c r="F27" s="5" t="str">
         <x:v>v1.5</x:v>
@@ -1925,22 +1971,22 @@
     </x:row>
     <x:row r="28" ht="33" customHeight="1">
       <x:c r="A28" s="5" t="str">
-        <x:v>smoke_link_window</x:v>
+        <x:v>power_rune_spawn_match_tolerance</x:v>
       </x:c>
       <x:c r="B28" s="5" t="str">
-        <x:v>120</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E28" s="5" t="str">
-        <x:v>开雾使用与modifier关联最大窗口</x:v>
+        <x:v>将结果事件反推到最近能量符刷新点的容差</x:v>
       </x:c>
       <x:c r="F28" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G28" s="5" t="str">
         <x:v>是</x:v>
@@ -1949,22 +1995,22 @@
     </x:row>
     <x:row r="29" ht="33" customHeight="1">
       <x:c r="A29" s="5" t="str">
-        <x:v>smoke_modifier_near_window</x:v>
+        <x:v>rune_bottle_pickup_suppression</x:v>
       </x:c>
       <x:c r="B29" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D29" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E29" s="5" t="str">
-        <x:v>无施法者关联时按同队modifier时间兜底</x:v>
+        <x:v>同英雄同神符罐装后拾取日志去重窗口</x:v>
       </x:c>
       <x:c r="F29" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G29" s="5" t="str">
         <x:v>是</x:v>
@@ -1973,22 +2019,22 @@
     </x:row>
     <x:row r="30" ht="33" customHeight="1">
       <x:c r="A30" s="5" t="str">
-        <x:v>smoke_fallback_near_radius</x:v>
+        <x:v>wisdom_rune_window</x:v>
       </x:c>
       <x:c r="B30" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C30" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D30" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E30" s="5" t="str">
-        <x:v>无modifier时按使用者附近队友兜底</x:v>
+        <x:v>智慧符事件起点=t-10</x:v>
       </x:c>
       <x:c r="F30" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G30" s="5" t="str">
         <x:v>是</x:v>
@@ -1997,19 +2043,19 @@
     </x:row>
     <x:row r="31" ht="33" customHeight="1">
       <x:c r="A31" s="5" t="str">
-        <x:v>combat_damage_min_event</x:v>
+        <x:v>smoke_link_window</x:v>
       </x:c>
       <x:c r="B31" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D31" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E31" s="5" t="str">
-        <x:v>进入战斗检测的单条伤害最小值</x:v>
+        <x:v>开雾使用与modifier关联最大窗口</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2021,19 +2067,19 @@
     </x:row>
     <x:row r="32" ht="33" customHeight="1">
       <x:c r="A32" s="5" t="str">
-        <x:v>combat_seed_damage</x:v>
+        <x:v>smoke_modifier_near_window</x:v>
       </x:c>
       <x:c r="B32" s="5" t="str">
-        <x:v>550</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C32" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E32" s="5" t="str">
-        <x:v>初始空间簇成为战斗候选的伤害阈值，死亡可替代</x:v>
+        <x:v>无施法者关联时按同队modifier时间兜底</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2045,19 +2091,19 @@
     </x:row>
     <x:row r="33" ht="33" customHeight="1">
       <x:c r="A33" s="5" t="str">
-        <x:v>combat_refined_damage</x:v>
+        <x:v>smoke_fallback_near_radius</x:v>
       </x:c>
       <x:c r="B33" s="5" t="str">
-        <x:v>900</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C33" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D33" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E33" s="5" t="str">
-        <x:v>细化后无死亡战斗的最低总伤害</x:v>
+        <x:v>无modifier时按使用者附近队友兜底</x:v>
       </x:c>
       <x:c r="F33" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2069,19 +2115,19 @@
     </x:row>
     <x:row r="34" ht="33" customHeight="1">
       <x:c r="A34" s="5" t="str">
-        <x:v>combat_bucket</x:v>
+        <x:v>combat_damage_min_event</x:v>
       </x:c>
       <x:c r="B34" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D34" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E34" s="5" t="str">
-        <x:v>战斗检测分桶</x:v>
+        <x:v>进入战斗检测的单条伤害最小值</x:v>
       </x:c>
       <x:c r="F34" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2093,19 +2139,19 @@
     </x:row>
     <x:row r="35" ht="33" customHeight="1">
       <x:c r="A35" s="5" t="str">
-        <x:v>combat_cluster_distance_raw</x:v>
+        <x:v>combat_seed_damage</x:v>
       </x:c>
       <x:c r="B35" s="5" t="str">
-        <x:v>38</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="C35" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D35" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E35" s="5" t="str">
-        <x:v>同10秒桶内空间聚类距离</x:v>
+        <x:v>初始空间簇成为战斗候选的伤害阈值，死亡可替代</x:v>
       </x:c>
       <x:c r="F35" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2117,19 +2163,19 @@
     </x:row>
     <x:row r="36" ht="33" customHeight="1">
       <x:c r="A36" s="5" t="str">
-        <x:v>combat_cluster_merge_gap</x:v>
+        <x:v>combat_refined_damage</x:v>
       </x:c>
       <x:c r="B36" s="5" t="str">
-        <x:v>12</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C36" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D36" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E36" s="5" t="str">
-        <x:v>相邻空间簇合并最大时间间隔</x:v>
+        <x:v>细化后无死亡战斗的最低总伤害</x:v>
       </x:c>
       <x:c r="F36" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2141,19 +2187,19 @@
     </x:row>
     <x:row r="37" ht="33" customHeight="1">
       <x:c r="A37" s="5" t="str">
-        <x:v>combat_cluster_merge_distance_raw</x:v>
+        <x:v>combat_bucket</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>48</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C37" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D37" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E37" s="5" t="str">
-        <x:v>相邻空间簇合并最大中心距离</x:v>
+        <x:v>战斗检测分桶</x:v>
       </x:c>
       <x:c r="F37" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2165,19 +2211,19 @@
     </x:row>
     <x:row r="38" ht="33" customHeight="1">
       <x:c r="A38" s="5" t="str">
-        <x:v>combat_refine_time_pad</x:v>
+        <x:v>combat_cluster_distance_raw</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>6</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C38" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D38" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E38" s="5" t="str">
-        <x:v>细化收集伤害/控制/死亡的前后时间</x:v>
+        <x:v>同10秒桶内空间聚类距离</x:v>
       </x:c>
       <x:c r="F38" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2189,19 +2235,19 @@
     </x:row>
     <x:row r="39" ht="33" customHeight="1">
       <x:c r="A39" s="5" t="str">
-        <x:v>combat_refine_distance_raw</x:v>
+        <x:v>combat_cluster_merge_gap</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
-        <x:v>62</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C39" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D39" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E39" s="5" t="str">
-        <x:v>细化事件距离中心最大距离</x:v>
+        <x:v>相邻空间簇合并最大时间间隔</x:v>
       </x:c>
       <x:c r="F39" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2213,22 +2259,22 @@
     </x:row>
     <x:row r="40" ht="33" customHeight="1">
       <x:c r="A40" s="5" t="str">
-        <x:v>combat_participant_radius</x:v>
+        <x:v>combat_cluster_merge_distance_raw</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
-        <x:v>1600</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="C40" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D40" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E40" s="5" t="str">
-        <x:v>英雄参与战斗核心的默认最大距离</x:v>
+        <x:v>相邻空间簇合并最大中心距离</x:v>
       </x:c>
       <x:c r="F40" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G40" s="5" t="str">
         <x:v>是</x:v>
@@ -2237,45 +2283,43 @@
     </x:row>
     <x:row r="41" ht="33" customHeight="1">
       <x:c r="A41" s="5" t="str">
-        <x:v>combat_midlane_exclusion_distance</x:v>
+        <x:v>combat_refine_time_pad</x:v>
       </x:c>
       <x:c r="B41" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C41" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D41" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E41" s="5" t="str">
-        <x:v>边路冲突中心时，中路线英雄超过该距离且未命中核心目标则排除</x:v>
+        <x:v>细化收集伤害/控制/死亡的前后时间</x:v>
       </x:c>
       <x:c r="F41" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G41" s="5" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="H41" s="5" t="str">
-        <x:v>本质是远端未交互排除，不限中路或10分钟前</x:v>
-      </x:c>
+      <x:c r="H41" s="5" t="str"/>
     </x:row>
     <x:row r="42" ht="33" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>combat_nearby_teammate_radius</x:v>
+        <x:v>combat_refine_distance_raw</x:v>
       </x:c>
       <x:c r="B42" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D42" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E42" s="5" t="str">
-        <x:v>细化阶段把近处同队英雄补入参战者</x:v>
+        <x:v>细化事件距离中心最大距离</x:v>
       </x:c>
       <x:c r="F42" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2287,22 +2331,22 @@
     </x:row>
     <x:row r="43" ht="33" customHeight="1">
       <x:c r="A43" s="5" t="str">
-        <x:v>teamfight_min_side_count</x:v>
+        <x:v>combat_participant_radius</x:v>
       </x:c>
       <x:c r="B43" s="5" t="str">
-        <x:v>4</x:v>
+        <x:v>1600</x:v>
       </x:c>
       <x:c r="C43" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D43" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E43" s="5" t="str">
-        <x:v>双方总参与各至少4人</x:v>
+        <x:v>英雄参与战斗核心的默认最大距离</x:v>
       </x:c>
       <x:c r="F43" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G43" s="5" t="str">
         <x:v>是</x:v>
@@ -2311,43 +2355,45 @@
     </x:row>
     <x:row r="44" ht="33" customHeight="1">
       <x:c r="A44" s="5" t="str">
-        <x:v>teamfight_min_direct_count</x:v>
+        <x:v>combat_midlane_exclusion_distance</x:v>
       </x:c>
       <x:c r="B44" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C44" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D44" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E44" s="5" t="str">
-        <x:v>双方直接参与各至少3人</x:v>
+        <x:v>边路冲突中心时，中路线英雄超过该距离且未命中核心目标则排除</x:v>
       </x:c>
       <x:c r="F44" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G44" s="5" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="H44" s="5" t="str"/>
+      <x:c r="H44" s="5" t="str">
+        <x:v>本质是远端未交互排除，不限中路或10分钟前</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="33" customHeight="1">
       <x:c r="A45" s="5" t="str">
-        <x:v>teamfight_damage_threshold</x:v>
+        <x:v>combat_nearby_teammate_radius</x:v>
       </x:c>
       <x:c r="B45" s="5" t="str">
-        <x:v>2500</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C45" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D45" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E45" s="5" t="str">
-        <x:v>达团战规模时的伤害阈值</x:v>
+        <x:v>细化阶段把近处同队英雄补入参战者</x:v>
       </x:c>
       <x:c r="F45" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2359,19 +2405,19 @@
     </x:row>
     <x:row r="46" ht="33" customHeight="1">
       <x:c r="A46" s="5" t="str">
-        <x:v>teamfight_death_threshold</x:v>
+        <x:v>teamfight_min_side_count</x:v>
       </x:c>
       <x:c r="B46" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str">
-        <x:v>死亡</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D46" s="5" t="str">
         <x:v>团战</x:v>
       </x:c>
       <x:c r="E46" s="5" t="str">
-        <x:v>达团战规模时死亡数阈值</x:v>
+        <x:v>双方总参与各至少4人</x:v>
       </x:c>
       <x:c r="F46" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2383,19 +2429,19 @@
     </x:row>
     <x:row r="47" ht="33" customHeight="1">
       <x:c r="A47" s="5" t="str">
-        <x:v>teamfight_duration_threshold</x:v>
+        <x:v>teamfight_min_direct_count</x:v>
       </x:c>
       <x:c r="B47" s="5" t="str">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D47" s="5" t="str">
         <x:v>团战</x:v>
       </x:c>
       <x:c r="E47" s="5" t="str">
-        <x:v>达团战规模时持续时长阈值</x:v>
+        <x:v>双方直接参与各至少3人</x:v>
       </x:c>
       <x:c r="F47" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2407,22 +2453,22 @@
     </x:row>
     <x:row r="48" ht="33" customHeight="1">
       <x:c r="A48" s="5" t="str">
-        <x:v>gank_min_attacker_side_heroes</x:v>
+        <x:v>teamfight_damage_threshold</x:v>
       </x:c>
       <x:c r="B48" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D48" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E48" s="5" t="str">
-        <x:v>GANK方至少有2名参与英雄，参与英雄指进入同一战斗簇的攻击者、受击者、被控制者或死亡者</x:v>
+        <x:v>达团战规模时的伤害阈值</x:v>
       </x:c>
       <x:c r="F48" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G48" s="5" t="str">
         <x:v>是</x:v>
@@ -2431,22 +2477,22 @@
     </x:row>
     <x:row r="49" ht="33" customHeight="1">
       <x:c r="A49" s="5" t="str">
-        <x:v>gank_max_victim_side_heroes</x:v>
+        <x:v>teamfight_death_threshold</x:v>
       </x:c>
       <x:c r="B49" s="5" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>死亡</x:v>
       </x:c>
       <x:c r="D49" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E49" s="5" t="str">
-        <x:v>被抓一方参与英雄最多1人，即N抓1</x:v>
+        <x:v>达团战规模时死亡数阈值</x:v>
       </x:c>
       <x:c r="F49" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G49" s="5" t="str">
         <x:v>是</x:v>
@@ -2455,19 +2501,19 @@
     </x:row>
     <x:row r="50" ht="33" customHeight="1">
       <x:c r="A50" s="5" t="str">
-        <x:v>skirmish_max_total_heroes</x:v>
+        <x:v>teamfight_duration_threshold</x:v>
       </x:c>
       <x:c r="B50" s="5" t="str">
-        <x:v>7</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D50" s="5" t="str">
-        <x:v>小规模冲突</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E50" s="5" t="str">
-        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
+        <x:v>达团战规模时持续时长阈值</x:v>
       </x:c>
       <x:c r="F50" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2479,7 +2525,7 @@
     </x:row>
     <x:row r="51" ht="33" customHeight="1">
       <x:c r="A51" s="5" t="str">
-        <x:v>fight_dedup_gap_initial</x:v>
+        <x:v>gank_open_window</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
         <x:v>8</x:v>
@@ -2488,13 +2534,13 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D51" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E51" s="5" t="str">
-        <x:v>初始fight record近邻合并时间</x:v>
+        <x:v>同一目标在短窗口内被同一方至少2名不同英雄命中，才进入GANK候选</x:v>
       </x:c>
       <x:c r="F51" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G51" s="5" t="str">
         <x:v>是</x:v>
@@ -2503,22 +2549,22 @@
     </x:row>
     <x:row r="52" ht="33" customHeight="1">
       <x:c r="A52" s="5" t="str">
-        <x:v>fight_dedup_distance_raw</x:v>
+        <x:v>gank_position_sample_window</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>58</x:v>
+        <x:v>±1</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D52" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E52" s="5" t="str">
-        <x:v>初始fight record近邻合并距离</x:v>
+        <x:v>读取发起时刻t0前后1秒的英雄位置；同一英雄取距离t0最近的位置</x:v>
       </x:c>
       <x:c r="F52" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G52" s="5" t="str">
         <x:v>是</x:v>
@@ -2527,22 +2573,22 @@
     </x:row>
     <x:row r="53" ht="33" customHeight="1">
       <x:c r="A53" s="5" t="str">
-        <x:v>fight_overlap_shared_heroes</x:v>
+        <x:v>gank_position_radius</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>1600</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D53" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E53" s="5" t="str">
-        <x:v>重叠fight record合并的共享英雄数</x:v>
+        <x:v>以被抓目标位置为中心统计发起阶段附近英雄</x:v>
       </x:c>
       <x:c r="F53" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G53" s="5" t="str">
         <x:v>是</x:v>
@@ -2551,22 +2597,22 @@
     </x:row>
     <x:row r="54" ht="33" customHeight="1">
       <x:c r="A54" s="5" t="str">
-        <x:v>pickoff_enemy_damage_ratio</x:v>
+        <x:v>gank_min_attacker_nearby_heroes</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>0.80</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D54" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E54" s="5" t="str">
-        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
+        <x:v>发起时刻战场半径内GANK方至少2名英雄，且至少2名英雄直接命中同一目标</x:v>
       </x:c>
       <x:c r="F54" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G54" s="5" t="str">
         <x:v>是</x:v>
@@ -2575,7 +2621,7 @@
     </x:row>
     <x:row r="55" ht="33" customHeight="1">
       <x:c r="A55" s="5" t="str">
-        <x:v>pickoff_ally_near_limit</x:v>
+        <x:v>gank_max_victim_nearby_heroes</x:v>
       </x:c>
       <x:c r="B55" s="5" t="str">
         <x:v>1</x:v>
@@ -2584,13 +2630,13 @@
         <x:v>人</x:v>
       </x:c>
       <x:c r="D55" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E55" s="5" t="str">
-        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
+        <x:v>发起时刻战场半径内被抓方只有被抓目标1名英雄；后续TP/走入只影响结果，不取消GANK</x:v>
       </x:c>
       <x:c r="F55" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G55" s="5" t="str">
         <x:v>是</x:v>
@@ -2599,22 +2645,22 @@
     </x:row>
     <x:row r="56" ht="33" customHeight="1">
       <x:c r="A56" s="5" t="str">
-        <x:v>escape_pickoff_window</x:v>
+        <x:v>skirmish_max_total_heroes</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>18</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D56" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E56" s="5" t="str">
-        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
+        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
       </x:c>
       <x:c r="F56" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G56" s="5" t="str">
         <x:v>是</x:v>
@@ -2623,22 +2669,22 @@
     </x:row>
     <x:row r="57" ht="33" customHeight="1">
       <x:c r="A57" s="5" t="str">
-        <x:v>escape_pickoff_damage_min</x:v>
+        <x:v>fight_dedup_gap_initial</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>180</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D57" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E57" s="5" t="str">
-        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
+        <x:v>初始fight record近邻合并时间</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
         <x:v>是</x:v>
@@ -2647,19 +2693,19 @@
     </x:row>
     <x:row r="58" ht="33" customHeight="1">
       <x:c r="A58" s="5" t="str">
-        <x:v>roshan_context_radius</x:v>
+        <x:v>fight_dedup_distance_raw</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>2000</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D58" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E58" s="5" t="str">
-        <x:v>肉山团上下文范围</x:v>
+        <x:v>初始fight record近邻合并距离</x:v>
       </x:c>
       <x:c r="F58" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2671,19 +2717,19 @@
     </x:row>
     <x:row r="59" ht="33" customHeight="1">
       <x:c r="A59" s="5" t="str">
-        <x:v>roshan_context_min_time</x:v>
+        <x:v>fight_overlap_shared_heroes</x:v>
       </x:c>
       <x:c r="B59" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D59" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E59" s="5" t="str">
-        <x:v>10分钟后靠近肉山坑可触发肉山上下文</x:v>
+        <x:v>重叠fight record合并的共享英雄数</x:v>
       </x:c>
       <x:c r="F59" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2695,22 +2741,22 @@
     </x:row>
     <x:row r="60" ht="33" customHeight="1">
       <x:c r="A60" s="5" t="str">
-        <x:v>roshan_damage_context_pad</x:v>
+        <x:v>pickoff_enemy_damage_ratio</x:v>
       </x:c>
       <x:c r="B60" s="5" t="str">
-        <x:v>30</x:v>
+        <x:v>0.80</x:v>
       </x:c>
       <x:c r="C60" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D60" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E60" s="5" t="str">
-        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
+        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
       </x:c>
       <x:c r="F60" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G60" s="5" t="str">
         <x:v>是</x:v>
@@ -2719,22 +2765,22 @@
     </x:row>
     <x:row r="61" ht="33" customHeight="1">
       <x:c r="A61" s="5" t="str">
-        <x:v>roshan_kill_context_before</x:v>
+        <x:v>pickoff_ally_near_limit</x:v>
       </x:c>
       <x:c r="B61" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D61" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E61" s="5" t="str">
-        <x:v>肉山击杀与战斗关联前置时间</x:v>
+        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
       </x:c>
       <x:c r="F61" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G61" s="5" t="str">
         <x:v>是</x:v>
@@ -2743,22 +2789,22 @@
     </x:row>
     <x:row r="62" ht="33" customHeight="1">
       <x:c r="A62" s="5" t="str">
-        <x:v>roshan_kill_context_after</x:v>
+        <x:v>escape_pickoff_window</x:v>
       </x:c>
       <x:c r="B62" s="5" t="str">
-        <x:v>75</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C62" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D62" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E62" s="5" t="str">
-        <x:v>肉山击杀与战斗关联后置时间</x:v>
+        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
       </x:c>
       <x:c r="F62" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G62" s="5" t="str">
         <x:v>是</x:v>
@@ -2767,22 +2813,22 @@
     </x:row>
     <x:row r="63" ht="33" customHeight="1">
       <x:c r="A63" s="5" t="str">
-        <x:v>roshan_respawn_suppression</x:v>
+        <x:v>escape_pickoff_damage_min</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
-        <x:v>480</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C63" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D63" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E63" s="5" t="str">
-        <x:v>肉山死亡后该时间内不视为存活</x:v>
+        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G63" s="5" t="str">
         <x:v>是</x:v>
@@ -2791,19 +2837,19 @@
     </x:row>
     <x:row r="64" ht="33" customHeight="1">
       <x:c r="A64" s="5" t="str">
-        <x:v>roshan_attempt_group_gap</x:v>
+        <x:v>roshan_context_radius</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="C64" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D64" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E64" s="5" t="str">
-        <x:v>Roshan伤害组分组间隔</x:v>
+        <x:v>肉山团上下文范围</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2815,19 +2861,19 @@
     </x:row>
     <x:row r="65" ht="33" customHeight="1">
       <x:c r="A65" s="5" t="str">
-        <x:v>roshan_attempt_damage_min</x:v>
+        <x:v>roshan_context_min_time</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C65" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D65" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E65" s="5" t="str">
-        <x:v>未击杀Roshan尝试最低伤害</x:v>
+        <x:v>10分钟后靠近肉山坑可触发肉山上下文</x:v>
       </x:c>
       <x:c r="F65" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2839,19 +2885,19 @@
     </x:row>
     <x:row r="66" ht="33" customHeight="1">
       <x:c r="A66" s="5" t="str">
-        <x:v>roshan_attempt_kill_grace</x:v>
+        <x:v>roshan_damage_context_pad</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C66" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D66" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E66" s="5" t="str">
-        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
+        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2863,22 +2909,22 @@
     </x:row>
     <x:row r="67" ht="33" customHeight="1">
       <x:c r="A67" s="5" t="str">
-        <x:v>roshan_drop_merge_window</x:v>
+        <x:v>roshan_kill_context_before</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
-        <x:v>20</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C67" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D67" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E67" s="5" t="str">
-        <x:v>肉山击杀后掉落合并窗口</x:v>
+        <x:v>肉山击杀与战斗关联前置时间</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G67" s="5" t="str">
         <x:v>是</x:v>
@@ -2887,22 +2933,22 @@
     </x:row>
     <x:row r="68" ht="33" customHeight="1">
       <x:c r="A68" s="5" t="str">
-        <x:v>roshan_owner_drop_fallback</x:v>
+        <x:v>roshan_kill_context_after</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C68" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D68" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E68" s="5" t="str">
-        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
+        <x:v>肉山击杀与战斗关联后置时间</x:v>
       </x:c>
       <x:c r="F68" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G68" s="5" t="str">
         <x:v>是</x:v>
@@ -2911,19 +2957,19 @@
     </x:row>
     <x:row r="69" ht="33" customHeight="1">
       <x:c r="A69" s="5" t="str">
-        <x:v>tormentor_alive_start</x:v>
+        <x:v>roshan_respawn_suppression</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
-        <x:v>1200</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="C69" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D69" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E69" s="5" t="str">
-        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
+        <x:v>肉山死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2935,19 +2981,19 @@
     </x:row>
     <x:row r="70" ht="33" customHeight="1">
       <x:c r="A70" s="5" t="str">
-        <x:v>tormentor_respawn_suppression</x:v>
+        <x:v>roshan_attempt_group_gap</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C70" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D70" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E70" s="5" t="str">
-        <x:v>魔晶死亡后该时间内不视为存活</x:v>
+        <x:v>Roshan伤害组分组间隔</x:v>
       </x:c>
       <x:c r="F70" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2959,19 +3005,19 @@
     </x:row>
     <x:row r="71" ht="33" customHeight="1">
       <x:c r="A71" s="5" t="str">
-        <x:v>tormentor_near_radius</x:v>
+        <x:v>roshan_attempt_damage_min</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="C71" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D71" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E71" s="5" t="str">
-        <x:v>独立魔晶击杀附近英雄判断</x:v>
+        <x:v>未击杀Roshan尝试最低伤害</x:v>
       </x:c>
       <x:c r="F71" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2983,19 +3029,19 @@
     </x:row>
     <x:row r="72" ht="33" customHeight="1">
       <x:c r="A72" s="5" t="str">
-        <x:v>highground_raw_corner</x:v>
+        <x:v>roshan_attempt_kill_grace</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
-        <x:v>95/158</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C72" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D72" s="5" t="str">
-        <x:v>高地团</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E72" s="5" t="str">
-        <x:v>高地团中心区域阈值</x:v>
+        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
       </x:c>
       <x:c r="F72" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3007,22 +3053,22 @@
     </x:row>
     <x:row r="73" ht="33" customHeight="1">
       <x:c r="A73" s="5" t="str">
-        <x:v>tower_context_radius</x:v>
+        <x:v>roshan_drop_merge_window</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C73" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D73" s="5" t="str">
-        <x:v>守塔团</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E73" s="5" t="str">
-        <x:v>防御塔上下文范围</x:v>
+        <x:v>肉山击杀后掉落合并窗口</x:v>
       </x:c>
       <x:c r="F73" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G73" s="5" t="str">
         <x:v>是</x:v>
@@ -3031,7 +3077,7 @@
     </x:row>
     <x:row r="74" ht="33" customHeight="1">
       <x:c r="A74" s="5" t="str">
-        <x:v>tower_context_time_pad</x:v>
+        <x:v>roshan_owner_drop_fallback</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
         <x:v>5</x:v>
@@ -3040,13 +3086,13 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D74" s="5" t="str">
-        <x:v>守塔团</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E74" s="5" t="str">
-        <x:v>战斗窗口前后塔状态检测</x:v>
+        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
       </x:c>
       <x:c r="F74" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G74" s="5" t="str">
         <x:v>是</x:v>
@@ -3055,22 +3101,22 @@
     </x:row>
     <x:row r="75" ht="33" customHeight="1">
       <x:c r="A75" s="5" t="str">
-        <x:v>aegis_valid_duration</x:v>
+        <x:v>tormentor_alive_start</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
-        <x:v>300</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="C75" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D75" s="5" t="str">
-        <x:v>带盾阵亡</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E75" s="5" t="str">
-        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
+        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G75" s="5" t="str">
         <x:v>是</x:v>
@@ -3079,22 +3125,22 @@
     </x:row>
     <x:row r="76" ht="33" customHeight="1">
       <x:c r="A76" s="5" t="str">
-        <x:v>v1_7_subordinate_overlap_ratio</x:v>
+        <x:v>tormentor_respawn_suppression</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
-        <x:v>0.60</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C76" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D76" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E76" s="5" t="str">
-        <x:v>旧单点候选与父窗口重叠比例</x:v>
+        <x:v>魔晶死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F76" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G76" s="5" t="str">
         <x:v>是</x:v>
@@ -3103,22 +3149,22 @@
     </x:row>
     <x:row r="77" ht="33" customHeight="1">
       <x:c r="A77" s="5" t="str">
-        <x:v>v1_7_parent_start_grace</x:v>
+        <x:v>tormentor_near_radius</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C77" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D77" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E77" s="5" t="str">
-        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
+        <x:v>独立魔晶击杀附近英雄判断</x:v>
       </x:c>
       <x:c r="F77" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G77" s="5" t="str">
         <x:v>是</x:v>
@@ -3127,22 +3173,22 @@
     </x:row>
     <x:row r="78" ht="33" customHeight="1">
       <x:c r="A78" s="5" t="str">
-        <x:v>v1_7_parent_end_grace</x:v>
+        <x:v>highground_raw_corner</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>95/158</x:v>
       </x:c>
       <x:c r="C78" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D78" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>高地团</x:v>
       </x:c>
       <x:c r="E78" s="5" t="str">
-        <x:v>父窗口允许比候选结束最多早5秒</x:v>
+        <x:v>高地团中心区域阈值</x:v>
       </x:c>
       <x:c r="F78" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G78" s="5" t="str">
         <x:v>是</x:v>
@@ -3151,22 +3197,22 @@
     </x:row>
     <x:row r="79" ht="33" customHeight="1">
       <x:c r="A79" s="5" t="str">
-        <x:v>v1_8_duplicate_no_kill_gap</x:v>
+        <x:v>tower_context_radius</x:v>
       </x:c>
       <x:c r="B79" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C79" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D79" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>守塔团</x:v>
       </x:c>
       <x:c r="E79" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
+        <x:v>防御塔上下文范围</x:v>
       </x:c>
       <x:c r="F79" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G79" s="5" t="str">
         <x:v>是</x:v>
@@ -3175,22 +3221,22 @@
     </x:row>
     <x:row r="80" ht="33" customHeight="1">
       <x:c r="A80" s="5" t="str">
-        <x:v>v1_8_duplicate_distance</x:v>
+        <x:v>tower_context_time_pad</x:v>
       </x:c>
       <x:c r="B80" s="5" t="str">
-        <x:v>1800</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C80" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D80" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>守塔团</x:v>
       </x:c>
       <x:c r="E80" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
+        <x:v>战斗窗口前后塔状态检测</x:v>
       </x:c>
       <x:c r="F80" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G80" s="5" t="str">
         <x:v>是</x:v>
@@ -3199,22 +3245,22 @@
     </x:row>
     <x:row r="81" ht="33" customHeight="1">
       <x:c r="A81" s="5" t="str">
-        <x:v>v1_8_duplicate_jaccard</x:v>
+        <x:v>aegis_valid_duration</x:v>
       </x:c>
       <x:c r="B81" s="5" t="str">
-        <x:v>0.50</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C81" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D81" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>带盾阵亡</x:v>
       </x:c>
       <x:c r="E81" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
+        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
       </x:c>
       <x:c r="F81" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G81" s="5" t="str">
         <x:v>是</x:v>
@@ -3223,22 +3269,22 @@
     </x:row>
     <x:row r="82" ht="33" customHeight="1">
       <x:c r="A82" s="5" t="str">
-        <x:v>v1_8_duplicate_shared_heroes</x:v>
+        <x:v>v1_7_subordinate_overlap_ratio</x:v>
       </x:c>
       <x:c r="B82" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>0.60</x:v>
       </x:c>
       <x:c r="C82" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D82" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E82" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
+        <x:v>旧单点候选与父窗口重叠比例</x:v>
       </x:c>
       <x:c r="F82" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="G82" s="5" t="str">
         <x:v>是</x:v>
@@ -3247,22 +3293,22 @@
     </x:row>
     <x:row r="83" ht="33" customHeight="1">
       <x:c r="A83" s="5" t="str">
-        <x:v>v1_9_kill_parent_gap</x:v>
+        <x:v>v1_7_parent_start_grace</x:v>
       </x:c>
       <x:c r="B83" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C83" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D83" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E83" s="5" t="str">
-        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
+        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
       </x:c>
       <x:c r="F83" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="G83" s="5" t="str">
         <x:v>是</x:v>
@@ -3271,22 +3317,22 @@
     </x:row>
     <x:row r="84" ht="33" customHeight="1">
       <x:c r="A84" s="5" t="str">
-        <x:v>v1_9_kill_parent_distance</x:v>
+        <x:v>v1_7_parent_end_grace</x:v>
       </x:c>
       <x:c r="B84" s="5" t="str">
-        <x:v>2500</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C84" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D84" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
       </x:c>
       <x:c r="E84" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
+        <x:v>父窗口允许比候选结束最多早5秒</x:v>
       </x:c>
       <x:c r="F84" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.7</x:v>
       </x:c>
       <x:c r="G84" s="5" t="str">
         <x:v>是</x:v>
@@ -3295,22 +3341,22 @@
     </x:row>
     <x:row r="85" ht="33" customHeight="1">
       <x:c r="A85" s="5" t="str">
-        <x:v>v1_9_kill_parent_jaccard</x:v>
+        <x:v>v1_8_duplicate_no_kill_gap</x:v>
       </x:c>
       <x:c r="B85" s="5" t="str">
-        <x:v>0.33</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C85" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D85" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E85" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
+        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
       </x:c>
       <x:c r="F85" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G85" s="5" t="str">
         <x:v>是</x:v>
@@ -3319,22 +3365,22 @@
     </x:row>
     <x:row r="86" ht="33" customHeight="1">
       <x:c r="A86" s="5" t="str">
-        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+        <x:v>v1_8_duplicate_distance</x:v>
       </x:c>
       <x:c r="B86" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="C86" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D86" s="5" t="str">
         <x:v>战斗类标签</x:v>
       </x:c>
       <x:c r="E86" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
       </x:c>
       <x:c r="F86" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.8</x:v>
       </x:c>
       <x:c r="G86" s="5" t="str">
         <x:v>是</x:v>
@@ -3343,27 +3389,171 @@
     </x:row>
     <x:row r="87" ht="33" customHeight="1">
       <x:c r="A87" s="5" t="str">
+        <x:v>v1_8_duplicate_jaccard</x:v>
+      </x:c>
+      <x:c r="B87" s="5" t="str">
+        <x:v>0.50</x:v>
+      </x:c>
+      <x:c r="C87" s="5" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="D87" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E87" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
+      </x:c>
+      <x:c r="F87" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G87" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H87" s="5" t="str"/>
+    </x:row>
+    <x:row r="88" ht="33" customHeight="1">
+      <x:c r="A88" s="5" t="str">
+        <x:v>v1_8_duplicate_shared_heroes</x:v>
+      </x:c>
+      <x:c r="B88" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C88" s="5" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="D88" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E88" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
+      </x:c>
+      <x:c r="F88" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G88" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H88" s="5" t="str"/>
+    </x:row>
+    <x:row r="89" ht="33" customHeight="1">
+      <x:c r="A89" s="5" t="str">
+        <x:v>v1_9_kill_parent_gap</x:v>
+      </x:c>
+      <x:c r="B89" s="5" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C89" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D89" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E89" s="5" t="str">
+        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
+      </x:c>
+      <x:c r="F89" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G89" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H89" s="5" t="str"/>
+    </x:row>
+    <x:row r="90" ht="33" customHeight="1">
+      <x:c r="A90" s="5" t="str">
+        <x:v>v1_9_kill_parent_distance</x:v>
+      </x:c>
+      <x:c r="B90" s="5" t="str">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="C90" s="5" t="str">
+        <x:v>码</x:v>
+      </x:c>
+      <x:c r="D90" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E90" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
+      </x:c>
+      <x:c r="F90" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G90" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H90" s="5" t="str"/>
+    </x:row>
+    <x:row r="91" ht="33" customHeight="1">
+      <x:c r="A91" s="5" t="str">
+        <x:v>v1_9_kill_parent_jaccard</x:v>
+      </x:c>
+      <x:c r="B91" s="5" t="str">
+        <x:v>0.33</x:v>
+      </x:c>
+      <x:c r="C91" s="5" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="D91" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E91" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
+      </x:c>
+      <x:c r="F91" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G91" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H91" s="5" t="str"/>
+    </x:row>
+    <x:row r="92" ht="33" customHeight="1">
+      <x:c r="A92" s="5" t="str">
+        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+      </x:c>
+      <x:c r="B92" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C92" s="5" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="D92" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E92" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+      </x:c>
+      <x:c r="F92" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G92" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H92" s="5" t="str"/>
+    </x:row>
+    <x:row r="93" ht="33" customHeight="1">
+      <x:c r="A93" s="5" t="str">
         <x:v>adjacent_combat_qc_scan_window</x:v>
       </x:c>
-      <x:c r="B87" s="5" t="str">
+      <x:c r="B93" s="5" t="str">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="C87" s="5" t="str">
+      <x:c r="C93" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
-      <x:c r="D87" s="5" t="str">
+      <x:c r="D93" s="5" t="str">
         <x:v>质量控制</x:v>
       </x:c>
-      <x:c r="E87" s="5" t="str">
+      <x:c r="E93" s="5" t="str">
         <x:v>生成后复查相邻战斗事件的建议扫描窗口</x:v>
       </x:c>
-      <x:c r="F87" s="5" t="str">
+      <x:c r="F93" s="5" t="str">
         <x:v>v1.9</x:v>
       </x:c>
-      <x:c r="G87" s="5" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="H87" s="5" t="str"/>
+      <x:c r="G93" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H93" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3482,16 +3672,16 @@
         <x:v>time, log_index, unit, team, ehandle, x, y, hp, max_hp, lifeState</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>线上小兵状态/轨迹</x:v>
+        <x:v>线上小兵/中立野怪状态与轨迹</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>对线区; 勾兵; 断线</x:v>
+        <x:v>对线区; 勾兵; 断线; 拉野</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
-        <x:v>按ehandle追踪小兵路线；判断死亡小兵500范围内是否有敌方线上小兵</x:v>
+        <x:v>按ehandle追踪小兵路线；判断死亡小兵500范围内是否有敌方线上小兵；拉野在combat锚点附近用线兵-野怪状态贴近补证据，无ehandle时用synthetic状态点兜底</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>默认只需抽取-5到650秒</x:v>
+        <x:v>默认只需抽取-5到900秒</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="45" customHeight="1">
@@ -3880,7 +4070,7 @@
         <x:v>fight_records</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>先判断GANK：一方参与英雄&gt;=2且另一方参与英雄&lt;=1；否则按参与人数、直接参与人数、伤害、死亡、持续时间输出小规模冲突或团战</x:v>
+        <x:v>先按发起时刻位置判断GANK：同一目标短窗口被同一方至少2人命中，读取t0±1秒位置，若进攻方附近&gt;=2且被抓方附近=1则输出GANK；否则按参与人数、直接参与人数、伤害、死亡、持续时间输出小规模冲突或团战</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
         <x:v>战斗类事件</x:v>
@@ -3889,7 +4079,7 @@
         <x:v>边界事件仍需人工复核</x:v>
       </x:c>
       <x:c r="G9" s="5" t="str">
-        <x:v>旧抓人候选不再作为最终标签，新增GANK承接N抓1语义</x:v>
+        <x:v>旧抓人候选不再作为最终标签，新增GANK承接发起阶段N抓1语义</x:v>
       </x:c>
       <x:c r="H9" s="5" t="str"/>
     </x:row>
@@ -4280,7 +4470,7 @@
         <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>符合N抓1则GANK；与已有团战窗口重叠则团战；与已有小规模冲突重叠则小规模冲突；否则总人数&gt;=8且双方&gt;=3为团战，其余为小规模冲突</x:v>
+        <x:v>符合发起阶段位置N抓1则GANK；与已有团战窗口重叠则团战；与已有小规模冲突重叠则小规模冲突；否则总人数&gt;=8且双方&gt;=3为团战，其余为小规模冲突</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
         <x:v>输出新标签，不输出抓人</x:v>

</xml_diff>

<commit_message>
Expand tactical event detection rules
</commit_message>
<xml_diff>
--- a/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
+++ b/outputs/dota2_tactical_event_recognition_algorithms_v1.9_20260609.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="Red11db88412e4bdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R17c3d3d7c9eb4569"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="R8716cca7ae95486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="R1a52a61d27574702"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="Rd082e5af087a4b67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="Ra1500f4977ed46d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="R88c458310b3340b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="Rdfb71f42f7814019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本说明" sheetId="1" r:id="R5e06e133eb70422b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="标签算法" sheetId="2" r:id="R3c03f4288c494485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数阈值" sheetId="3" r:id="R89ab81d638f1481f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据源字段" sheetId="4" r:id="Rfa8dae8cc7a4435f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="处理流程" sheetId="5" r:id="R650a148913e943a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合并去重" sheetId="6" r:id="R4c4f4eda2c204f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="输出格式" sheetId="7" r:id="Ra0a4dd3d058f4019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="人工修改入口" sheetId="8" r:id="R53a110c925554085"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,10 +366,10 @@
         <x:v>输出标签数</x:v>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>对线分路、勾兵、断线、拉野、囤野/堆野、控符、蹲人、开雾、GANK、小规模冲突、团战、肉山团、肉山击杀、高地团、塔下、肉山尝试、魔晶团、资源获得、带盾阵亡</x:v>
+        <x:v>对线分路、出门抢远程兵、出门抢近战兵、勾兵、断线、拉野、囤野/堆野、控符、蹲人、开雾、GANK、小规模冲突、团战、肉山团、肉山击杀、高地团、塔下、肉山尝试、魔晶团、资源获得、带盾阵亡</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str"/>
     </x:row>
@@ -546,91 +546,91 @@
     </x:row>
     <x:row r="3" ht="58.5" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>出门抢远程兵</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>candidate_review</x:v>
+        <x:v>auto</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>B</x:v>
+        <x:v>A/B</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
+        <x:v>combat_logs; dota_model_neutral_siege_creep</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内存在敌方线上小兵；若敌方英雄获得该小兵死亡经验，则输出勾兵</x:v>
+        <x:v>0-31秒内上路/下路远程兵死亡；判断该兵来源路线、补刀/金钱获得者、经验分享者；中路不识别</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
-        <x:v>通常00:00-10:00</x:v>
+        <x:v>00:00-00:31</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
-        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；连续小兵死亡默认10秒窗口合并</x:v>
+        <x:v>死亡日志前后1秒相邻日志块；排除开局发钱gold_reason=17和负数金钱；路线优先ehandle早期轨迹，缺失用死亡点坐标；source_lane=mid直接跳过</x:v>
       </x:c>
       <x:c r="H3" s="5" t="str">
-        <x:v>获得经验的敌方英雄；多人获得经验则全部列入；结果中附获得经验英雄0-5分钟主对线路</x:v>
+        <x:v>heroes输出金钱获得者、经验获得者、击杀来源英雄</x:v>
       </x:c>
       <x:c r="I3" s="5" t="str">
-        <x:v>结果=获得经验英雄获得被勾兵阵营某来源路线小兵死亡经验；可附死亡小兵数量、附近敌方小兵证据和source_lane_method</x:v>
+        <x:v>结果=某方某路远程兵死亡；补到/获得金钱英雄；金钱分配；经验分配</x:v>
       </x:c>
       <x:c r="J3" s="5" t="str">
-        <x:v>单个小兵死亡作为证据；按获得经验阵营+被勾兵阵营+source_lane聚合，连续窗口合并输出；塔下吃兵不输出</x:v>
+        <x:v>每个死亡远程兵一行，不聚合</x:v>
       </x:c>
       <x:c r="K3" s="5" t="str">
-        <x:v>与断线互斥：附近无敌方小兵为断线证据，附近有敌方小兵且敌方英雄获经验则输出勾兵</x:v>
+        <x:v>早期边路资源争夺事实类；低于战斗类</x:v>
       </x:c>
       <x:c r="L3" s="5" t="str">
-        <x:v>需要lane_zone、活体线上小兵位置、经验获得明细和source_lane；缺失个体轨迹时必须在evidence标记xy_fallback</x:v>
+        <x:v>如果金钱日志缺失，用死亡击杀来源兜底；需人工核查反补/召唤物击杀边界</x:v>
       </x:c>
       <x:c r="M3" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="N3" s="5" t="str"/>
     </x:row>
     <x:row r="4" ht="58.5" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>出门抢近战兵</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>candidate_review</x:v>
+        <x:v>auto</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
-        <x:v>B</x:v>
+        <x:v>A/B</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
-        <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
+        <x:v>combat_logs; dota_model_neutral_siege_creep</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>10分钟前某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内无敌方线上小兵；击杀来源可映射为敌方英雄</x:v>
+        <x:v>0-31秒内上路/下路近战兵死亡；判断该兵来源路线、补刀/金钱获得者、经验分享者；中路不识别</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
-        <x:v>通常00:00-10:00</x:v>
+        <x:v>00:00-00:31</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str">
-        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；同一英雄同一source_lane 10秒内连续触发&gt;=2或&gt;=3个小兵死亡后输出</x:v>
+        <x:v>死亡日志前后1秒相邻日志块；排除开局发钱gold_reason=17和负数金钱；路线优先ehandle早期轨迹，缺失用死亡点坐标；source_lane=mid直接跳过</x:v>
       </x:c>
       <x:c r="H4" s="5" t="str">
-        <x:v>执行断兵的敌方英雄；结果中附执行英雄0-5分钟主对线路</x:v>
+        <x:v>heroes输出金钱获得者、经验获得者、击杀来源英雄</x:v>
       </x:c>
       <x:c r="I4" s="5" t="str">
-        <x:v>结果=断兵英雄主对线路、被断兵阵营、小兵来源路线、小兵数量、一塔存活证据；例：中路英雄在下路断下路兵</x:v>
+        <x:v>结果=某方某路近战兵死亡；补到/获得金钱英雄；金钱分配；经验分配</x:v>
       </x:c>
       <x:c r="J4" s="5" t="str">
-        <x:v>单个小兵死亡只作为证据；按击杀英雄+被断兵阵营+source_lane聚合，连续10秒窗口达到阈值才输出事件；塔下吃兵不输出</x:v>
+        <x:v>每个死亡近战兵一行，不聚合</x:v>
       </x:c>
       <x:c r="K4" s="5" t="str">
-        <x:v>与拉野、正常兵线交汇清线互斥；一塔已掉后不判断线</x:v>
+        <x:v>早期边路资源争夺事实类；低于战斗类</x:v>
       </x:c>
       <x:c r="L4" s="5" t="str">
-        <x:v>需要lane_zone、活体线上小兵位置和source_lane；若缺少个体轨迹，必须在evidence标记xy_fallback</x:v>
+        <x:v>如果金钱日志缺失，用死亡击杀来源兜底；需人工核查反补/召唤物击杀边界</x:v>
       </x:c>
       <x:c r="M4" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="N4" s="5" t="str"/>
     </x:row>
     <x:row r="5" ht="58.5" customHeight="1">
       <x:c r="A5" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -639,31 +639,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>combat_logs; dota_model_neutral_siege_creep; player_intervals2</x:v>
+        <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>15分钟前线上小兵与中立单位发生直接伤害/死亡交互；combat直接交互作为锚点，若连续伤害缺失，则用锚点前45秒到后5秒内线兵-同名野怪距离&lt;=550码的状态贴近补证据；若没有combat锚点，则全局扫描状态表中的550码内连续贴近与双方掉血片段；中路排除；路线优先用线兵ehandle全段主路线</x:v>
+        <x:v>某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内存在敌方线上小兵；若敌方英雄获得该小兵死亡经验，则输出勾兵</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>00:00-15:00</x:v>
+        <x:v>通常00:00-10:00</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
-        <x:v>拉野组间隔35秒；位置距离28 raw；状态贴近距离550码（约4.23 raw）；执行者交互窗口为拉野开始前30秒到后10秒；位置兜底800码；附近英雄1500码</x:v>
+        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；连续小兵死亡默认10秒窗口合并</x:v>
       </x:c>
       <x:c r="H5" s="5" t="str">
-        <x:v>heroes输出推断出的拉野执行者；优先取同阵营英雄/召唤物与该组野怪的交互者，找不到再取800码内最近同阵营英雄；附近双方英雄只写结果/evidence</x:v>
+        <x:v>获得经验的敌方英雄；多人获得经验则全部列入；结果中附获得经验英雄0-5分钟主对线路</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
-        <x:v>结果=某方某路小兵与中立单位连续交战，并保留附近英雄环境证据；evidence写pull_executor method=neutral_interaction或position_nearest；无ehandle时evidence写synthetic状态点</x:v>
+        <x:v>结果=获得经验英雄获得被勾兵阵营某来源路线小兵死亡经验；可附死亡小兵数量、附近敌方小兵证据和source_lane_method</x:v>
       </x:c>
       <x:c r="J5" s="5" t="str">
-        <x:v>死亡&lt;2且交互&lt;3则过滤；无combat锚点的状态片段需连续秒数和线兵/野怪掉血门槛</x:v>
+        <x:v>单个小兵死亡作为证据；按获得经验阵营+被勾兵阵营+source_lane聚合，连续窗口合并输出；塔下吃兵不输出</x:v>
       </x:c>
       <x:c r="K5" s="5" t="str">
-        <x:v>与断线、普通野区交互需复核</x:v>
+        <x:v>与断线互斥：附近无敌方小兵为断线证据，附近有敌方小兵且敌方英雄获经验则输出勾兵</x:v>
       </x:c>
       <x:c r="L5" s="5" t="str">
-        <x:v>英雄拉仇恨起点仍需人工核查；召唤物交互按sourcename/targetsourcename归属英雄</x:v>
+        <x:v>需要lane_zone、活体线上小兵位置、经验获得明细和source_lane；缺失个体轨迹时必须在evidence标记xy_fallback</x:v>
       </x:c>
       <x:c r="M5" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -672,7 +672,7 @@
     </x:row>
     <x:row r="6" ht="58.5" customHeight="1">
       <x:c r="A6" s="5" t="str">
-        <x:v>囤野/堆野</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -681,73 +681,73 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>player_intervals2</x:v>
+        <x:v>combat_logs; tower_status_update; dota_model_neutral_siege_creep; derived: lane_zone</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
-        <x:v>camps_stacked 或 creeps_stacked 计数较上一快照增加</x:v>
+        <x:v>10分钟前某阵营某一路线上小兵死亡；路线按小兵来源路source_lane判定，优先用ehandle出生/早期轨迹验证，缺失时用死亡坐标兜底；该阵营该路线一塔仍存活；死亡位置在该路线lane_zone外且不在双方一塔保护区内；死亡小兵500范围内无敌方线上小兵；击杀来源可映射为敌方英雄</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>计数增加时刻±5秒</x:v>
+        <x:v>通常00:00-10:00</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
-        <x:v>计数增量&gt;0</x:v>
+        <x:v>lane_zone外；一塔保护区12 raw内跳过；附近敌方小兵半径500码；同一英雄同一source_lane 10秒内连续触发&gt;=2或&gt;=3个小兵死亡后输出</x:v>
       </x:c>
       <x:c r="H6" s="5" t="str">
-        <x:v>执行英雄及阵营</x:v>
+        <x:v>执行断兵的敌方英雄；结果中附执行英雄0-5分钟主对线路</x:v>
       </x:c>
       <x:c r="I6" s="5" t="str">
-        <x:v>结果默认留空或写 camps/creeps 增量</x:v>
+        <x:v>结果=断兵英雄主对线路、被断兵阵营、小兵来源路线、小兵数量、一塔存活证据；例：中路英雄在下路断下路兵</x:v>
       </x:c>
       <x:c r="J6" s="5" t="str">
-        <x:v>同一快照只输出一次</x:v>
+        <x:v>单个小兵死亡只作为证据；按击杀英雄+被断兵阵营+source_lane聚合，连续10秒窗口达到阈值才输出事件；塔下吃兵不输出</x:v>
       </x:c>
       <x:c r="K6" s="5" t="str">
-        <x:v>事实较可靠但成功语义需核查</x:v>
+        <x:v>与拉野、正常兵线交汇清线互斥；一塔已掉后不判断线</x:v>
       </x:c>
       <x:c r="L6" s="5" t="str">
-        <x:v>数据库计数可定位堆野，但不能解释完整动作过程</x:v>
+        <x:v>需要lane_zone、活体线上小兵位置和source_lane；若缺少个体轨迹，必须在evidence标记xy_fallback</x:v>
       </x:c>
       <x:c r="M6" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N6" s="5" t="str"/>
     </x:row>
     <x:row r="7" ht="58.5" customHeight="1">
       <x:c r="A7" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>auto</x:v>
+        <x:v>candidate_review</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
-        <x:v>A/B</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>match_chat_events; player_intervals2</x:v>
+        <x:v>combat_logs; dota_model_neutral_siege_creep; player_intervals2</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
-        <x:v>RUNE_PICKUP/RUNE_BOTTLE/RUNE_DENY；智慧/赏金/水符/护盾/能量符统一为控符；能量符未刷新侧若有英雄也记录控符；value=5赏金神符单独走四赏金符点逻辑：上河道、下河道、天辉赏金server=(590,-4637)/raw≈(133.6,90.4)、夜魇赏金server=(-1000,4443)/raw≈(120.0,166.8)；value=8智慧符单独走两智慧符点逻辑：天辉智慧raw≈(66.0,134.0)/server≈(-7468,610)、夜魇智慧raw≈(191.0,118.0)/server≈(7537,-1285)</x:v>
+        <x:v>15分钟前线上小兵与中立单位发生直接伤害/死亡交互；combat直接交互作为锚点，若连续伤害缺失，则用锚点前45秒到后5秒内线兵-同名野怪距离&lt;=550码的状态贴近补证据；若没有combat锚点，则全局扫描状态表中的550码内连续贴近与双方掉血片段；中路排除；路线优先用线兵ehandle全段主路线；先确认野怪被拉动并勾走线兵仇恨，最后线兵与野怪连续交战/贴近停滞</x:v>
       </x:c>
       <x:c r="F7" s="5" t="str">
-        <x:v>结果事件t-5到t；智慧符t-10到t；未刷新侧spawn_time-5到spawn_time</x:v>
+        <x:v>00:00-15:00</x:v>
       </x:c>
       <x:c r="G7" s="5" t="str">
-        <x:v>符点附近1000码；能量符刷新间隔120秒；罐装后90秒内同英雄同神符拾取去重</x:v>
+        <x:v>拉野组间隔35秒；位置距离28 raw；状态贴近距离550码（约4.23 raw）；执行者仇恨交互窗口为拉野开始前12秒到后10秒；同一波8秒内多候选只保留最早仇恨触发者；附近英雄1500码</x:v>
       </x:c>
       <x:c r="H7" s="5" t="str">
-        <x:v>heroes=某符点附近两方英雄；赏金符按四个赏金点附近英雄记录；智慧符按两个智慧符点附近英雄记录</x:v>
+        <x:v>heroes输出推断出的拉野执行者；先判定拉野链条成立，再从野怪移动最早阶段反推谁触发该组野怪仇恨；当前实现以英雄主动打到该组野怪或该组野怪最早打到英雄的第一条日志为强证据，不再用位置兜底归因；附近双方英雄只写结果/evidence</x:v>
       </x:c>
       <x:c r="I7" s="5" t="str">
-        <x:v>结果=英雄名+拾取/罐装/反补+上河道/下河道/天辉赏金符点/夜魇赏金符点/天辉智慧符点/夜魇智慧符点+神符；未刷新侧=神符刷新在另一侧；无结果可留空</x:v>
+        <x:v>结果=某方某路小兵与中立单位连续交战，并保留附近英雄环境证据；evidence写pull_executor method=neutral_interaction；无ehandle时evidence写synthetic状态点</x:v>
       </x:c>
       <x:c r="J7" s="5" t="str">
-        <x:v>每颗神符只记录一次；value=5按四赏金符点区分；value=8按两智慧符点区分；罐装优先于后续拾取</x:v>
+        <x:v>死亡&lt;2且交互&lt;3则过滤；无combat锚点的状态片段需连续秒数和线兵/野怪掉血门槛；无英雄-野怪仇恨交互证据不输出执行者</x:v>
       </x:c>
       <x:c r="K7" s="5" t="str">
-        <x:v>控符统一标签，不再输出帮控符/控智慧神符</x:v>
+        <x:v>与断线、普通野区交互需复核</x:v>
       </x:c>
       <x:c r="L7" s="5" t="str">
-        <x:v>符点归属和附近英雄可人工复核</x:v>
+        <x:v>后续需补全英雄走近但无伤害的移动归因；召唤物交互按sourcename/targetsourcename归属英雄</x:v>
       </x:c>
       <x:c r="M7" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -756,7 +756,7 @@
     </x:row>
     <x:row r="8" ht="58.5" customHeight="1">
       <x:c r="A8" s="5" t="str">
-        <x:v>蹲人</x:v>
+        <x:v>囤野/堆野</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -765,31 +765,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:v>英雄位置; 视野/路径上下文</x:v>
+        <x:v>player_intervals2</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>英雄在潜在目标500-1000码范围长期隐藏/等待，通常在树林、阴影、视野盲区</x:v>
+        <x:v>camps_stacked 或 creeps_stacked 计数较上一快照增加</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
-        <x:v>等待开始-接触或离开</x:v>
+        <x:v>计数增加时刻±5秒</x:v>
       </x:c>
       <x:c r="G8" s="5" t="str">
-        <x:v>建议500-1000码；等待时长需人工设定</x:v>
+        <x:v>计数增量&gt;0</x:v>
       </x:c>
       <x:c r="H8" s="5" t="str">
-        <x:v>蹲守方与被蹲目标</x:v>
+        <x:v>执行英雄及阵营</x:v>
       </x:c>
       <x:c r="I8" s="5" t="str">
-        <x:v>结果可留空或写蹲守结果</x:v>
+        <x:v>结果默认留空或写 camps/creeps 增量</x:v>
       </x:c>
       <x:c r="J8" s="5" t="str">
-        <x:v>当前建议人工核查，不强制自动输出</x:v>
+        <x:v>同一快照只输出一次</x:v>
       </x:c>
       <x:c r="K8" s="5" t="str">
-        <x:v>若后续造成战斗，优先战斗类标签</x:v>
+        <x:v>事实较可靠但成功语义需核查</x:v>
       </x:c>
       <x:c r="L8" s="5" t="str">
-        <x:v>语义强依赖录像和视野</x:v>
+        <x:v>数据库计数可定位堆野，但不能解释完整动作过程</x:v>
       </x:c>
       <x:c r="M8" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -798,49 +798,49 @@
     </x:row>
     <x:row r="9" ht="58.5" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>candidate_review</x:v>
+        <x:v>auto</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>B</x:v>
+        <x:v>A/B</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
-        <x:v>combat_logs</x:v>
+        <x:v>match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>item_smoke_of_deceit 使用；结合 smoke modifier 添加/移除确定进入雾英雄和结束时间</x:v>
+        <x:v>RUNE_PICKUP/RUNE_BOTTLE/RUNE_DENY；智慧/赏金/水符/护盾/能量符统一为控符；能量符未刷新侧若有英雄也记录控符；value=5赏金神符单独走四赏金符点逻辑：上河道、下河道、天辉赏金server=(590,-4637)/raw≈(133.6,90.4)、夜魇赏金server=(-1000,4443)/raw≈(120.0,166.8)；value=8智慧符单独走两智慧符点逻辑：天辉智慧raw≈(66.0,134.0)/server≈(-7468,610)、夜魇智慧raw≈(191.0,118.0)/server≈(7537,-1285)</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
-        <x:v>使用时刻到第一个相关modifier移除；默认最短t+8，最长t+120或下一次同施法者开雾前</x:v>
+        <x:v>结果事件t-5到t；智慧符t-10到t；未刷新侧spawn_time-5到spawn_time</x:v>
       </x:c>
       <x:c r="G9" s="5" t="str">
-        <x:v>进入英雄1000码兜底；modifier linked window 120秒</x:v>
+        <x:v>符点附近1000码；能量符刷新间隔120秒；罐装后90秒内同英雄同神符拾取去重</x:v>
       </x:c>
       <x:c r="H9" s="5" t="str">
-        <x:v>使用者+进入雾的英雄</x:v>
+        <x:v>heroes=某符点附近两方英雄；赏金符按四个赏金点附近英雄记录；智慧符按两个智慧符点附近英雄记录</x:v>
       </x:c>
       <x:c r="I9" s="5" t="str">
-        <x:v>结果=使用者、进入英雄、位置</x:v>
+        <x:v>结果=英雄名+拾取/罐装/反补+上河道/下河道/天辉赏金符点/夜魇赏金符点/天辉智慧符点/夜魇智慧符点+神符；未刷新侧=神符刷新在另一侧；无结果可留空</x:v>
       </x:c>
       <x:c r="J9" s="5" t="str">
-        <x:v>按使用时间+队伍+英雄集合去重</x:v>
+        <x:v>每颗神符只记录一次；value=5按四赏金符点区分；value=8按两智慧符点区分；罐装优先于后续拾取</x:v>
       </x:c>
       <x:c r="K9" s="5" t="str">
-        <x:v>可与后续战斗并存</x:v>
+        <x:v>控符统一标签，不再输出帮控符/控智慧神符</x:v>
       </x:c>
       <x:c r="L9" s="5" t="str">
-        <x:v>DB可确定用雾，但开雾意图需复核</x:v>
+        <x:v>符点归属和附近英雄可人工复核</x:v>
       </x:c>
       <x:c r="M9" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N9" s="5" t="str"/>
     </x:row>
     <x:row r="10" ht="58.5" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>蹲人</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -849,40 +849,40 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>combat_logs; player_intervals2</x:v>
+        <x:v>英雄位置; 视野/路径上下文</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>发起阶段 N 抓 1：短窗口内同一目标被同一方至少2名英雄命中，且发起时刻目标附近被抓方只有该目标1人；被抓目标承受非远程主战斗伤害&gt;=600或死亡才保留；2000码外贡献者只标远程，不增加参与人数</x:v>
+        <x:v>英雄在潜在目标500-1000码范围长期隐藏/等待，通常在树林、阴影、视野盲区</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
-        <x:v>发起时刻t0所在战斗窗口</x:v>
+        <x:v>等待开始-接触或离开</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
-        <x:v>GANK_OPEN_WINDOW=8秒；t0取第二名不同进攻方英雄第一次命中目标；读取t0±1秒英雄位置；以被抓目标为中心1600码统计附近英雄；gank_victim_damage_min=600；远程贡献阈值2000码</x:v>
+        <x:v>建议500-1000码；等待时长需人工设定</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str">
-        <x:v>gank方发起英雄 + 被抓英雄 + 后续支援/反打英雄；远程贡献者写作英雄（远程）</x:v>
+        <x:v>蹲守方与被蹲目标</x:v>
       </x:c>
       <x:c r="I10" s="5" t="str">
-        <x:v>结果=GANK方、被抓目标、后续支援/反打、击杀比分和死亡列表；evidence写damage_taken_by_hero；1换1仍保留GANK语义</x:v>
+        <x:v>结果可留空或写蹲守结果</x:v>
       </x:c>
       <x:c r="J10" s="5" t="str">
-        <x:v>优先于小规模冲突；后续TP/走入/支援不取消GANK；远程贡献者不计入人数；被抓目标未死亡且承伤&lt;600的2v1消耗不输出为GANK；塔附近信息写入结果/evidence，不自动改成塔下</x:v>
+        <x:v>当前建议人工核查，不强制自动输出</x:v>
       </x:c>
       <x:c r="K10" s="5" t="str">
-        <x:v>高于小规模冲突；默认不被塔下/肉山团等上下文改写</x:v>
+        <x:v>若后续造成战斗，优先战斗类标签</x:v>
       </x:c>
       <x:c r="L10" s="5" t="str">
-        <x:v>需要人工校准远程消耗、多人已在场、支援是否已在t0±1秒战场半径内等边界</x:v>
+        <x:v>语义强依赖录像和视野</x:v>
       </x:c>
       <x:c r="M10" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N10" s="5" t="str"/>
     </x:row>
     <x:row r="11" ht="58.5" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>小规模冲突</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -891,40 +891,40 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
-        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+        <x:v>combat_logs</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>双方局部伤害/控制/死亡聚类；通常双方各2人以上且总人数&lt;=7，或总人数&gt;=4且有死亡但未达团战规模</x:v>
+        <x:v>item_smoke_of_deceit 使用；结合 smoke modifier 添加/移除确定进入雾英雄和结束时间</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>聚类开始-结束；候选先手可提前到控制/大伤害/先手技能时刻</x:v>
+        <x:v>使用时刻到第一个相关modifier移除；默认最短t+8，最长t+120或下一次同施法者开雾前</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
-        <x:v>跨信号间隔12秒；用尾部动态中心合并：最近12秒、最多8条有位置的信号平均位置到新信号距离&lt;=2200码才合并；英雄参与默认1600码</x:v>
+        <x:v>进入英雄1000码兜底；modifier linked window 120秒</x:v>
       </x:c>
       <x:c r="H11" s="5" t="str">
-        <x:v>只保留战斗核心附近或对参与英雄造成伤害/控制的英雄；排除远处未命中核心的独立消耗</x:v>
+        <x:v>使用者+进入雾的英雄</x:v>
       </x:c>
       <x:c r="I11" s="5" t="str">
-        <x:v>结果=击杀比分；死亡列表；无死亡写未记录英雄击杀/死亡无</x:v>
+        <x:v>结果=使用者、进入英雄、位置</x:v>
       </x:c>
       <x:c r="J11" s="5" t="str">
-        <x:v>v1.7+吸收旧单点候选；v1.10使用尾部动态中心，允许边打边走/追击累计到同一事件，同时避免跨区域消耗串联</x:v>
+        <x:v>按使用时间+队伍+英雄集合去重</x:v>
       </x:c>
       <x:c r="K11" s="5" t="str">
-        <x:v>低于团战，高于纯资源/控符事实</x:v>
+        <x:v>可与后续战斗并存</x:v>
       </x:c>
       <x:c r="L11" s="5" t="str">
-        <x:v>边界和语义建议录像复核</x:v>
+        <x:v>DB可确定用雾，但开雾意图需复核</x:v>
       </x:c>
       <x:c r="M11" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N11" s="5" t="str"/>
     </x:row>
     <x:row r="12" ht="58.5" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -933,40 +933,40 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+        <x:v>combat_logs; player_intervals2</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>双方多人持续交战；双方总参与通常各4人以上，且直接参与各&gt;=3人，并满足总伤害&gt;=2500、死亡&gt;=2或持续&gt;=15秒之一</x:v>
+        <x:v>发起阶段 N 抓 1：短窗口内同一目标被同一方至少2名英雄命中，且发起时刻目标附近被抓方只有该目标1人；被抓目标承受非远程主战斗伤害&gt;=600或死亡才保留；2000码外贡献者只标远程，不增加参与人数</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
-        <x:v>聚类开始-结束；先手技能可提前开始</x:v>
+        <x:v>发起时刻t0所在战斗窗口</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
-        <x:v>团战人数阈值4v4；直接参与3v3；伤害2500；死亡2；持续15秒</x:v>
+        <x:v>GANK_OPEN_WINDOW=8秒；t0取第二名不同进攻方英雄第一次命中目标；读取t0±1秒英雄位置；以被抓目标为中心1600码统计附近英雄；gank_victim_damage_min=600；远程贡献阈值2000码</x:v>
       </x:c>
       <x:c r="H12" s="5" t="str">
-        <x:v>同小规模冲突，按空间/交互排除远端独立交互</x:v>
+        <x:v>gank方发起英雄 + 被抓英雄 + 后续支援/反打英雄；远程贡献者写作英雄（远程）</x:v>
       </x:c>
       <x:c r="I12" s="5" t="str">
-        <x:v>结果=击杀比分；死亡列表；带盾阵亡需标注</x:v>
+        <x:v>结果=GANK方、被抓目标、后续支援/反打、击杀比分和死亡列表；evidence写damage_taken_by_hero；1换1仍保留GANK语义</x:v>
       </x:c>
       <x:c r="J12" s="5" t="str">
-        <x:v>与特殊战斗标签可并存：肉山团/高地团/塔下/魔晶团</x:v>
+        <x:v>优先于小规模冲突；后续TP/走入/支援不取消GANK；远程贡献者不计入人数；被抓目标未死亡且承伤&lt;600的2v1消耗不输出为GANK；塔附近信息写入结果/evidence，不自动改成塔下</x:v>
       </x:c>
       <x:c r="K12" s="5" t="str">
-        <x:v>优先级高于小规模冲突；被特殊战斗标签修饰</x:v>
+        <x:v>高于小规模冲突；默认不被塔下/肉山团等上下文改写</x:v>
       </x:c>
       <x:c r="L12" s="5" t="str">
-        <x:v>远距离同时开战要拆分，不可只按时间合并</x:v>
+        <x:v>需要人工校准远程消耗、多人已在场、支援是否已在t0±1秒战场半径内等边界</x:v>
       </x:c>
       <x:c r="M12" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N12" s="5" t="str"/>
     </x:row>
     <x:row r="13" ht="58.5" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -978,79 +978,79 @@
         <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>肉山仍存活，且战斗围绕肉山坑/肉山伤害/肉山击杀上下文展开；团战/小规模冲突中心在肉山上路坑或下路坑2000码内时，记录为对应坑位战斗</x:v>
+        <x:v>双方局部伤害/控制/死亡聚类；通常双方各2人以上且总人数&lt;=7，或总人数&gt;=4且有死亡但未达团战规模；前10分钟使用对线期分段口径，单条伤害阈值30、跨信号间隔7秒；短事件&lt;=12秒保留单个英雄承伤&gt;400或总伤害&gt;900；长事件&gt;12秒改看滑动8秒爆发窗口，8秒内总伤害&gt;=700或单英雄承伤&gt;=360或有死亡才保留；10分钟后维持旧口径，单条伤害阈值45、跨信号间隔12秒，总伤害&gt;=550或有英雄死亡即可保留</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
-        <x:v>战斗窗口；肉山伤害前后30秒；肉山击杀前45秒到后75秒</x:v>
+        <x:v>聚类开始-结束；候选先手可提前到控制/大伤害/先手技能时刻</x:v>
       </x:c>
       <x:c r="G13" s="5" t="str">
-        <x:v>肉山上路坑server=(-3084,2296)，raw≈(102.6,148.3)；肉山下路坑server=(2842,-2743)，raw≈(152.1,105.9)；坑位半径2000码；肉山死亡后480秒内视为未刷新</x:v>
+        <x:v>0&lt;=time&lt;600：跨信号间隔7秒，尾部动态中心最近7秒；duration&lt;=12秒看整段单英雄承伤&gt;400或总伤害&gt;900；duration&gt;12秒看滑动8秒窗口，总伤害&gt;=700或单英雄承伤&gt;=360或有死亡；time&gt;=600：跨信号间隔12秒，尾部动态中心最近12秒；两个阶段均最多8条有位置信号，中心到新信号距离&lt;=2200码才合并；英雄参与默认1600码</x:v>
       </x:c>
       <x:c r="H13" s="5" t="str">
-        <x:v>参与战斗双方英雄</x:v>
+        <x:v>只保留战斗核心附近或对参与英雄造成伤害/控制的英雄；排除远处未命中核心的独立消耗</x:v>
       </x:c>
       <x:c r="I13" s="5" t="str">
-        <x:v>结果追加目标：肉山相关；坑位空间命中时补充“肉山上路坑战斗/肉山下路坑战斗”；肉山击杀结果由肉山击杀标签独立记录</x:v>
+        <x:v>结果=击杀比分；死亡列表；无死亡写未记录英雄击杀/死亡无</x:v>
       </x:c>
       <x:c r="J13" s="5" t="str">
-        <x:v>坑位空间规则只修饰团战/小规模冲突，不改写GANK/单杀；肉山死亡后的追击不再因靠近肉山坑误标肉山团</x:v>
+        <x:v>v1.7+吸收旧单点候选；v1.10使用尾部动态中心，允许边打边走/追击累计到同一事件，同时避免跨区域消耗串联；前10分钟长窗口必须有明确爆发，避免对线换血被过长串联或低强度死亡单独带出</x:v>
       </x:c>
       <x:c r="K13" s="5" t="str">
-        <x:v>可与团战/小规模冲突并存</x:v>
+        <x:v>低于团战，高于纯资源/控符事实</x:v>
       </x:c>
       <x:c r="L13" s="5" t="str">
-        <x:v>需区分肉山尝试、肉山击杀、肉山后追击</x:v>
+        <x:v>边界和语义建议录像复核</x:v>
       </x:c>
       <x:c r="M13" s="5" t="str">
-        <x:v>v1.4-v1.10草案</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="N13" s="5" t="str"/>
     </x:row>
     <x:row r="14" ht="58.5" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>auto</x:v>
+        <x:v>candidate_review</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
-        <x:v>combat_logs; match_chat_events</x:v>
+        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E14" s="5" t="str">
-        <x:v>Roshan死亡事件；统一记录为肉山击杀，不再作为普通资源获得输出；合并同一波肉山掉落</x:v>
+        <x:v>双方多人持续交战；双方总参与通常各4人以上，且直接参与各&gt;=3人，并满足总伤害&gt;=2500、死亡&gt;=2或持续&gt;=15秒之一</x:v>
       </x:c>
       <x:c r="F14" s="5" t="str">
-        <x:v>击杀时刻到最后一个20秒内相关掉落</x:v>
+        <x:v>聚类开始-结束；先手技能可提前开始</x:v>
       </x:c>
       <x:c r="G14" s="5" t="str">
-        <x:v>掉落合并窗口20秒；击杀归属优先combat_logs roshan_death；缺失时用5秒内掉落阵营兜底</x:v>
+        <x:v>团战人数阈值4v4；直接参与3v3；伤害2500；死亡2；持续15秒</x:v>
       </x:c>
       <x:c r="H14" s="5" t="str">
-        <x:v>获得掉落的英雄/阵营；heroes合并击杀和掉落相关英雄</x:v>
+        <x:v>同小规模冲突，按空间/交互排除远端独立交互</x:v>
       </x:c>
       <x:c r="I14" s="5" t="str">
-        <x:v>结果=哪方击杀肉山；哪个英雄获得盾/奶酪/刷新碎片/战旗等</x:v>
+        <x:v>结果=击杀比分；死亡列表；带盾阵亡需标注</x:v>
       </x:c>
       <x:c r="J14" s="5" t="str">
-        <x:v>CHAT_MESSAGE_ROSHAN_KILL的player/value不作为击杀英雄依据</x:v>
+        <x:v>与特殊战斗标签可并存：肉山团/高地团/塔下/魔晶团</x:v>
       </x:c>
       <x:c r="K14" s="5" t="str">
-        <x:v>优先级高于资源获得；同一肉山只一行</x:v>
+        <x:v>优先级高于小规模冲突；被特殊战斗标签修饰</x:v>
       </x:c>
       <x:c r="L14" s="5" t="str">
-        <x:v>需人工检查掉落事件是否完整合并</x:v>
+        <x:v>远距离同时开战要拆分，不可只按时间合并</x:v>
       </x:c>
       <x:c r="M14" s="5" t="str">
-        <x:v>v1.8-v1.9</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N14" s="5" t="str"/>
     </x:row>
     <x:row r="15" ht="58.5" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>高地团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1059,82 +1059,82 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D15" s="5" t="str">
-        <x:v>combat_logs; tower/barracks events; player_intervals2</x:v>
+        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
-        <x:v>一方或双方在高地、基地入口、破路区域发生团战/小规模冲突</x:v>
+        <x:v>15分钟后，团战/小规模冲突中读取开战后的前3个秒点(start,start+1,start+2)，对所有参与英雄本体坐标求平均；该平均坐标在肉山坑1000码内时，记录为对应坑位战斗；肉山击杀/掉落只作为资源事实，不作为肉山团充分条件</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
-        <x:v>战斗窗口；兵营击杀前20秒到后60秒</x:v>
+        <x:v>15:00后；战斗开始后前3秒</x:v>
       </x:c>
       <x:c r="G15" s="5" t="str">
-        <x:v>中心raw坐标x&lt;95且y&lt;95或x&gt;158且y&gt;158；或兵营事件附近</x:v>
+        <x:v>肉山上路坑server=(-2924.964844,1522.657715)，raw≈(104.0,141.7)；肉山下路坑server=(2867.646973,-3401.379395)，raw≈(152.3,100.5)；坑位半径1000码；15分钟前不计算肉山团</x:v>
       </x:c>
       <x:c r="H15" s="5" t="str">
         <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I15" s="5" t="str">
-        <x:v>结果继承战斗结果</x:v>
+        <x:v>结果追加目标：肉山相关；坑位空间命中时补充“肉山上路坑战斗/肉山下路坑战斗”；肉山击杀结果由肉山击杀标签独立记录</x:v>
       </x:c>
       <x:c r="J15" s="5" t="str">
-        <x:v>作为附加标签插入战斗标签前</x:v>
+        <x:v>不再用任意一条伤害/控制/死亡交互点靠近肉山坑作为充分条件；坑位空间规则只修饰15分钟后的团战/小规模冲突，不改写GANK/单杀；肉山死亡后的追击不再因靠近肉山坑误标肉山团</x:v>
       </x:c>
       <x:c r="K15" s="5" t="str">
-        <x:v>特殊战斗标签优先级高</x:v>
+        <x:v>可与团战/小规模冲突并存</x:v>
       </x:c>
       <x:c r="L15" s="5" t="str">
-        <x:v>高地前poke与正式开团需复核</x:v>
+        <x:v>需区分肉山尝试、肉山击杀、肉山后追击；15分钟前即使靠近肉山坑也不标肉山团</x:v>
       </x:c>
       <x:c r="M15" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="N15" s="5" t="str"/>
     </x:row>
     <x:row r="16" ht="58.5" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>塔下</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>candidate_review</x:v>
+        <x:v>auto</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
-        <x:v>tower_status_update; combat_logs</x:v>
+        <x:v>combat_logs; match_chat_events</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>一方在防御塔附近约1000码内防守时发生的战斗</x:v>
+        <x:v>Roshan死亡事件；统一记录为肉山击杀，不再作为普通资源获得输出；合并同一波肉山掉落</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
-        <x:v>战斗开始前5秒到结束后5秒内塔上下文</x:v>
+        <x:v>击杀时刻到最后一个20秒内相关掉落</x:v>
       </x:c>
       <x:c r="G16" s="5" t="str">
-        <x:v>防御塔1000码；塔hp&gt;0</x:v>
+        <x:v>掉落合并窗口20秒；击杀归属优先combat_logs roshan_death；缺失时用5秒内掉落阵营兜底</x:v>
       </x:c>
       <x:c r="H16" s="5" t="str">
-        <x:v>参与战斗双方英雄</x:v>
+        <x:v>获得掉落的英雄/阵营；heroes合并击杀和掉落相关英雄</x:v>
       </x:c>
       <x:c r="I16" s="5" t="str">
-        <x:v>结果继承战斗结果并附塔上下文</x:v>
+        <x:v>结果=哪方击杀肉山；哪个英雄获得盾/奶酪/刷新碎片/战旗等</x:v>
       </x:c>
       <x:c r="J16" s="5" t="str">
-        <x:v>作为附加标签追加，可与小规模冲突/团战并存</x:v>
+        <x:v>CHAT_MESSAGE_ROSHAN_KILL的player/value不作为击杀英雄依据</x:v>
       </x:c>
       <x:c r="K16" s="5" t="str">
-        <x:v>特殊上下文标签</x:v>
+        <x:v>优先级高于资源获得；同一肉山只一行</x:v>
       </x:c>
       <x:c r="L16" s="5" t="str">
-        <x:v>塔已掉或追击阶段不应误标</x:v>
+        <x:v>需人工检查掉落事件是否完整合并</x:v>
       </x:c>
       <x:c r="M16" s="5" t="str">
-        <x:v>v1.4-v1.9</x:v>
+        <x:v>v1.8-v1.9</x:v>
       </x:c>
       <x:c r="N16" s="5" t="str"/>
     </x:row>
     <x:row r="17" ht="58.5" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>高地团</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1143,31 +1143,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D17" s="5" t="str">
-        <x:v>combat_logs</x:v>
+        <x:v>combat_logs; tower/barracks events; player_intervals2</x:v>
       </x:c>
       <x:c r="E17" s="5" t="str">
-        <x:v>对Roshan造成伤害但未完成击杀，也未转化为肉山团</x:v>
+        <x:v>一方或双方在高地、基地入口、破路区域发生团战/小规模冲突</x:v>
       </x:c>
       <x:c r="F17" s="5" t="str">
-        <x:v>连续Roshan伤害组；组内间隔&lt;=45秒；结束后+10秒</x:v>
+        <x:v>战斗窗口；兵营击杀前20秒到后60秒</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
-        <x:v>总伤害&gt;=1500；攻击英雄&gt;=1；组内无击杀且结束后8秒无击杀</x:v>
+        <x:v>中心raw坐标x&lt;95且y&lt;95或x&gt;158且y&gt;158；或兵营事件附近</x:v>
       </x:c>
       <x:c r="H17" s="5" t="str">
-        <x:v>对肉山造成伤害的英雄</x:v>
+        <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I17" s="5" t="str">
-        <x:v>结果=Roshan总伤害和未击杀说明</x:v>
+        <x:v>结果继承战斗结果</x:v>
       </x:c>
       <x:c r="J17" s="5" t="str">
-        <x:v>若双方围绕肉山开战，优先肉山团</x:v>
+        <x:v>作为附加标签插入战斗标签前</x:v>
       </x:c>
       <x:c r="K17" s="5" t="str">
-        <x:v>低于肉山团/肉山击杀</x:v>
+        <x:v>特殊战斗标签优先级高</x:v>
       </x:c>
       <x:c r="L17" s="5" t="str">
-        <x:v>偷Roshan试探与真尝试需复核</x:v>
+        <x:v>高地前poke与正式开团需复核</x:v>
       </x:c>
       <x:c r="M17" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -1176,7 +1176,7 @@
     </x:row>
     <x:row r="18" ht="58.5" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>塔下</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
         <x:v>candidate_review</x:v>
@@ -1185,31 +1185,31 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
-        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+        <x:v>tower_status_update; combat_logs</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
-        <x:v>折磨者/魔晶仍存活时，围绕魔晶区域发生团战或资源争夺</x:v>
+        <x:v>一方在防御塔附近约1000码内防守时发生的战斗</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>战斗窗口；魔晶伤害前后30秒；击杀前45秒到后60秒</x:v>
+        <x:v>战斗开始前5秒到结束后5秒内塔上下文</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
-        <x:v>魔晶区域1500-2000码；20分钟后可存活；击杀后600秒内视为未刷新</x:v>
+        <x:v>防御塔1000码；塔hp&gt;0</x:v>
       </x:c>
       <x:c r="H18" s="5" t="str">
         <x:v>参与战斗双方英雄</x:v>
       </x:c>
       <x:c r="I18" s="5" t="str">
-        <x:v>结果继承战斗结果或写魔晶归属</x:v>
+        <x:v>结果继承战斗结果并附塔上下文</x:v>
       </x:c>
       <x:c r="J18" s="5" t="str">
-        <x:v>魔晶击杀后追击不再误标魔晶团</x:v>
+        <x:v>作为附加标签追加，可与小规模冲突/团战并存</x:v>
       </x:c>
       <x:c r="K18" s="5" t="str">
-        <x:v>特殊战斗标签优先级高</x:v>
+        <x:v>特殊上下文标签</x:v>
       </x:c>
       <x:c r="L18" s="5" t="str">
-        <x:v>需区分单方打魔晶与双方争夺</x:v>
+        <x:v>塔已掉或追击阶段不应误标</x:v>
       </x:c>
       <x:c r="M18" s="5" t="str">
         <x:v>v1.4-v1.9</x:v>
@@ -1218,87 +1218,171 @@
     </x:row>
     <x:row r="19" ht="58.5" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>资源获得</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>auto</x:v>
+        <x:v>candidate_review</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D19" s="5" t="str">
-        <x:v>match_chat_events; combat_logs</x:v>
+        <x:v>combat_logs</x:v>
       </x:c>
       <x:c r="E19" s="5" t="str">
-        <x:v>独立记录关键资源事实：魔晶/折磨者、战旗等；v1.8后肉山击杀与肉山掉落并入肉山击杀，不再单独输出普通资源获得</x:v>
+        <x:v>对Roshan造成伤害但未完成击杀，也未转化为肉山团</x:v>
       </x:c>
       <x:c r="F19" s="5" t="str">
-        <x:v>资源事件时刻</x:v>
+        <x:v>连续Roshan伤害组；组内间隔&lt;=45秒；结束后+10秒</x:v>
       </x:c>
       <x:c r="G19" s="5" t="str">
-        <x:v>Roshan kill归属兜底5秒；普通资源按chat事件</x:v>
+        <x:v>总伤害&gt;=1500；攻击英雄&gt;=1；组内无击杀且结束后8秒无击杀</x:v>
       </x:c>
       <x:c r="H19" s="5" t="str">
-        <x:v>获得资源的英雄或阵营</x:v>
+        <x:v>对肉山造成伤害的英雄</x:v>
       </x:c>
       <x:c r="I19" s="5" t="str">
-        <x:v>结果=英雄/阵营+资源动作</x:v>
+        <x:v>结果=Roshan总伤害和未击杀说明</x:v>
       </x:c>
       <x:c r="J19" s="5" t="str">
-        <x:v>旧抢盾/抢奶/抢刷新并入资源获得或肉山击杀口径</x:v>
+        <x:v>若双方围绕肉山开战，优先肉山团</x:v>
       </x:c>
       <x:c r="K19" s="5" t="str">
-        <x:v>低于肉山击杀</x:v>
+        <x:v>低于肉山团/肉山击杀</x:v>
       </x:c>
       <x:c r="L19" s="5" t="str">
-        <x:v>需要确认非肉山资源未被误合并</x:v>
+        <x:v>偷Roshan试探与真尝试需复核</x:v>
       </x:c>
       <x:c r="M19" s="5" t="str">
-        <x:v>v1.5-v1.9</x:v>
+        <x:v>v1.4-v1.9</x:v>
       </x:c>
       <x:c r="N19" s="5" t="str"/>
     </x:row>
     <x:row r="20" ht="58.5" customHeight="1">
       <x:c r="A20" s="5" t="str">
+        <x:v>魔晶团</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="str">
+        <x:v>candidate_review</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="str">
+        <x:v>combat_logs; match_chat_events; player_intervals2</x:v>
+      </x:c>
+      <x:c r="E20" s="5" t="str">
+        <x:v>折磨者/魔晶仍存活时，围绕魔晶区域发生团战或资源争夺</x:v>
+      </x:c>
+      <x:c r="F20" s="5" t="str">
+        <x:v>战斗窗口；魔晶伤害前后30秒；击杀前45秒到后60秒</x:v>
+      </x:c>
+      <x:c r="G20" s="5" t="str">
+        <x:v>魔晶区域1500-2000码；20分钟后可存活；击杀后600秒内视为未刷新</x:v>
+      </x:c>
+      <x:c r="H20" s="5" t="str">
+        <x:v>参与战斗双方英雄</x:v>
+      </x:c>
+      <x:c r="I20" s="5" t="str">
+        <x:v>结果继承战斗结果或写魔晶归属</x:v>
+      </x:c>
+      <x:c r="J20" s="5" t="str">
+        <x:v>魔晶击杀后追击不再误标魔晶团</x:v>
+      </x:c>
+      <x:c r="K20" s="5" t="str">
+        <x:v>特殊战斗标签优先级高</x:v>
+      </x:c>
+      <x:c r="L20" s="5" t="str">
+        <x:v>需区分单方打魔晶与双方争夺</x:v>
+      </x:c>
+      <x:c r="M20" s="5" t="str">
+        <x:v>v1.4-v1.9</x:v>
+      </x:c>
+      <x:c r="N20" s="5" t="str"/>
+    </x:row>
+    <x:row r="21" ht="58.5" customHeight="1">
+      <x:c r="A21" s="5" t="str">
+        <x:v>资源获得</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="str">
+        <x:v>auto</x:v>
+      </x:c>
+      <x:c r="C21" s="5" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D21" s="5" t="str">
+        <x:v>match_chat_events; combat_logs</x:v>
+      </x:c>
+      <x:c r="E21" s="5" t="str">
+        <x:v>独立记录关键资源事实：魔晶/折磨者、战旗等；v1.8后肉山击杀与肉山掉落并入肉山击杀，不再单独输出普通资源获得</x:v>
+      </x:c>
+      <x:c r="F21" s="5" t="str">
+        <x:v>资源事件时刻</x:v>
+      </x:c>
+      <x:c r="G21" s="5" t="str">
+        <x:v>Roshan kill归属兜底5秒；普通资源按chat事件</x:v>
+      </x:c>
+      <x:c r="H21" s="5" t="str">
+        <x:v>获得资源的英雄或阵营</x:v>
+      </x:c>
+      <x:c r="I21" s="5" t="str">
+        <x:v>结果=英雄/阵营+资源动作</x:v>
+      </x:c>
+      <x:c r="J21" s="5" t="str">
+        <x:v>旧抢盾/抢奶/抢刷新并入资源获得或肉山击杀口径</x:v>
+      </x:c>
+      <x:c r="K21" s="5" t="str">
+        <x:v>低于肉山击杀</x:v>
+      </x:c>
+      <x:c r="L21" s="5" t="str">
+        <x:v>需要确认非肉山资源未被误合并</x:v>
+      </x:c>
+      <x:c r="M21" s="5" t="str">
+        <x:v>v1.5-v1.9</x:v>
+      </x:c>
+      <x:c r="N21" s="5" t="str"/>
+    </x:row>
+    <x:row r="22" ht="58.5" customHeight="1">
+      <x:c r="A22" s="5" t="str">
         <x:v>带盾阵亡</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="str">
+      <x:c r="B22" s="5" t="str">
         <x:v>auto</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="str">
+      <x:c r="C22" s="5" t="str">
         <x:v>A/B</x:v>
       </x:c>
-      <x:c r="D20" s="5" t="str">
+      <x:c r="D22" s="5" t="str">
         <x:v>match_chat_events; combat_logs</x:v>
       </x:c>
-      <x:c r="E20" s="5" t="str">
+      <x:c r="E22" s="5" t="str">
         <x:v>持有不朽盾的英雄死亡/消耗盾时独立记录；战斗死亡列表也标注[带盾阵亡]</x:v>
       </x:c>
-      <x:c r="F20" s="5" t="str">
+      <x:c r="F22" s="5" t="str">
         <x:v>死亡时刻</x:v>
       </x:c>
-      <x:c r="G20" s="5" t="str">
+      <x:c r="G22" s="5" t="str">
         <x:v>Aegis领取后300秒内的同英雄死亡；每个盾只消费一次</x:v>
       </x:c>
-      <x:c r="H20" s="5" t="str">
+      <x:c r="H22" s="5" t="str">
         <x:v>带盾阵亡英雄及阵营</x:v>
       </x:c>
-      <x:c r="I20" s="5" t="str">
+      <x:c r="I22" s="5" t="str">
         <x:v>结果=死亡时间、英雄、Aegis获取时间</x:v>
       </x:c>
-      <x:c r="J20" s="5" t="str">
+      <x:c r="J22" s="5" t="str">
         <x:v>可与团战/小规模冲突并存</x:v>
       </x:c>
-      <x:c r="K20" s="5" t="str">
+      <x:c r="K22" s="5" t="str">
         <x:v>资源消耗事实类</x:v>
       </x:c>
-      <x:c r="L20" s="5" t="str">
+      <x:c r="L22" s="5" t="str">
         <x:v>复活/盾消耗边界建议复核</x:v>
       </x:c>
-      <x:c r="M20" s="5" t="str">
+      <x:c r="M22" s="5" t="str">
         <x:v>v1.5-v1.9</x:v>
       </x:c>
-      <x:c r="N20" s="5" t="str"/>
+      <x:c r="N22" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1347,22 +1431,22 @@
     </x:row>
     <x:row r="2" ht="33" customHeight="1">
       <x:c r="A2" s="5" t="str">
-        <x:v>lane_initial_window</x:v>
+        <x:v>opening_creep_contest_max_time</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>0-300</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>seconds</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
-        <x:v>对线分路</x:v>
+        <x:v>出门抢远程兵/近战兵</x:v>
       </x:c>
       <x:c r="E2" s="5" t="str">
-        <x:v>初始分路线判断窗口</x:v>
+        <x:v>只统计0-31秒内死亡的上路/下路远程兵/近战兵，中路不识别</x:v>
       </x:c>
       <x:c r="F2" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="G2" s="5" t="str">
         <x:v>是</x:v>
@@ -1371,22 +1455,22 @@
     </x:row>
     <x:row r="3" ht="33" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>secondary_lane_seconds</x:v>
+        <x:v>opening_creep_reward_window</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>60</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>seconds</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>对线分路</x:v>
+        <x:v>出门抢远程兵/近战兵</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>超过该停留时长记录游走/次要路</x:v>
+        <x:v>读取小兵死亡日志前后1秒相邻日志块中的金钱和经验</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
         <x:v>是</x:v>
@@ -1395,22 +1479,22 @@
     </x:row>
     <x:row r="4" ht="33" customHeight="1">
       <x:c r="A4" s="5" t="str">
-        <x:v>lane_zone_sample_window</x:v>
+        <x:v>opening_creep_gold_exclude_reason</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>0-600</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>gold_reason</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
-        <x:v>对线区</x:v>
+        <x:v>出门抢远程兵/近战兵</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>生成本局对线区的正常交汇样本窗口</x:v>
+        <x:v>排除开局发钱；负数金钱也不计入金钱获得者</x:v>
       </x:c>
       <x:c r="F4" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str">
         <x:v>是</x:v>
@@ -1419,22 +1503,22 @@
     </x:row>
     <x:row r="5" ht="33" customHeight="1">
       <x:c r="A5" s="5" t="str">
-        <x:v>lane_zone_near_enemy_creep_radius</x:v>
+        <x:v>lane_initial_window</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>500</x:v>
+        <x:v>0-300</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>对线区</x:v>
+        <x:v>对线分路</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>正常交汇样本要求死亡点附近存在敌方同路线线上小兵</x:v>
+        <x:v>初始分路线判断窗口</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
         <x:v>是</x:v>
@@ -1443,22 +1527,22 @@
     </x:row>
     <x:row r="6" ht="33" customHeight="1">
       <x:c r="A6" s="5" t="str">
-        <x:v>lane_zone_quantile_low</x:v>
+        <x:v>secondary_lane_seconds</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>0.10</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C6" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D6" s="5" t="str">
-        <x:v>对线区</x:v>
+        <x:v>对线分路</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
-        <x:v>生成对线区bbox时x/y低分位，去除极端死亡点</x:v>
+        <x:v>超过该停留时长记录游走/次要路</x:v>
       </x:c>
       <x:c r="F6" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
         <x:v>是</x:v>
@@ -1467,19 +1551,19 @@
     </x:row>
     <x:row r="7" ht="33" customHeight="1">
       <x:c r="A7" s="5" t="str">
-        <x:v>lane_zone_quantile_high</x:v>
+        <x:v>lane_zone_sample_window</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>0.90</x:v>
+        <x:v>0-600</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
         <x:v>对线区</x:v>
       </x:c>
       <x:c r="E7" s="5" t="str">
-        <x:v>生成对线区bbox时x/y高分位，去除极端死亡点</x:v>
+        <x:v>生成本局对线区的正常交汇样本窗口</x:v>
       </x:c>
       <x:c r="F7" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1491,19 +1575,19 @@
     </x:row>
     <x:row r="8" ht="33" customHeight="1">
       <x:c r="A8" s="5" t="str">
-        <x:v>lane_zone_margin_raw</x:v>
+        <x:v>lane_zone_near_enemy_creep_radius</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="C8" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
         <x:v>对线区</x:v>
       </x:c>
       <x:c r="E8" s="5" t="str">
-        <x:v>对线区bbox外扩容差</x:v>
+        <x:v>正常交汇样本要求死亡点附近存在敌方同路线线上小兵</x:v>
       </x:c>
       <x:c r="F8" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1515,19 +1599,19 @@
     </x:row>
     <x:row r="9" ht="33" customHeight="1">
       <x:c r="A9" s="5" t="str">
-        <x:v>lane_zone_min_samples</x:v>
+        <x:v>lane_zone_quantile_low</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>12</x:v>
+        <x:v>0.10</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>个</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>对线区</x:v>
       </x:c>
       <x:c r="E9" s="5" t="str">
-        <x:v>单路线本局自适应对线区所需最少正常交汇样本</x:v>
+        <x:v>生成对线区bbox时x/y低分位，去除极端死亡点</x:v>
       </x:c>
       <x:c r="F9" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1539,19 +1623,19 @@
     </x:row>
     <x:row r="10" ht="33" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>lane_zone_tower_protect_radius</x:v>
+        <x:v>lane_zone_quantile_high</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>12</x:v>
+        <x:v>0.90</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
         <x:v>对线区</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>该路线任一存活一塔附近视为正常塔下吃兵区，不进入断线/勾兵候选</x:v>
+        <x:v>生成对线区bbox时x/y高分位，去除极端死亡点</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1563,19 +1647,19 @@
     </x:row>
     <x:row r="11" ht="33" customHeight="1">
       <x:c r="A11" s="5" t="str">
-        <x:v>lane_creep_source_early_seconds</x:v>
+        <x:v>lane_zone_margin_raw</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C11" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D11" s="5" t="str">
         <x:v>对线区</x:v>
       </x:c>
       <x:c r="E11" s="5" t="str">
-        <x:v>有ehandle时用小兵最早出现后8秒内轨迹判断source_lane</x:v>
+        <x:v>对线区bbox外扩容差</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1587,22 +1671,22 @@
     </x:row>
     <x:row r="12" ht="33" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>stack_event_window</x:v>
+        <x:v>lane_zone_min_samples</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>±5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C12" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="D12" s="5" t="str">
-        <x:v>囤野/堆野</x:v>
+        <x:v>对线区</x:v>
       </x:c>
       <x:c r="E12" s="5" t="str">
-        <x:v>堆野计数增加事件输出窗口</x:v>
+        <x:v>单路线本局自适应对线区所需最少正常交汇样本</x:v>
       </x:c>
       <x:c r="F12" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
         <x:v>是</x:v>
@@ -1611,22 +1695,22 @@
     </x:row>
     <x:row r="13" ht="33" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>pull_lane_max_time</x:v>
+        <x:v>lane_zone_tower_protect_radius</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>900</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C13" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D13" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>对线区</x:v>
       </x:c>
       <x:c r="E13" s="5" t="str">
-        <x:v>拉野候选只看前15分钟</x:v>
+        <x:v>该路线任一存活一塔附近视为正常塔下吃兵区，不进入断线/勾兵候选</x:v>
       </x:c>
       <x:c r="F13" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G13" s="5" t="str">
         <x:v>是</x:v>
@@ -1635,22 +1719,22 @@
     </x:row>
     <x:row r="14" ht="33" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>pull_group_gap</x:v>
+        <x:v>lane_creep_source_early_seconds</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>35</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D14" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>对线区</x:v>
       </x:c>
       <x:c r="E14" s="5" t="str">
-        <x:v>线上兵与中立交互合并为同一拉野组的最大间隔</x:v>
+        <x:v>有ehandle时用小兵最早出现后8秒内轨迹判断source_lane</x:v>
       </x:c>
       <x:c r="F14" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G14" s="5" t="str">
         <x:v>是</x:v>
@@ -1659,19 +1743,19 @@
     </x:row>
     <x:row r="15" ht="33" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>pull_group_distance_raw</x:v>
+        <x:v>stack_event_window</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>28</x:v>
+        <x:v>±5</x:v>
       </x:c>
       <x:c r="C15" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D15" s="5" t="str">
-        <x:v>拉野</x:v>
+        <x:v>囤野/堆野</x:v>
       </x:c>
       <x:c r="E15" s="5" t="str">
-        <x:v>拉野组位置合并距离</x:v>
+        <x:v>堆野计数增加事件输出窗口</x:v>
       </x:c>
       <x:c r="F15" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -1683,22 +1767,22 @@
     </x:row>
     <x:row r="16" ht="33" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>pull_status_proximity_game</x:v>
+        <x:v>pull_lane_max_time</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>550</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C16" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E16" s="5" t="str">
-        <x:v>线兵与中立野怪状态贴近的最大距离；有combat锚点时做锚点附近扫描，无combat锚点时做全局状态扫描；实现时换算为raw约4.23</x:v>
+        <x:v>拉野候选只看前15分钟</x:v>
       </x:c>
       <x:c r="F16" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G16" s="5" t="str">
         <x:v>是</x:v>
@@ -1707,10 +1791,10 @@
     </x:row>
     <x:row r="17" ht="33" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>pull_status_anchor_pre_window</x:v>
+        <x:v>pull_group_gap</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C17" s="5" t="str">
         <x:v>秒</x:v>
@@ -1719,10 +1803,10 @@
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E17" s="5" t="str">
-        <x:v>combat锚点前回溯状态贴近证据的最大窗口</x:v>
+        <x:v>线上兵与中立交互合并为同一拉野组的最大间隔</x:v>
       </x:c>
       <x:c r="F17" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
         <x:v>是</x:v>
@@ -1731,22 +1815,22 @@
     </x:row>
     <x:row r="18" ht="33" customHeight="1">
       <x:c r="A18" s="5" t="str">
-        <x:v>pull_status_anchor_post_window</x:v>
+        <x:v>pull_group_distance_raw</x:v>
       </x:c>
       <x:c r="B18" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C18" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D18" s="5" t="str">
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
-        <x:v>combat锚点后补充状态贴近证据的最大窗口</x:v>
+        <x:v>拉野组位置合并距离</x:v>
       </x:c>
       <x:c r="F18" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
         <x:v>是</x:v>
@@ -1755,10 +1839,10 @@
     </x:row>
     <x:row r="19" ht="33" customHeight="1">
       <x:c r="A19" s="5" t="str">
-        <x:v>pull_nearby_hero_radius</x:v>
+        <x:v>pull_status_proximity_game</x:v>
       </x:c>
       <x:c r="B19" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="C19" s="5" t="str">
         <x:v>码</x:v>
@@ -1767,10 +1851,10 @@
         <x:v>拉野</x:v>
       </x:c>
       <x:c r="E19" s="5" t="str">
-        <x:v>拉野附近英雄归属半径</x:v>
+        <x:v>线兵与中立野怪状态贴近的最大距离；有combat锚点时做锚点附近扫描，无combat锚点时做全局状态扫描；实现时换算为raw约4.23</x:v>
       </x:c>
       <x:c r="F19" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G19" s="5" t="str">
         <x:v>是</x:v>
@@ -1779,19 +1863,19 @@
     </x:row>
     <x:row r="20" ht="33" customHeight="1">
       <x:c r="A20" s="5" t="str">
-        <x:v>aggro_lane_max_time</x:v>
+        <x:v>pull_status_anchor_pre_window</x:v>
       </x:c>
       <x:c r="B20" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C20" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D20" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E20" s="5" t="str">
-        <x:v>勾兵候选默认只看前10分钟，可由人工样本校准</x:v>
+        <x:v>combat锚点前回溯状态贴近证据的最大窗口</x:v>
       </x:c>
       <x:c r="F20" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1803,19 +1887,19 @@
     </x:row>
     <x:row r="21" ht="33" customHeight="1">
       <x:c r="A21" s="5" t="str">
-        <x:v>aggro_lane_enemy_creep_radius</x:v>
+        <x:v>pull_status_anchor_post_window</x:v>
       </x:c>
       <x:c r="B21" s="5" t="str">
-        <x:v>500</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C21" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D21" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E21" s="5" t="str">
-        <x:v>死亡小兵附近存在敌方线上小兵的判定半径</x:v>
+        <x:v>combat锚点后补充状态贴近证据的最大窗口</x:v>
       </x:c>
       <x:c r="F21" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1827,22 +1911,22 @@
     </x:row>
     <x:row r="22" ht="33" customHeight="1">
       <x:c r="A22" s="5" t="str">
-        <x:v>aggro_lane_group_gap</x:v>
+        <x:v>pull_nearby_hero_radius</x:v>
       </x:c>
       <x:c r="B22" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C22" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D22" s="5" t="str">
-        <x:v>勾兵</x:v>
+        <x:v>拉野</x:v>
       </x:c>
       <x:c r="E22" s="5" t="str">
-        <x:v>同一路线连续勾兵证据合并窗口</x:v>
+        <x:v>拉野附近英雄归属半径</x:v>
       </x:c>
       <x:c r="F22" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G22" s="5" t="str">
         <x:v>是</x:v>
@@ -1851,7 +1935,7 @@
     </x:row>
     <x:row r="23" ht="33" customHeight="1">
       <x:c r="A23" s="5" t="str">
-        <x:v>cut_lane_max_time</x:v>
+        <x:v>aggro_lane_max_time</x:v>
       </x:c>
       <x:c r="B23" s="5" t="str">
         <x:v>600</x:v>
@@ -1860,10 +1944,10 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D23" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E23" s="5" t="str">
-        <x:v>断线候选只看前10分钟</x:v>
+        <x:v>勾兵候选默认只看前10分钟，可由人工样本校准</x:v>
       </x:c>
       <x:c r="F23" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1875,7 +1959,7 @@
     </x:row>
     <x:row r="24" ht="33" customHeight="1">
       <x:c r="A24" s="5" t="str">
-        <x:v>cut_lane_enemy_creep_radius</x:v>
+        <x:v>aggro_lane_enemy_creep_radius</x:v>
       </x:c>
       <x:c r="B24" s="5" t="str">
         <x:v>500</x:v>
@@ -1884,10 +1968,10 @@
         <x:v>码</x:v>
       </x:c>
       <x:c r="D24" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E24" s="5" t="str">
-        <x:v>死亡小兵附近无敌方线上小兵的判定半径</x:v>
+        <x:v>死亡小兵附近存在敌方线上小兵的判定半径</x:v>
       </x:c>
       <x:c r="F24" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1899,7 +1983,7 @@
     </x:row>
     <x:row r="25" ht="33" customHeight="1">
       <x:c r="A25" s="5" t="str">
-        <x:v>cut_lane_group_gap</x:v>
+        <x:v>aggro_lane_group_gap</x:v>
       </x:c>
       <x:c r="B25" s="5" t="str">
         <x:v>10</x:v>
@@ -1908,10 +1992,10 @@
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D25" s="5" t="str">
-        <x:v>断线</x:v>
+        <x:v>勾兵</x:v>
       </x:c>
       <x:c r="E25" s="5" t="str">
-        <x:v>同一英雄同一路线连续断兵证据合并窗口</x:v>
+        <x:v>同一路线连续勾兵证据合并窗口</x:v>
       </x:c>
       <x:c r="F25" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1923,19 +2007,19 @@
     </x:row>
     <x:row r="26" ht="33" customHeight="1">
       <x:c r="A26" s="5" t="str">
-        <x:v>cut_lane_min_creep_deaths</x:v>
+        <x:v>cut_lane_max_time</x:v>
       </x:c>
       <x:c r="B26" s="5" t="str">
-        <x:v>2或3</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C26" s="5" t="str">
-        <x:v>个</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D26" s="5" t="str">
         <x:v>断线</x:v>
       </x:c>
       <x:c r="E26" s="5" t="str">
-        <x:v>10秒窗口内符合断线单条证据的小兵死亡数量阈值；2偏召回，3偏精确，需假设检验确定</x:v>
+        <x:v>断线候选只看前10分钟</x:v>
       </x:c>
       <x:c r="F26" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1947,22 +2031,22 @@
     </x:row>
     <x:row r="27" ht="33" customHeight="1">
       <x:c r="A27" s="5" t="str">
-        <x:v>rune_near_radius</x:v>
+        <x:v>cut_lane_enemy_creep_radius</x:v>
       </x:c>
       <x:c r="B27" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="C27" s="5" t="str">
         <x:v>码</x:v>
       </x:c>
       <x:c r="D27" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E27" s="5" t="str">
-        <x:v>符点附近两方英雄识别半径</x:v>
+        <x:v>死亡小兵附近无敌方线上小兵的判定半径</x:v>
       </x:c>
       <x:c r="F27" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G27" s="5" t="str">
         <x:v>是</x:v>
@@ -1971,19 +2055,19 @@
     </x:row>
     <x:row r="28" ht="33" customHeight="1">
       <x:c r="A28" s="5" t="str">
-        <x:v>radiant_bounty_rune_spot</x:v>
+        <x:v>cut_lane_group_gap</x:v>
       </x:c>
       <x:c r="B28" s="5" t="str">
-        <x:v>server=(590,-4637); raw≈(133.6,90.4)</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
-        <x:v>坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E28" s="5" t="str">
-        <x:v>天辉赏金符点；raw由当前homography从server坐标换算</x:v>
+        <x:v>同一英雄同一路线连续断兵证据合并窗口</x:v>
       </x:c>
       <x:c r="F28" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -1995,19 +2079,19 @@
     </x:row>
     <x:row r="29" ht="33" customHeight="1">
       <x:c r="A29" s="5" t="str">
-        <x:v>dire_bounty_rune_spot</x:v>
+        <x:v>cut_lane_min_creep_deaths</x:v>
       </x:c>
       <x:c r="B29" s="5" t="str">
-        <x:v>server=(-1000,4443); raw≈(120.0,166.8)</x:v>
+        <x:v>2或3</x:v>
       </x:c>
       <x:c r="C29" s="5" t="str">
-        <x:v>坐标</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="D29" s="5" t="str">
-        <x:v>控符</x:v>
+        <x:v>断线</x:v>
       </x:c>
       <x:c r="E29" s="5" t="str">
-        <x:v>夜魇赏金符点；raw由当前homography从server坐标换算</x:v>
+        <x:v>10秒窗口内符合断线单条证据的小兵死亡数量阈值；2偏召回，3偏精确，需假设检验确定</x:v>
       </x:c>
       <x:c r="F29" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -2019,22 +2103,22 @@
     </x:row>
     <x:row r="30" ht="33" customHeight="1">
       <x:c r="A30" s="5" t="str">
-        <x:v>radiant_wisdom_rune_spot</x:v>
+        <x:v>rune_near_radius</x:v>
       </x:c>
       <x:c r="B30" s="5" t="str">
-        <x:v>raw≈(66.0,134.0); server≈(-7468,610)</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C30" s="5" t="str">
-        <x:v>坐标</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D30" s="5" t="str">
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E30" s="5" t="str">
-        <x:v>天辉智慧符点；match_chat_events不直接给x/y，用拾取英雄同秒位置校准</x:v>
+        <x:v>符点附近两方英雄识别半径</x:v>
       </x:c>
       <x:c r="F30" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G30" s="5" t="str">
         <x:v>是</x:v>
@@ -2043,10 +2127,10 @@
     </x:row>
     <x:row r="31" ht="33" customHeight="1">
       <x:c r="A31" s="5" t="str">
-        <x:v>dire_wisdom_rune_spot</x:v>
+        <x:v>radiant_bounty_rune_spot</x:v>
       </x:c>
       <x:c r="B31" s="5" t="str">
-        <x:v>raw≈(191.0,118.0); server≈(7537,-1285)</x:v>
+        <x:v>server=(590,-4637); raw≈(133.6,90.4)</x:v>
       </x:c>
       <x:c r="C31" s="5" t="str">
         <x:v>坐标</x:v>
@@ -2055,7 +2139,7 @@
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E31" s="5" t="str">
-        <x:v>夜魇智慧符点；match_chat_events不直接给x/y，用拾取英雄同秒位置校准</x:v>
+        <x:v>天辉赏金符点；raw由当前homography从server坐标换算</x:v>
       </x:c>
       <x:c r="F31" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -2067,22 +2151,22 @@
     </x:row>
     <x:row r="32" ht="33" customHeight="1">
       <x:c r="A32" s="5" t="str">
-        <x:v>power_rune_spawn_interval</x:v>
+        <x:v>dire_bounty_rune_spot</x:v>
       </x:c>
       <x:c r="B32" s="5" t="str">
-        <x:v>120</x:v>
+        <x:v>server=(-1000,4443); raw≈(120.0,166.8)</x:v>
       </x:c>
       <x:c r="C32" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>坐标</x:v>
       </x:c>
       <x:c r="D32" s="5" t="str">
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E32" s="5" t="str">
-        <x:v>河道能量符刷新间隔，用于未刷新侧控符</x:v>
+        <x:v>夜魇赏金符点；raw由当前homography从server坐标换算</x:v>
       </x:c>
       <x:c r="F32" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G32" s="5" t="str">
         <x:v>是</x:v>
@@ -2091,22 +2175,22 @@
     </x:row>
     <x:row r="33" ht="33" customHeight="1">
       <x:c r="A33" s="5" t="str">
-        <x:v>power_rune_min_spawn_time</x:v>
+        <x:v>radiant_wisdom_rune_spot</x:v>
       </x:c>
       <x:c r="B33" s="5" t="str">
-        <x:v>360</x:v>
+        <x:v>raw≈(66.0,134.0); server≈(-7468,610)</x:v>
       </x:c>
       <x:c r="C33" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>坐标</x:v>
       </x:c>
       <x:c r="D33" s="5" t="str">
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E33" s="5" t="str">
-        <x:v>能量符最早按6分钟刷新计算</x:v>
+        <x:v>天辉智慧符点；match_chat_events不直接给x/y，用拾取英雄同秒位置校准</x:v>
       </x:c>
       <x:c r="F33" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G33" s="5" t="str">
         <x:v>是</x:v>
@@ -2115,22 +2199,22 @@
     </x:row>
     <x:row r="34" ht="33" customHeight="1">
       <x:c r="A34" s="5" t="str">
-        <x:v>power_rune_spawn_match_tolerance</x:v>
+        <x:v>dire_wisdom_rune_spot</x:v>
       </x:c>
       <x:c r="B34" s="5" t="str">
-        <x:v>90</x:v>
+        <x:v>raw≈(191.0,118.0); server≈(7537,-1285)</x:v>
       </x:c>
       <x:c r="C34" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>坐标</x:v>
       </x:c>
       <x:c r="D34" s="5" t="str">
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E34" s="5" t="str">
-        <x:v>将结果事件反推到最近能量符刷新点的容差</x:v>
+        <x:v>夜魇智慧符点；match_chat_events不直接给x/y，用拾取英雄同秒位置校准</x:v>
       </x:c>
       <x:c r="F34" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G34" s="5" t="str">
         <x:v>是</x:v>
@@ -2139,10 +2223,10 @@
     </x:row>
     <x:row r="35" ht="33" customHeight="1">
       <x:c r="A35" s="5" t="str">
-        <x:v>rune_bottle_pickup_suppression</x:v>
+        <x:v>power_rune_spawn_interval</x:v>
       </x:c>
       <x:c r="B35" s="5" t="str">
-        <x:v>90</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C35" s="5" t="str">
         <x:v>秒</x:v>
@@ -2151,7 +2235,7 @@
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E35" s="5" t="str">
-        <x:v>同英雄同神符罐装后拾取日志去重窗口</x:v>
+        <x:v>河道能量符刷新间隔，用于未刷新侧控符</x:v>
       </x:c>
       <x:c r="F35" s="5" t="str">
         <x:v>v1.5</x:v>
@@ -2163,10 +2247,10 @@
     </x:row>
     <x:row r="36" ht="33" customHeight="1">
       <x:c r="A36" s="5" t="str">
-        <x:v>wisdom_rune_window</x:v>
+        <x:v>power_rune_min_spawn_time</x:v>
       </x:c>
       <x:c r="B36" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C36" s="5" t="str">
         <x:v>秒</x:v>
@@ -2175,7 +2259,7 @@
         <x:v>控符</x:v>
       </x:c>
       <x:c r="E36" s="5" t="str">
-        <x:v>智慧符事件起点=t-10</x:v>
+        <x:v>能量符最早按6分钟刷新计算</x:v>
       </x:c>
       <x:c r="F36" s="5" t="str">
         <x:v>v1.5</x:v>
@@ -2187,22 +2271,22 @@
     </x:row>
     <x:row r="37" ht="33" customHeight="1">
       <x:c r="A37" s="5" t="str">
-        <x:v>smoke_link_window</x:v>
+        <x:v>power_rune_spawn_match_tolerance</x:v>
       </x:c>
       <x:c r="B37" s="5" t="str">
-        <x:v>120</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C37" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D37" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E37" s="5" t="str">
-        <x:v>开雾使用与modifier关联最大窗口</x:v>
+        <x:v>将结果事件反推到最近能量符刷新点的容差</x:v>
       </x:c>
       <x:c r="F37" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G37" s="5" t="str">
         <x:v>是</x:v>
@@ -2211,22 +2295,22 @@
     </x:row>
     <x:row r="38" ht="33" customHeight="1">
       <x:c r="A38" s="5" t="str">
-        <x:v>smoke_modifier_near_window</x:v>
+        <x:v>rune_bottle_pickup_suppression</x:v>
       </x:c>
       <x:c r="B38" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C38" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D38" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E38" s="5" t="str">
-        <x:v>无施法者关联时按同队modifier时间兜底</x:v>
+        <x:v>同英雄同神符罐装后拾取日志去重窗口</x:v>
       </x:c>
       <x:c r="F38" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G38" s="5" t="str">
         <x:v>是</x:v>
@@ -2235,22 +2319,22 @@
     </x:row>
     <x:row r="39" ht="33" customHeight="1">
       <x:c r="A39" s="5" t="str">
-        <x:v>smoke_fallback_near_radius</x:v>
+        <x:v>wisdom_rune_window</x:v>
       </x:c>
       <x:c r="B39" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C39" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D39" s="5" t="str">
-        <x:v>开雾</x:v>
+        <x:v>控符</x:v>
       </x:c>
       <x:c r="E39" s="5" t="str">
-        <x:v>无modifier时按使用者附近队友兜底</x:v>
+        <x:v>智慧符事件起点=t-10</x:v>
       </x:c>
       <x:c r="F39" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G39" s="5" t="str">
         <x:v>是</x:v>
@@ -2259,19 +2343,19 @@
     </x:row>
     <x:row r="40" ht="33" customHeight="1">
       <x:c r="A40" s="5" t="str">
-        <x:v>combat_damage_min_event</x:v>
+        <x:v>smoke_link_window</x:v>
       </x:c>
       <x:c r="B40" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C40" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D40" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E40" s="5" t="str">
-        <x:v>进入战斗检测的单条伤害最小值</x:v>
+        <x:v>开雾使用与modifier关联最大窗口</x:v>
       </x:c>
       <x:c r="F40" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2283,19 +2367,19 @@
     </x:row>
     <x:row r="41" ht="33" customHeight="1">
       <x:c r="A41" s="5" t="str">
-        <x:v>combat_seed_damage</x:v>
+        <x:v>smoke_modifier_near_window</x:v>
       </x:c>
       <x:c r="B41" s="5" t="str">
-        <x:v>550</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C41" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D41" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E41" s="5" t="str">
-        <x:v>初始空间簇成为战斗候选的伤害阈值，死亡可替代</x:v>
+        <x:v>无施法者关联时按同队modifier时间兜底</x:v>
       </x:c>
       <x:c r="F41" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2307,19 +2391,19 @@
     </x:row>
     <x:row r="42" ht="33" customHeight="1">
       <x:c r="A42" s="5" t="str">
-        <x:v>combat_refined_damage</x:v>
+        <x:v>smoke_fallback_near_radius</x:v>
       </x:c>
       <x:c r="B42" s="5" t="str">
-        <x:v>900</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C42" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D42" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>开雾</x:v>
       </x:c>
       <x:c r="E42" s="5" t="str">
-        <x:v>细化后无死亡战斗的最低总伤害</x:v>
+        <x:v>无modifier时按使用者附近队友兜底</x:v>
       </x:c>
       <x:c r="F42" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2331,22 +2415,22 @@
     </x:row>
     <x:row r="43" ht="33" customHeight="1">
       <x:c r="A43" s="5" t="str">
-        <x:v>combat_bucket</x:v>
+        <x:v>combat_damage_min_event_pre10</x:v>
       </x:c>
       <x:c r="B43" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C43" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D43" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E43" s="5" t="str">
-        <x:v>战斗检测分桶</x:v>
+        <x:v>0&lt;=time&lt;600 时进入战斗检测的单条伤害最小值</x:v>
       </x:c>
       <x:c r="F43" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G43" s="5" t="str">
         <x:v>是</x:v>
@@ -2355,19 +2439,19 @@
     </x:row>
     <x:row r="44" ht="33" customHeight="1">
       <x:c r="A44" s="5" t="str">
-        <x:v>combat_cluster_distance_raw</x:v>
+        <x:v>combat_damage_min_event_post10</x:v>
       </x:c>
       <x:c r="B44" s="5" t="str">
-        <x:v>38</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C44" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D44" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E44" s="5" t="str">
-        <x:v>同10秒桶内空间聚类距离</x:v>
+        <x:v>time&gt;=600 时进入战斗检测的单条伤害最小值；10分钟后计算方式不变</x:v>
       </x:c>
       <x:c r="F44" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2379,19 +2463,19 @@
     </x:row>
     <x:row r="45" ht="33" customHeight="1">
       <x:c r="A45" s="5" t="str">
-        <x:v>combat_cluster_merge_gap</x:v>
+        <x:v>combat_seed_damage</x:v>
       </x:c>
       <x:c r="B45" s="5" t="str">
-        <x:v>12</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="C45" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D45" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E45" s="5" t="str">
-        <x:v>相邻空间簇合并最大时间间隔</x:v>
+        <x:v>初始空间簇成为战斗候选的伤害阈值，死亡可替代</x:v>
       </x:c>
       <x:c r="F45" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2403,22 +2487,22 @@
     </x:row>
     <x:row r="46" ht="33" customHeight="1">
       <x:c r="A46" s="5" t="str">
-        <x:v>combat_cluster_merge_distance_game</x:v>
+        <x:v>combat_refined_damage</x:v>
       </x:c>
       <x:c r="B46" s="5" t="str">
-        <x:v>2200</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C46" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D46" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E46" s="5" t="str">
-        <x:v>相邻战斗信号合并最大中心距离；超过则拆成独立战斗</x:v>
+        <x:v>细化后无死亡战斗的最低总伤害</x:v>
       </x:c>
       <x:c r="F46" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G46" s="5" t="str">
         <x:v>是</x:v>
@@ -2427,10 +2511,10 @@
     </x:row>
     <x:row r="47" ht="33" customHeight="1">
       <x:c r="A47" s="5" t="str">
-        <x:v>combat_cluster_tail_seconds</x:v>
+        <x:v>combat_bucket</x:v>
       </x:c>
       <x:c r="B47" s="5" t="str">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C47" s="5" t="str">
         <x:v>秒</x:v>
@@ -2439,10 +2523,10 @@
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E47" s="5" t="str">
-        <x:v>尾部动态中心时间窗口；只取最近该秒数内的信号位置参与合并中心计算</x:v>
+        <x:v>战斗检测分桶</x:v>
       </x:c>
       <x:c r="F47" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G47" s="5" t="str">
         <x:v>是</x:v>
@@ -2451,22 +2535,22 @@
     </x:row>
     <x:row r="48" ht="33" customHeight="1">
       <x:c r="A48" s="5" t="str">
-        <x:v>combat_cluster_tail_signal_count</x:v>
+        <x:v>combat_cluster_distance_raw</x:v>
       </x:c>
       <x:c r="B48" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C48" s="5" t="str">
-        <x:v>条</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D48" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E48" s="5" t="str">
-        <x:v>尾部动态中心最多使用的最近有位置信号数</x:v>
+        <x:v>同10秒桶内空间聚类距离</x:v>
       </x:c>
       <x:c r="F48" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G48" s="5" t="str">
         <x:v>是</x:v>
@@ -2475,10 +2559,10 @@
     </x:row>
     <x:row r="49" ht="33" customHeight="1">
       <x:c r="A49" s="5" t="str">
-        <x:v>combat_refine_time_pad</x:v>
+        <x:v>combat_cluster_merge_gap_pre10</x:v>
       </x:c>
       <x:c r="B49" s="5" t="str">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C49" s="5" t="str">
         <x:v>秒</x:v>
@@ -2487,10 +2571,10 @@
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E49" s="5" t="str">
-        <x:v>细化收集伤害/控制/死亡的前后时间</x:v>
+        <x:v>0&lt;=time&lt;600 时相邻战斗信号合并最大时间间隔</x:v>
       </x:c>
       <x:c r="F49" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G49" s="5" t="str">
         <x:v>是</x:v>
@@ -2499,19 +2583,19 @@
     </x:row>
     <x:row r="50" ht="33" customHeight="1">
       <x:c r="A50" s="5" t="str">
-        <x:v>combat_refine_distance_raw</x:v>
+        <x:v>combat_cluster_merge_gap_post10</x:v>
       </x:c>
       <x:c r="B50" s="5" t="str">
-        <x:v>62</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C50" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D50" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E50" s="5" t="str">
-        <x:v>细化事件距离中心最大距离</x:v>
+        <x:v>time&gt;=600 时相邻战斗信号合并最大时间间隔；10分钟后计算方式不变</x:v>
       </x:c>
       <x:c r="F50" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2523,10 +2607,10 @@
     </x:row>
     <x:row r="51" ht="33" customHeight="1">
       <x:c r="A51" s="5" t="str">
-        <x:v>combat_participant_radius</x:v>
+        <x:v>combat_cluster_merge_distance_game</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
-        <x:v>1600</x:v>
+        <x:v>2200</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str">
         <x:v>码</x:v>
@@ -2535,10 +2619,10 @@
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E51" s="5" t="str">
-        <x:v>英雄参与战斗核心的默认最大距离</x:v>
+        <x:v>相邻战斗信号合并最大中心距离；超过则拆成独立战斗</x:v>
       </x:c>
       <x:c r="F51" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G51" s="5" t="str">
         <x:v>是</x:v>
@@ -2547,72 +2631,70 @@
     </x:row>
     <x:row r="52" ht="33" customHeight="1">
       <x:c r="A52" s="5" t="str">
-        <x:v>remote_contribution_distance</x:v>
+        <x:v>combat_cluster_tail_seconds_pre10</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>2000</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str">
-        <x:v>?</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D52" s="5" t="str">
-        <x:v>GANK/?????/??</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E52" s="5" t="str">
-        <x:v>????2000???????????/BUFF?????????????????????????????????</x:v>
+        <x:v>0&lt;=time&lt;600 时尾部动态中心时间窗口；只取最近该秒数内的信号位置参与合并中心计算</x:v>
       </x:c>
       <x:c r="F52" s="5" t="str">
-        <x:v>v1.10??</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G52" s="5" t="str">
-        <x:v>?</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H52" s="5" t="str"/>
     </x:row>
     <x:row r="53" ht="33" customHeight="1">
       <x:c r="A53" s="5" t="str">
-        <x:v>combat_midlane_exclusion_distance</x:v>
+        <x:v>combat_cluster_tail_seconds_post10</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D53" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E53" s="5" t="str">
-        <x:v>边路冲突中心时，中路线英雄超过该距离且未命中核心目标则排除</x:v>
+        <x:v>time&gt;=600 时尾部动态中心时间窗口；10分钟后计算方式不变</x:v>
       </x:c>
       <x:c r="F53" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G53" s="5" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="H53" s="5" t="str">
-        <x:v>本质是远端未交互排除，不限中路或10分钟前</x:v>
-      </x:c>
+      <x:c r="H53" s="5" t="str"/>
     </x:row>
     <x:row r="54" ht="33" customHeight="1">
       <x:c r="A54" s="5" t="str">
-        <x:v>combat_nearby_teammate_radius</x:v>
+        <x:v>combat_cluster_tail_signal_count</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>条</x:v>
       </x:c>
       <x:c r="D54" s="5" t="str">
         <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E54" s="5" t="str">
-        <x:v>细化阶段把近处同队英雄补入参战者</x:v>
+        <x:v>尾部动态中心最多使用的最近有位置信号数</x:v>
       </x:c>
       <x:c r="F54" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G54" s="5" t="str">
         <x:v>是</x:v>
@@ -2621,22 +2703,22 @@
     </x:row>
     <x:row r="55" ht="33" customHeight="1">
       <x:c r="A55" s="5" t="str">
-        <x:v>teamfight_min_side_count</x:v>
+        <x:v>skirmish_pre10_single_hero_damage_threshold</x:v>
       </x:c>
       <x:c r="B55" s="5" t="str">
-        <x:v>4</x:v>
+        <x:v>400</x:v>
       </x:c>
       <x:c r="C55" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D55" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E55" s="5" t="str">
-        <x:v>双方总参与各至少4人</x:v>
+        <x:v>0&lt;=time&lt;600 小规模冲突保留条件：任一英雄承伤必须 &gt;400；也可由总伤害&gt;900替代</x:v>
       </x:c>
       <x:c r="F55" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G55" s="5" t="str">
         <x:v>是</x:v>
@@ -2645,22 +2727,22 @@
     </x:row>
     <x:row r="56" ht="33" customHeight="1">
       <x:c r="A56" s="5" t="str">
-        <x:v>teamfight_min_direct_count</x:v>
+        <x:v>skirmish_pre10_total_damage_threshold</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D56" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E56" s="5" t="str">
-        <x:v>双方直接参与各至少3人</x:v>
+        <x:v>0&lt;=time&lt;600 小规模冲突保留条件：总伤害必须 &gt;900；也可由单英雄承伤&gt;400替代</x:v>
       </x:c>
       <x:c r="F56" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G56" s="5" t="str">
         <x:v>是</x:v>
@@ -2669,22 +2751,22 @@
     </x:row>
     <x:row r="57" ht="33" customHeight="1">
       <x:c r="A57" s="5" t="str">
-        <x:v>teamfight_damage_threshold</x:v>
+        <x:v>skirmish_pre10_short_duration_seconds</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>2500</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D57" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E57" s="5" t="str">
-        <x:v>达团战规模时的伤害阈值</x:v>
+        <x:v>0&lt;=time&lt;600 且 duration&lt;=12秒时使用整段伤害保留条件</x:v>
       </x:c>
       <x:c r="F57" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G57" s="5" t="str">
         <x:v>是</x:v>
@@ -2693,22 +2775,22 @@
     </x:row>
     <x:row r="58" ht="33" customHeight="1">
       <x:c r="A58" s="5" t="str">
-        <x:v>teamfight_death_threshold</x:v>
+        <x:v>skirmish_pre10_burst_window_seconds</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str">
-        <x:v>死亡</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D58" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E58" s="5" t="str">
-        <x:v>达团战规模时死亡数阈值</x:v>
+        <x:v>0&lt;=time&lt;600 且 duration&gt;12秒时使用滑动爆发窗口</x:v>
       </x:c>
       <x:c r="F58" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G58" s="5" t="str">
         <x:v>是</x:v>
@@ -2717,22 +2799,22 @@
     </x:row>
     <x:row r="59" ht="33" customHeight="1">
       <x:c r="A59" s="5" t="str">
-        <x:v>teamfight_duration_threshold</x:v>
+        <x:v>skirmish_pre10_burst_total_damage_threshold</x:v>
       </x:c>
       <x:c r="B59" s="5" t="str">
-        <x:v>15</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="C59" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D59" s="5" t="str">
-        <x:v>团战</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E59" s="5" t="str">
-        <x:v>达团战规模时持续时长阈值</x:v>
+        <x:v>长事件滑动8秒窗口内总伤害 &gt;=700 才保留；也可由单英雄承伤&gt;=360或死亡替代</x:v>
       </x:c>
       <x:c r="F59" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G59" s="5" t="str">
         <x:v>是</x:v>
@@ -2741,19 +2823,19 @@
     </x:row>
     <x:row r="60" ht="33" customHeight="1">
       <x:c r="A60" s="5" t="str">
-        <x:v>gank_open_window</x:v>
+        <x:v>skirmish_pre10_burst_single_hero_damage_threshold</x:v>
       </x:c>
       <x:c r="B60" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C60" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D60" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E60" s="5" t="str">
-        <x:v>同一目标在短窗口内被同一方至少2名不同英雄命中，才进入GANK候选</x:v>
+        <x:v>长事件滑动8秒窗口内任一英雄承伤 &gt;=360 才保留；也可由总伤害&gt;=700或死亡替代</x:v>
       </x:c>
       <x:c r="F60" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -2765,22 +2847,22 @@
     </x:row>
     <x:row r="61" ht="33" customHeight="1">
       <x:c r="A61" s="5" t="str">
-        <x:v>gank_position_sample_window</x:v>
+        <x:v>combat_refine_time_pad</x:v>
       </x:c>
       <x:c r="B61" s="5" t="str">
-        <x:v>±1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C61" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D61" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E61" s="5" t="str">
-        <x:v>读取发起时刻t0前后1秒的英雄位置；同一英雄取距离t0最近的位置</x:v>
+        <x:v>细化收集伤害/控制/死亡的前后时间</x:v>
       </x:c>
       <x:c r="F61" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G61" s="5" t="str">
         <x:v>是</x:v>
@@ -2789,22 +2871,22 @@
     </x:row>
     <x:row r="62" ht="33" customHeight="1">
       <x:c r="A62" s="5" t="str">
-        <x:v>gank_position_radius</x:v>
+        <x:v>combat_refine_distance_raw</x:v>
       </x:c>
       <x:c r="B62" s="5" t="str">
-        <x:v>1600</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C62" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D62" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E62" s="5" t="str">
-        <x:v>以被抓目标位置为中心统计发起阶段附近英雄</x:v>
+        <x:v>细化事件距离中心最大距离</x:v>
       </x:c>
       <x:c r="F62" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G62" s="5" t="str">
         <x:v>是</x:v>
@@ -2813,22 +2895,22 @@
     </x:row>
     <x:row r="63" ht="33" customHeight="1">
       <x:c r="A63" s="5" t="str">
-        <x:v>gank_min_attacker_nearby_heroes</x:v>
+        <x:v>combat_participant_radius</x:v>
       </x:c>
       <x:c r="B63" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>1600</x:v>
       </x:c>
       <x:c r="C63" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D63" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E63" s="5" t="str">
-        <x:v>发起时刻战场半径内GANK方至少2名英雄，且至少2名英雄直接命中同一目标</x:v>
+        <x:v>英雄参与战斗核心的默认最大距离</x:v>
       </x:c>
       <x:c r="F63" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G63" s="5" t="str">
         <x:v>是</x:v>
@@ -2837,67 +2919,69 @@
     </x:row>
     <x:row r="64" ht="33" customHeight="1">
       <x:c r="A64" s="5" t="str">
-        <x:v>gank_max_victim_nearby_heroes</x:v>
+        <x:v>remote_contribution_distance</x:v>
       </x:c>
       <x:c r="B64" s="5" t="str">
-        <x:v>1</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="C64" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>?</x:v>
       </x:c>
       <x:c r="D64" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>GANK/?????/??</x:v>
       </x:c>
       <x:c r="E64" s="5" t="str">
-        <x:v>发起时刻战场半径内被抓方只有被抓目标1名英雄；后续TP/走入只影响结果，不取消GANK</x:v>
+        <x:v>????2000???????????/BUFF?????????????????????????????????</x:v>
       </x:c>
       <x:c r="F64" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.10??</x:v>
       </x:c>
       <x:c r="G64" s="5" t="str">
-        <x:v>是</x:v>
+        <x:v>?</x:v>
       </x:c>
       <x:c r="H64" s="5" t="str"/>
     </x:row>
     <x:row r="65" ht="33" customHeight="1">
       <x:c r="A65" s="5" t="str">
-        <x:v>gank_victim_damage_min</x:v>
+        <x:v>combat_midlane_exclusion_distance</x:v>
       </x:c>
       <x:c r="B65" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C65" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D65" s="5" t="str">
-        <x:v>GANK</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E65" s="5" t="str">
-        <x:v>N抓1成立后，被抓目标承受非远程主战斗伤害达到该阈值才保留；死亡可替代</x:v>
+        <x:v>边路冲突中心时，中路线英雄超过该距离且未命中核心目标则排除</x:v>
       </x:c>
       <x:c r="F65" s="5" t="str">
-        <x:v>v1.10草案</x:v>
+        <x:v>v1.5</x:v>
       </x:c>
       <x:c r="G65" s="5" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="H65" s="5" t="str"/>
+      <x:c r="H65" s="5" t="str">
+        <x:v>本质是远端未交互排除，不限中路或10分钟前</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="33" customHeight="1">
       <x:c r="A66" s="5" t="str">
-        <x:v>skirmish_max_total_heroes</x:v>
+        <x:v>combat_nearby_teammate_radius</x:v>
       </x:c>
       <x:c r="B66" s="5" t="str">
-        <x:v>7</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C66" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D66" s="5" t="str">
-        <x:v>小规模冲突</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E66" s="5" t="str">
-        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
+        <x:v>细化阶段把近处同队英雄补入参战者</x:v>
       </x:c>
       <x:c r="F66" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2909,19 +2993,19 @@
     </x:row>
     <x:row r="67" ht="33" customHeight="1">
       <x:c r="A67" s="5" t="str">
-        <x:v>fight_dedup_gap_initial</x:v>
+        <x:v>teamfight_min_side_count</x:v>
       </x:c>
       <x:c r="B67" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C67" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D67" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E67" s="5" t="str">
-        <x:v>初始fight record近邻合并时间</x:v>
+        <x:v>双方总参与各至少4人</x:v>
       </x:c>
       <x:c r="F67" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2933,19 +3017,19 @@
     </x:row>
     <x:row r="68" ht="33" customHeight="1">
       <x:c r="A68" s="5" t="str">
-        <x:v>fight_dedup_distance_raw</x:v>
+        <x:v>teamfight_min_direct_count</x:v>
       </x:c>
       <x:c r="B68" s="5" t="str">
-        <x:v>58</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C68" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D68" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E68" s="5" t="str">
-        <x:v>初始fight record近邻合并距离</x:v>
+        <x:v>双方直接参与各至少3人</x:v>
       </x:c>
       <x:c r="F68" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2957,19 +3041,19 @@
     </x:row>
     <x:row r="69" ht="33" customHeight="1">
       <x:c r="A69" s="5" t="str">
-        <x:v>fight_overlap_shared_heroes</x:v>
+        <x:v>teamfight_damage_threshold</x:v>
       </x:c>
       <x:c r="B69" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>2500</x:v>
       </x:c>
       <x:c r="C69" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D69" s="5" t="str">
-        <x:v>小规模冲突/团战</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E69" s="5" t="str">
-        <x:v>重叠fight record合并的共享英雄数</x:v>
+        <x:v>达团战规模时的伤害阈值</x:v>
       </x:c>
       <x:c r="F69" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -2981,22 +3065,22 @@
     </x:row>
     <x:row r="70" ht="33" customHeight="1">
       <x:c r="A70" s="5" t="str">
-        <x:v>pickoff_enemy_damage_ratio</x:v>
+        <x:v>teamfight_death_threshold</x:v>
       </x:c>
       <x:c r="B70" s="5" t="str">
-        <x:v>0.80</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C70" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>死亡</x:v>
       </x:c>
       <x:c r="D70" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E70" s="5" t="str">
-        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
+        <x:v>达团战规模时死亡数阈值</x:v>
       </x:c>
       <x:c r="F70" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G70" s="5" t="str">
         <x:v>是</x:v>
@@ -3005,22 +3089,22 @@
     </x:row>
     <x:row r="71" ht="33" customHeight="1">
       <x:c r="A71" s="5" t="str">
-        <x:v>pickoff_ally_near_limit</x:v>
+        <x:v>teamfight_duration_threshold</x:v>
       </x:c>
       <x:c r="B71" s="5" t="str">
-        <x:v>1</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C71" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D71" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>团战</x:v>
       </x:c>
       <x:c r="E71" s="5" t="str">
-        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
+        <x:v>达团战规模时持续时长阈值</x:v>
       </x:c>
       <x:c r="F71" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G71" s="5" t="str">
         <x:v>是</x:v>
@@ -3029,22 +3113,22 @@
     </x:row>
     <x:row r="72" ht="33" customHeight="1">
       <x:c r="A72" s="5" t="str">
-        <x:v>escape_pickoff_window</x:v>
+        <x:v>gank_open_window</x:v>
       </x:c>
       <x:c r="B72" s="5" t="str">
-        <x:v>18</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C72" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D72" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E72" s="5" t="str">
-        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
+        <x:v>同一目标在短窗口内被同一方至少2名不同英雄命中，才进入GANK候选</x:v>
       </x:c>
       <x:c r="F72" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G72" s="5" t="str">
         <x:v>是</x:v>
@@ -3053,22 +3137,22 @@
     </x:row>
     <x:row r="73" ht="33" customHeight="1">
       <x:c r="A73" s="5" t="str">
-        <x:v>escape_pickoff_damage_min</x:v>
+        <x:v>gank_position_sample_window</x:v>
       </x:c>
       <x:c r="B73" s="5" t="str">
-        <x:v>180</x:v>
+        <x:v>±1</x:v>
       </x:c>
       <x:c r="C73" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D73" s="5" t="str">
-        <x:v>历史抓人候选</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E73" s="5" t="str">
-        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
+        <x:v>读取发起时刻t0前后1秒的英雄位置；同一英雄取距离t0最近的位置</x:v>
       </x:c>
       <x:c r="F73" s="5" t="str">
-        <x:v>v1.6</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G73" s="5" t="str">
         <x:v>是</x:v>
@@ -3077,22 +3161,22 @@
     </x:row>
     <x:row r="74" ht="33" customHeight="1">
       <x:c r="A74" s="5" t="str">
-        <x:v>roshan_context_radius</x:v>
+        <x:v>gank_position_radius</x:v>
       </x:c>
       <x:c r="B74" s="5" t="str">
-        <x:v>2000</x:v>
+        <x:v>1600</x:v>
       </x:c>
       <x:c r="C74" s="5" t="str">
         <x:v>码</x:v>
       </x:c>
       <x:c r="D74" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E74" s="5" t="str">
-        <x:v>肉山团上下文范围</x:v>
+        <x:v>以被抓目标位置为中心统计发起阶段附近英雄</x:v>
       </x:c>
       <x:c r="F74" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G74" s="5" t="str">
         <x:v>是</x:v>
@@ -3101,19 +3185,19 @@
     </x:row>
     <x:row r="75" ht="33" customHeight="1">
       <x:c r="A75" s="5" t="str">
-        <x:v>roshan_upper_pit_server</x:v>
+        <x:v>gank_min_attacker_nearby_heroes</x:v>
       </x:c>
       <x:c r="B75" s="5" t="str">
-        <x:v>(-3084,2296)</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C75" s="5" t="str">
-        <x:v>server坐标</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D75" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E75" s="5" t="str">
-        <x:v>肉山上路坑中心点；换算raw约(102.6,148.3)</x:v>
+        <x:v>发起时刻战场半径内GANK方至少2名英雄，且至少2名英雄直接命中同一目标</x:v>
       </x:c>
       <x:c r="F75" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -3125,19 +3209,19 @@
     </x:row>
     <x:row r="76" ht="33" customHeight="1">
       <x:c r="A76" s="5" t="str">
-        <x:v>roshan_lower_pit_server</x:v>
+        <x:v>gank_max_victim_nearby_heroes</x:v>
       </x:c>
       <x:c r="B76" s="5" t="str">
-        <x:v>(2842,-2743)</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C76" s="5" t="str">
-        <x:v>server坐标</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D76" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E76" s="5" t="str">
-        <x:v>肉山下路坑中心点；换算raw约(152.1,105.9)</x:v>
+        <x:v>发起时刻战场半径内被抓方只有被抓目标1名英雄；后续TP/走入只影响结果，不取消GANK</x:v>
       </x:c>
       <x:c r="F76" s="5" t="str">
         <x:v>v1.10草案</x:v>
@@ -3149,22 +3233,22 @@
     </x:row>
     <x:row r="77" ht="33" customHeight="1">
       <x:c r="A77" s="5" t="str">
-        <x:v>roshan_context_min_time</x:v>
+        <x:v>gank_victim_damage_min</x:v>
       </x:c>
       <x:c r="B77" s="5" t="str">
         <x:v>600</x:v>
       </x:c>
       <x:c r="C77" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D77" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>GANK</x:v>
       </x:c>
       <x:c r="E77" s="5" t="str">
-        <x:v>10分钟后靠近肉山坑可触发肉山上下文</x:v>
+        <x:v>N抓1成立后，被抓目标承受非远程主战斗伤害达到该阈值才保留；死亡可替代</x:v>
       </x:c>
       <x:c r="F77" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G77" s="5" t="str">
         <x:v>是</x:v>
@@ -3173,19 +3257,19 @@
     </x:row>
     <x:row r="78" ht="33" customHeight="1">
       <x:c r="A78" s="5" t="str">
-        <x:v>roshan_damage_context_pad</x:v>
+        <x:v>skirmish_max_total_heroes</x:v>
       </x:c>
       <x:c r="B78" s="5" t="str">
-        <x:v>30</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C78" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D78" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突</x:v>
       </x:c>
       <x:c r="E78" s="5" t="str">
-        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
+        <x:v>双方至少2v2且总人数不超过7时归为小规模冲突</x:v>
       </x:c>
       <x:c r="F78" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3197,19 +3281,19 @@
     </x:row>
     <x:row r="79" ht="33" customHeight="1">
       <x:c r="A79" s="5" t="str">
-        <x:v>roshan_kill_context_before</x:v>
+        <x:v>fight_dedup_gap_initial</x:v>
       </x:c>
       <x:c r="B79" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C79" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D79" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E79" s="5" t="str">
-        <x:v>肉山击杀与战斗关联前置时间</x:v>
+        <x:v>初始fight record近邻合并时间</x:v>
       </x:c>
       <x:c r="F79" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3221,19 +3305,19 @@
     </x:row>
     <x:row r="80" ht="33" customHeight="1">
       <x:c r="A80" s="5" t="str">
-        <x:v>roshan_kill_context_after</x:v>
+        <x:v>fight_dedup_distance_raw</x:v>
       </x:c>
       <x:c r="B80" s="5" t="str">
-        <x:v>75</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C80" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D80" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E80" s="5" t="str">
-        <x:v>肉山击杀与战斗关联后置时间</x:v>
+        <x:v>初始fight record近邻合并距离</x:v>
       </x:c>
       <x:c r="F80" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3245,19 +3329,19 @@
     </x:row>
     <x:row r="81" ht="33" customHeight="1">
       <x:c r="A81" s="5" t="str">
-        <x:v>roshan_respawn_suppression</x:v>
+        <x:v>fight_overlap_shared_heroes</x:v>
       </x:c>
       <x:c r="B81" s="5" t="str">
-        <x:v>480</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C81" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D81" s="5" t="str">
-        <x:v>肉山团</x:v>
+        <x:v>小规模冲突/团战</x:v>
       </x:c>
       <x:c r="E81" s="5" t="str">
-        <x:v>肉山死亡后该时间内不视为存活</x:v>
+        <x:v>重叠fight record合并的共享英雄数</x:v>
       </x:c>
       <x:c r="F81" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3269,22 +3353,22 @@
     </x:row>
     <x:row r="82" ht="33" customHeight="1">
       <x:c r="A82" s="5" t="str">
-        <x:v>roshan_attempt_group_gap</x:v>
+        <x:v>pickoff_enemy_damage_ratio</x:v>
       </x:c>
       <x:c r="B82" s="5" t="str">
-        <x:v>45</x:v>
+        <x:v>0.80</x:v>
       </x:c>
       <x:c r="C82" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>比例</x:v>
       </x:c>
       <x:c r="D82" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E82" s="5" t="str">
-        <x:v>Roshan伤害组分组间隔</x:v>
+        <x:v>旧单点击杀候选生成条件；最终不输出抓人标签</x:v>
       </x:c>
       <x:c r="F82" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G82" s="5" t="str">
         <x:v>是</x:v>
@@ -3293,22 +3377,22 @@
     </x:row>
     <x:row r="83" ht="33" customHeight="1">
       <x:c r="A83" s="5" t="str">
-        <x:v>roshan_attempt_damage_min</x:v>
+        <x:v>pickoff_ally_near_limit</x:v>
       </x:c>
       <x:c r="B83" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C83" s="5" t="str">
-        <x:v>伤害</x:v>
+        <x:v>人</x:v>
       </x:c>
       <x:c r="D83" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E83" s="5" t="str">
-        <x:v>未击杀Roshan尝试最低伤害</x:v>
+        <x:v>旧单点击杀候选受害方附近队友上限</x:v>
       </x:c>
       <x:c r="F83" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G83" s="5" t="str">
         <x:v>是</x:v>
@@ -3317,22 +3401,22 @@
     </x:row>
     <x:row r="84" ht="33" customHeight="1">
       <x:c r="A84" s="5" t="str">
-        <x:v>roshan_attempt_kill_grace</x:v>
+        <x:v>escape_pickoff_window</x:v>
       </x:c>
       <x:c r="B84" s="5" t="str">
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C84" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D84" s="5" t="str">
-        <x:v>肉山尝试</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E84" s="5" t="str">
-        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
+        <x:v>BKB/TP逃脱前受伤/受控窗口；最终需重映射或合并</x:v>
       </x:c>
       <x:c r="F84" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G84" s="5" t="str">
         <x:v>是</x:v>
@@ -3341,22 +3425,22 @@
     </x:row>
     <x:row r="85" ht="33" customHeight="1">
       <x:c r="A85" s="5" t="str">
-        <x:v>roshan_drop_merge_window</x:v>
+        <x:v>escape_pickoff_damage_min</x:v>
       </x:c>
       <x:c r="B85" s="5" t="str">
-        <x:v>20</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C85" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D85" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>历史抓人候选</x:v>
       </x:c>
       <x:c r="E85" s="5" t="str">
-        <x:v>肉山击杀后掉落合并窗口</x:v>
+        <x:v>无控制时逃脱候选最低敌方伤害</x:v>
       </x:c>
       <x:c r="F85" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.6</x:v>
       </x:c>
       <x:c r="G85" s="5" t="str">
         <x:v>是</x:v>
@@ -3365,22 +3449,22 @@
     </x:row>
     <x:row r="86" ht="33" customHeight="1">
       <x:c r="A86" s="5" t="str">
-        <x:v>roshan_owner_drop_fallback</x:v>
+        <x:v>roshan_context_radius</x:v>
       </x:c>
       <x:c r="B86" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>2000</x:v>
       </x:c>
       <x:c r="C86" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D86" s="5" t="str">
-        <x:v>肉山击杀</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E86" s="5" t="str">
-        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
+        <x:v>肉山团上下文范围</x:v>
       </x:c>
       <x:c r="F86" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G86" s="5" t="str">
         <x:v>是</x:v>
@@ -3389,22 +3473,22 @@
     </x:row>
     <x:row r="87" ht="33" customHeight="1">
       <x:c r="A87" s="5" t="str">
-        <x:v>tormentor_alive_start</x:v>
+        <x:v>roshan_upper_pit_server</x:v>
       </x:c>
       <x:c r="B87" s="5" t="str">
-        <x:v>1200</x:v>
+        <x:v>(-2924.964844,1522.657715)</x:v>
       </x:c>
       <x:c r="C87" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>server坐标</x:v>
       </x:c>
       <x:c r="D87" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E87" s="5" t="str">
-        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
+        <x:v>肉山上路坑中心点；换算raw约(104.0,141.7)</x:v>
       </x:c>
       <x:c r="F87" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G87" s="5" t="str">
         <x:v>是</x:v>
@@ -3413,22 +3497,22 @@
     </x:row>
     <x:row r="88" ht="33" customHeight="1">
       <x:c r="A88" s="5" t="str">
-        <x:v>tormentor_respawn_suppression</x:v>
+        <x:v>roshan_lower_pit_server</x:v>
       </x:c>
       <x:c r="B88" s="5" t="str">
-        <x:v>600</x:v>
+        <x:v>(2867.646973,-3401.379395)</x:v>
       </x:c>
       <x:c r="C88" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>server坐标</x:v>
       </x:c>
       <x:c r="D88" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E88" s="5" t="str">
-        <x:v>魔晶死亡后该时间内不视为存活</x:v>
+        <x:v>肉山下路坑中心点；换算raw约(152.3,100.5)</x:v>
       </x:c>
       <x:c r="F88" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.10草案</x:v>
       </x:c>
       <x:c r="G88" s="5" t="str">
         <x:v>是</x:v>
@@ -3437,22 +3521,22 @@
     </x:row>
     <x:row r="89" ht="33" customHeight="1">
       <x:c r="A89" s="5" t="str">
-        <x:v>tormentor_near_radius</x:v>
+        <x:v>roshan_context_min_time</x:v>
       </x:c>
       <x:c r="B89" s="5" t="str">
-        <x:v>1500</x:v>
+        <x:v>900</x:v>
       </x:c>
       <x:c r="C89" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D89" s="5" t="str">
-        <x:v>魔晶团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E89" s="5" t="str">
-        <x:v>独立魔晶击杀附近英雄判断</x:v>
+        <x:v>15分钟后靠近肉山坑才可触发肉山上下文；15分钟前不计算肉山团</x:v>
       </x:c>
       <x:c r="F89" s="5" t="str">
-        <x:v>v1.4</x:v>
+        <x:v>v1.11草案</x:v>
       </x:c>
       <x:c r="G89" s="5" t="str">
         <x:v>是</x:v>
@@ -3461,19 +3545,19 @@
     </x:row>
     <x:row r="90" ht="33" customHeight="1">
       <x:c r="A90" s="5" t="str">
-        <x:v>highground_raw_corner</x:v>
+        <x:v>roshan_damage_context_pad</x:v>
       </x:c>
       <x:c r="B90" s="5" t="str">
-        <x:v>95/158</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C90" s="5" t="str">
-        <x:v>raw坐标</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D90" s="5" t="str">
-        <x:v>高地团</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E90" s="5" t="str">
-        <x:v>高地团中心区域阈值</x:v>
+        <x:v>肉山伤害与战斗窗口前后关联时间</x:v>
       </x:c>
       <x:c r="F90" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3485,19 +3569,19 @@
     </x:row>
     <x:row r="91" ht="33" customHeight="1">
       <x:c r="A91" s="5" t="str">
-        <x:v>tower_context_radius</x:v>
+        <x:v>roshan_kill_context_before</x:v>
       </x:c>
       <x:c r="B91" s="5" t="str">
-        <x:v>1000</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C91" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D91" s="5" t="str">
-        <x:v>塔下</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E91" s="5" t="str">
-        <x:v>防御塔上下文范围</x:v>
+        <x:v>肉山击杀与战斗关联前置时间</x:v>
       </x:c>
       <x:c r="F91" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3509,19 +3593,19 @@
     </x:row>
     <x:row r="92" ht="33" customHeight="1">
       <x:c r="A92" s="5" t="str">
-        <x:v>tower_context_time_pad</x:v>
+        <x:v>roshan_kill_context_after</x:v>
       </x:c>
       <x:c r="B92" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C92" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D92" s="5" t="str">
-        <x:v>塔下</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E92" s="5" t="str">
-        <x:v>战斗窗口前后塔状态检测</x:v>
+        <x:v>肉山击杀与战斗关联后置时间</x:v>
       </x:c>
       <x:c r="F92" s="5" t="str">
         <x:v>v1.4</x:v>
@@ -3533,22 +3617,22 @@
     </x:row>
     <x:row r="93" ht="33" customHeight="1">
       <x:c r="A93" s="5" t="str">
-        <x:v>aegis_valid_duration</x:v>
+        <x:v>roshan_respawn_suppression</x:v>
       </x:c>
       <x:c r="B93" s="5" t="str">
-        <x:v>300</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="C93" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D93" s="5" t="str">
-        <x:v>带盾阵亡</x:v>
+        <x:v>肉山团</x:v>
       </x:c>
       <x:c r="E93" s="5" t="str">
-        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
+        <x:v>肉山死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F93" s="5" t="str">
-        <x:v>v1.5</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G93" s="5" t="str">
         <x:v>是</x:v>
@@ -3557,22 +3641,22 @@
     </x:row>
     <x:row r="94" ht="33" customHeight="1">
       <x:c r="A94" s="5" t="str">
-        <x:v>v1_7_subordinate_overlap_ratio</x:v>
+        <x:v>roshan_attempt_group_gap</x:v>
       </x:c>
       <x:c r="B94" s="5" t="str">
-        <x:v>0.60</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="C94" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D94" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E94" s="5" t="str">
-        <x:v>旧单点候选与父窗口重叠比例</x:v>
+        <x:v>Roshan伤害组分组间隔</x:v>
       </x:c>
       <x:c r="F94" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G94" s="5" t="str">
         <x:v>是</x:v>
@@ -3581,22 +3665,22 @@
     </x:row>
     <x:row r="95" ht="33" customHeight="1">
       <x:c r="A95" s="5" t="str">
-        <x:v>v1_7_parent_start_grace</x:v>
+        <x:v>roshan_attempt_damage_min</x:v>
       </x:c>
       <x:c r="B95" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C95" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>伤害</x:v>
       </x:c>
       <x:c r="D95" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E95" s="5" t="str">
-        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
+        <x:v>未击杀Roshan尝试最低伤害</x:v>
       </x:c>
       <x:c r="F95" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G95" s="5" t="str">
         <x:v>是</x:v>
@@ -3605,22 +3689,22 @@
     </x:row>
     <x:row r="96" ht="33" customHeight="1">
       <x:c r="A96" s="5" t="str">
-        <x:v>v1_7_parent_end_grace</x:v>
+        <x:v>roshan_attempt_kill_grace</x:v>
       </x:c>
       <x:c r="B96" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C96" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D96" s="5" t="str">
-        <x:v>小规模冲突/团战/特殊战斗</x:v>
+        <x:v>肉山尝试</x:v>
       </x:c>
       <x:c r="E96" s="5" t="str">
-        <x:v>父窗口允许比候选结束最多早5秒</x:v>
+        <x:v>伤害组结束后若8秒内击杀则不输出尝试</x:v>
       </x:c>
       <x:c r="F96" s="5" t="str">
-        <x:v>v1.7</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G96" s="5" t="str">
         <x:v>是</x:v>
@@ -3629,19 +3713,19 @@
     </x:row>
     <x:row r="97" ht="33" customHeight="1">
       <x:c r="A97" s="5" t="str">
-        <x:v>v1_8_duplicate_no_kill_gap</x:v>
+        <x:v>roshan_drop_merge_window</x:v>
       </x:c>
       <x:c r="B97" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C97" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D97" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E97" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
+        <x:v>肉山击杀后掉落合并窗口</x:v>
       </x:c>
       <x:c r="F97" s="5" t="str">
         <x:v>v1.8</x:v>
@@ -3653,19 +3737,19 @@
     </x:row>
     <x:row r="98" ht="33" customHeight="1">
       <x:c r="A98" s="5" t="str">
-        <x:v>v1_8_duplicate_distance</x:v>
+        <x:v>roshan_owner_drop_fallback</x:v>
       </x:c>
       <x:c r="B98" s="5" t="str">
-        <x:v>1800</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C98" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D98" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>肉山击杀</x:v>
       </x:c>
       <x:c r="E98" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
+        <x:v>缺少roshan_death时用掉落阵营兜底归属</x:v>
       </x:c>
       <x:c r="F98" s="5" t="str">
         <x:v>v1.8</x:v>
@@ -3677,22 +3761,22 @@
     </x:row>
     <x:row r="99" ht="33" customHeight="1">
       <x:c r="A99" s="5" t="str">
-        <x:v>v1_8_duplicate_jaccard</x:v>
+        <x:v>tormentor_alive_start</x:v>
       </x:c>
       <x:c r="B99" s="5" t="str">
-        <x:v>0.50</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="C99" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D99" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E99" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
+        <x:v>20分钟后魔晶/折磨者才可能存活</x:v>
       </x:c>
       <x:c r="F99" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G99" s="5" t="str">
         <x:v>是</x:v>
@@ -3701,22 +3785,22 @@
     </x:row>
     <x:row r="100" ht="33" customHeight="1">
       <x:c r="A100" s="5" t="str">
-        <x:v>v1_8_duplicate_shared_heroes</x:v>
+        <x:v>tormentor_respawn_suppression</x:v>
       </x:c>
       <x:c r="B100" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="C100" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D100" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E100" s="5" t="str">
-        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
+        <x:v>魔晶死亡后该时间内不视为存活</x:v>
       </x:c>
       <x:c r="F100" s="5" t="str">
-        <x:v>v1.8</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G100" s="5" t="str">
         <x:v>是</x:v>
@@ -3725,22 +3809,22 @@
     </x:row>
     <x:row r="101" ht="33" customHeight="1">
       <x:c r="A101" s="5" t="str">
-        <x:v>v1_9_kill_parent_gap</x:v>
+        <x:v>tormentor_near_radius</x:v>
       </x:c>
       <x:c r="B101" s="5" t="str">
-        <x:v>5</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="C101" s="5" t="str">
-        <x:v>秒</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D101" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>魔晶团</x:v>
       </x:c>
       <x:c r="E101" s="5" t="str">
-        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
+        <x:v>独立魔晶击杀附近英雄判断</x:v>
       </x:c>
       <x:c r="F101" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G101" s="5" t="str">
         <x:v>是</x:v>
@@ -3749,22 +3833,22 @@
     </x:row>
     <x:row r="102" ht="33" customHeight="1">
       <x:c r="A102" s="5" t="str">
-        <x:v>v1_9_kill_parent_distance</x:v>
+        <x:v>highground_raw_corner</x:v>
       </x:c>
       <x:c r="B102" s="5" t="str">
-        <x:v>2500</x:v>
+        <x:v>95/158</x:v>
       </x:c>
       <x:c r="C102" s="5" t="str">
-        <x:v>码</x:v>
+        <x:v>raw坐标</x:v>
       </x:c>
       <x:c r="D102" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>高地团</x:v>
       </x:c>
       <x:c r="E102" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
+        <x:v>高地团中心区域阈值</x:v>
       </x:c>
       <x:c r="F102" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G102" s="5" t="str">
         <x:v>是</x:v>
@@ -3773,22 +3857,22 @@
     </x:row>
     <x:row r="103" ht="33" customHeight="1">
       <x:c r="A103" s="5" t="str">
-        <x:v>v1_9_kill_parent_jaccard</x:v>
+        <x:v>tower_context_radius</x:v>
       </x:c>
       <x:c r="B103" s="5" t="str">
-        <x:v>0.33</x:v>
+        <x:v>1000</x:v>
       </x:c>
       <x:c r="C103" s="5" t="str">
-        <x:v>比例</x:v>
+        <x:v>码</x:v>
       </x:c>
       <x:c r="D103" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>塔下</x:v>
       </x:c>
       <x:c r="E103" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
+        <x:v>防御塔上下文范围</x:v>
       </x:c>
       <x:c r="F103" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G103" s="5" t="str">
         <x:v>是</x:v>
@@ -3797,22 +3881,22 @@
     </x:row>
     <x:row r="104" ht="33" customHeight="1">
       <x:c r="A104" s="5" t="str">
-        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+        <x:v>tower_context_time_pad</x:v>
       </x:c>
       <x:c r="B104" s="5" t="str">
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C104" s="5" t="str">
-        <x:v>人</x:v>
+        <x:v>秒</x:v>
       </x:c>
       <x:c r="D104" s="5" t="str">
-        <x:v>战斗类标签</x:v>
+        <x:v>塔下</x:v>
       </x:c>
       <x:c r="E104" s="5" t="str">
-        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+        <x:v>战斗窗口前后塔状态检测</x:v>
       </x:c>
       <x:c r="F104" s="5" t="str">
-        <x:v>v1.9</x:v>
+        <x:v>v1.4</x:v>
       </x:c>
       <x:c r="G104" s="5" t="str">
         <x:v>是</x:v>
@@ -3821,27 +3905,315 @@
     </x:row>
     <x:row r="105" ht="33" customHeight="1">
       <x:c r="A105" s="5" t="str">
-        <x:v>adjacent_combat_qc_scan_window</x:v>
+        <x:v>aegis_valid_duration</x:v>
       </x:c>
       <x:c r="B105" s="5" t="str">
-        <x:v>10</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="C105" s="5" t="str">
         <x:v>秒</x:v>
       </x:c>
       <x:c r="D105" s="5" t="str">
+        <x:v>带盾阵亡</x:v>
+      </x:c>
+      <x:c r="E105" s="5" t="str">
+        <x:v>Aegis领取后可触发带盾阵亡的窗口</x:v>
+      </x:c>
+      <x:c r="F105" s="5" t="str">
+        <x:v>v1.5</x:v>
+      </x:c>
+      <x:c r="G105" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H105" s="5" t="str"/>
+    </x:row>
+    <x:row r="106" ht="33" customHeight="1">
+      <x:c r="A106" s="5" t="str">
+        <x:v>v1_7_subordinate_overlap_ratio</x:v>
+      </x:c>
+      <x:c r="B106" s="5" t="str">
+        <x:v>0.60</x:v>
+      </x:c>
+      <x:c r="C106" s="5" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="D106" s="5" t="str">
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
+      </x:c>
+      <x:c r="E106" s="5" t="str">
+        <x:v>旧单点候选与父窗口重叠比例</x:v>
+      </x:c>
+      <x:c r="F106" s="5" t="str">
+        <x:v>v1.7</x:v>
+      </x:c>
+      <x:c r="G106" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H106" s="5" t="str"/>
+    </x:row>
+    <x:row r="107" ht="33" customHeight="1">
+      <x:c r="A107" s="5" t="str">
+        <x:v>v1_7_parent_start_grace</x:v>
+      </x:c>
+      <x:c r="B107" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C107" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D107" s="5" t="str">
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
+      </x:c>
+      <x:c r="E107" s="5" t="str">
+        <x:v>父窗口允许比候选开始最多晚2秒</x:v>
+      </x:c>
+      <x:c r="F107" s="5" t="str">
+        <x:v>v1.7</x:v>
+      </x:c>
+      <x:c r="G107" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H107" s="5" t="str"/>
+    </x:row>
+    <x:row r="108" ht="33" customHeight="1">
+      <x:c r="A108" s="5" t="str">
+        <x:v>v1_7_parent_end_grace</x:v>
+      </x:c>
+      <x:c r="B108" s="5" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C108" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D108" s="5" t="str">
+        <x:v>小规模冲突/团战/特殊战斗</x:v>
+      </x:c>
+      <x:c r="E108" s="5" t="str">
+        <x:v>父窗口允许比候选结束最多早5秒</x:v>
+      </x:c>
+      <x:c r="F108" s="5" t="str">
+        <x:v>v1.7</x:v>
+      </x:c>
+      <x:c r="G108" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H108" s="5" t="str"/>
+    </x:row>
+    <x:row r="109" ht="33" customHeight="1">
+      <x:c r="A109" s="5" t="str">
+        <x:v>v1_8_duplicate_no_kill_gap</x:v>
+      </x:c>
+      <x:c r="B109" s="5" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C109" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D109" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E109" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选合并最大间隔</x:v>
+      </x:c>
+      <x:c r="F109" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G109" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H109" s="5" t="str"/>
+    </x:row>
+    <x:row r="110" ht="33" customHeight="1">
+      <x:c r="A110" s="5" t="str">
+        <x:v>v1_8_duplicate_distance</x:v>
+      </x:c>
+      <x:c r="B110" s="5" t="str">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="C110" s="5" t="str">
+        <x:v>码</x:v>
+      </x:c>
+      <x:c r="D110" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E110" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选中心最大距离</x:v>
+      </x:c>
+      <x:c r="F110" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G110" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H110" s="5" t="str"/>
+    </x:row>
+    <x:row r="111" ht="33" customHeight="1">
+      <x:c r="A111" s="5" t="str">
+        <x:v>v1_8_duplicate_jaccard</x:v>
+      </x:c>
+      <x:c r="B111" s="5" t="str">
+        <x:v>0.50</x:v>
+      </x:c>
+      <x:c r="C111" s="5" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="D111" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E111" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选英雄Jaccard阈值</x:v>
+      </x:c>
+      <x:c r="F111" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G111" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H111" s="5" t="str"/>
+    </x:row>
+    <x:row r="112" ht="33" customHeight="1">
+      <x:c r="A112" s="5" t="str">
+        <x:v>v1_8_duplicate_shared_heroes</x:v>
+      </x:c>
+      <x:c r="B112" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C112" s="5" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="D112" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E112" s="5" t="str">
+        <x:v>无独立击杀重复战斗候选共享英雄阈值</x:v>
+      </x:c>
+      <x:c r="F112" s="5" t="str">
+        <x:v>v1.8</x:v>
+      </x:c>
+      <x:c r="G112" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H112" s="5" t="str"/>
+    </x:row>
+    <x:row r="113" ht="33" customHeight="1">
+      <x:c r="A113" s="5" t="str">
+        <x:v>v1_9_kill_parent_gap</x:v>
+      </x:c>
+      <x:c r="B113" s="5" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C113" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D113" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E113" s="5" t="str">
+        <x:v>有击杀父事件吸收无独立击杀短窗口的最大相邻间隔</x:v>
+      </x:c>
+      <x:c r="F113" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G113" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H113" s="5" t="str"/>
+    </x:row>
+    <x:row r="114" ht="33" customHeight="1">
+      <x:c r="A114" s="5" t="str">
+        <x:v>v1_9_kill_parent_distance</x:v>
+      </x:c>
+      <x:c r="B114" s="5" t="str">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="C114" s="5" t="str">
+        <x:v>码</x:v>
+      </x:c>
+      <x:c r="D114" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E114" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的最大距离；未知位置允许通过</x:v>
+      </x:c>
+      <x:c r="F114" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G114" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H114" s="5" t="str"/>
+    </x:row>
+    <x:row r="115" ht="33" customHeight="1">
+      <x:c r="A115" s="5" t="str">
+        <x:v>v1_9_kill_parent_jaccard</x:v>
+      </x:c>
+      <x:c r="B115" s="5" t="str">
+        <x:v>0.33</x:v>
+      </x:c>
+      <x:c r="C115" s="5" t="str">
+        <x:v>比例</x:v>
+      </x:c>
+      <x:c r="D115" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E115" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的英雄Jaccard阈值</x:v>
+      </x:c>
+      <x:c r="F115" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G115" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H115" s="5" t="str"/>
+    </x:row>
+    <x:row r="116" ht="33" customHeight="1">
+      <x:c r="A116" s="5" t="str">
+        <x:v>v1_9_kill_parent_shared_heroes</x:v>
+      </x:c>
+      <x:c r="B116" s="5" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C116" s="5" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="D116" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="E116" s="5" t="str">
+        <x:v>有击杀父事件吸收短窗口的共享英雄阈值</x:v>
+      </x:c>
+      <x:c r="F116" s="5" t="str">
+        <x:v>v1.9</x:v>
+      </x:c>
+      <x:c r="G116" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H116" s="5" t="str"/>
+    </x:row>
+    <x:row r="117" ht="33" customHeight="1">
+      <x:c r="A117" s="5" t="str">
+        <x:v>adjacent_combat_qc_scan_window</x:v>
+      </x:c>
+      <x:c r="B117" s="5" t="str">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C117" s="5" t="str">
+        <x:v>秒</x:v>
+      </x:c>
+      <x:c r="D117" s="5" t="str">
         <x:v>质量控制</x:v>
       </x:c>
-      <x:c r="E105" s="5" t="str">
+      <x:c r="E117" s="5" t="str">
         <x:v>生成后复查相邻战斗事件的建议扫描窗口</x:v>
       </x:c>
-      <x:c r="F105" s="5" t="str">
+      <x:c r="F117" s="5" t="str">
         <x:v>v1.9</x:v>
       </x:c>
-      <x:c r="G105" s="5" t="str">
-        <x:v>是</x:v>
-      </x:c>
-      <x:c r="H105" s="5" t="str"/>
+      <x:c r="G117" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="H117" s="5" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4562,6 +4934,58 @@
         <x:v>v1.9把原因写入规则，后续可继续收敛</x:v>
       </x:c>
       <x:c r="H17" s="5" t="str"/>
+    </x:row>
+    <x:row r="18" ht="49.5" customHeight="1">
+      <x:c r="A18" s="5" t="str">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>合并后重判主标签</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="str">
+        <x:v>合并后的fight_records</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="str">
+        <x:v>相邻合并、追击合并或续团合并后，用合并后的双方人数、直接参与人数、总伤害、死亡数和持续时间重新判定主战斗标签；满足团战条件则从小规模冲突升级为团战</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="str">
+        <x:v>更新后的战斗标签</x:v>
+      </x:c>
+      <x:c r="F18" s="5" t="str">
+        <x:v>第一段小规模冲突合并后达到团战规模但未升级</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="str">
+        <x:v>8842468101 21:36-22:14 应由小规模冲突升级为团战</x:v>
+      </x:c>
+      <x:c r="H18" s="5" t="str">
+        <x:v>v1.10草案</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="49.5" customHeight="1">
+      <x:c r="A19" s="5" t="str">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="str">
+        <x:v>远程交互不作为续团共享英雄</x:v>
+      </x:c>
+      <x:c r="C19" s="5" t="str">
+        <x:v>interaction_positions; player_intervals2</x:v>
+      </x:c>
+      <x:c r="D19" s="5" t="str">
+        <x:v>续团/追击合并取共享交互英雄时，若施加者与目标英雄本体距离&gt;2000码，则远程施加者不进入共享英雄集合；该交互只保留被命中目标作为现场交互英雄</x:v>
+      </x:c>
+      <x:c r="E19" s="5" t="str">
+        <x:v>更干净的续团合并结果</x:v>
+      </x:c>
+      <x:c r="F19" s="5" t="str">
+        <x:v>先知大招等全图远程伤害把两个空间独立战斗误合并</x:v>
+      </x:c>
+      <x:c r="G19" s="5" t="str">
+        <x:v>8842468101 25:28-25:46 拆为两条GANK</x:v>
+      </x:c>
+      <x:c r="H19" s="5" t="str">
+        <x:v>v1.10草案</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4963,6 +5387,60 @@
       </x:c>
       <x:c r="I14" s="5" t="str"/>
     </x:row>
+    <x:row r="15" ht="51" customHeight="1">
+      <x:c r="A15" s="5" t="str">
+        <x:v>M14</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="str">
+        <x:v>合并后重判主标签</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="str">
+        <x:v>战斗候选完成相邻合并、追击合并或续团合并后，重新按合并后的规模与强度调用主分类规则</x:v>
+      </x:c>
+      <x:c r="E15" s="5" t="str">
+        <x:v>小规模冲突可升级为团战，GANK追击可被父战斗吸收</x:v>
+      </x:c>
+      <x:c r="F15" s="5" t="str">
+        <x:v>修复合并后仍沿用第一段小规模冲突标签的问题</x:v>
+      </x:c>
+      <x:c r="G15" s="5" t="str">
+        <x:v>v1.10草案</x:v>
+      </x:c>
+      <x:c r="H15" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I15" s="5" t="str"/>
+    </x:row>
+    <x:row r="16" ht="51" customHeight="1">
+      <x:c r="A16" s="5" t="str">
+        <x:v>M15</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="str">
+        <x:v>远程共享英雄排除</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="str">
+        <x:v>战斗类标签</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="str">
+        <x:v>续团/追击合并时，距离&gt;2000码的远程施加者不作为共享交互英雄；全图/超远距离技能只作为远程贡献</x:v>
+      </x:c>
+      <x:c r="E16" s="5" t="str">
+        <x:v>避免跨区域战斗被远程技能粘连</x:v>
+      </x:c>
+      <x:c r="F16" s="5" t="str">
+        <x:v>修复先知大招把25:28潮汐战斗和25:33树精死亡合并的问题</x:v>
+      </x:c>
+      <x:c r="G16" s="5" t="str">
+        <x:v>v1.10草案</x:v>
+      </x:c>
+      <x:c r="H16" s="5" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="I16" s="5" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>